<commit_message>
Deploy Test Reports — 1200 Tests All PASSED 7e5425d7e5e25ebdcd95feff7c7d50818f326a8c
</commit_message>
<xml_diff>
--- a/reports/latest/Appium_Report.xlsx
+++ b/reports/latest/Appium_Report.xlsx
@@ -521,12 +521,12 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>224</v>
+        <v>1095</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-10T04:31:50.000Z</t>
+          <t>2026-07-10T04:47:24.000Z</t>
         </is>
       </c>
     </row>
@@ -550,12 +550,12 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>445</v>
+        <v>499</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-10T04:31:50.000Z</t>
+          <t>2026-07-10T04:47:25.000Z</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>890</v>
+        <v>725</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-10T04:31:51.000Z</t>
+          <t>2026-07-10T04:47:26.000Z</t>
         </is>
       </c>
     </row>
@@ -608,12 +608,12 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>712</v>
+        <v>773</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-10T04:31:52.000Z</t>
+          <t>2026-07-10T04:47:27.000Z</t>
         </is>
       </c>
     </row>
@@ -637,12 +637,12 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>594</v>
+        <v>615</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-10T04:31:53.000Z</t>
+          <t>2026-07-10T04:47:28.000Z</t>
         </is>
       </c>
     </row>
@@ -666,12 +666,12 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1198</v>
+        <v>1171</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-10T04:31:54.000Z</t>
+          <t>2026-07-10T04:47:28.000Z</t>
         </is>
       </c>
     </row>
@@ -695,12 +695,12 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1141</v>
+        <v>328</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-07-10T04:31:54.000Z</t>
+          <t>2026-07-10T04:47:29.000Z</t>
         </is>
       </c>
     </row>
@@ -724,12 +724,12 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>895</v>
+        <v>151</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-07-10T04:31:55.000Z</t>
+          <t>2026-07-10T04:47:30.000Z</t>
         </is>
       </c>
     </row>
@@ -753,12 +753,12 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>782</v>
+        <v>747</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-07-10T04:31:56.000Z</t>
+          <t>2026-07-10T04:47:31.000Z</t>
         </is>
       </c>
     </row>
@@ -782,12 +782,12 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>542</v>
+        <v>241</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-07-10T04:31:57.000Z</t>
+          <t>2026-07-10T04:47:32.000Z</t>
         </is>
       </c>
     </row>
@@ -811,12 +811,12 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1013</v>
+        <v>664</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-10T04:31:58.000Z</t>
+          <t>2026-07-10T04:47:32.000Z</t>
         </is>
       </c>
     </row>
@@ -840,12 +840,12 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>785</v>
+        <v>1029</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-07-10T04:31:58.000Z</t>
+          <t>2026-07-10T04:47:33.000Z</t>
         </is>
       </c>
     </row>
@@ -869,12 +869,12 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>110</v>
+        <v>705</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-10T04:31:59.000Z</t>
+          <t>2026-07-10T04:47:34.000Z</t>
         </is>
       </c>
     </row>
@@ -898,12 +898,12 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>308</v>
+        <v>411</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:00.000Z</t>
+          <t>2026-07-10T04:47:35.000Z</t>
         </is>
       </c>
     </row>
@@ -927,12 +927,12 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>269</v>
+        <v>682</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:01.000Z</t>
+          <t>2026-07-10T04:47:36.000Z</t>
         </is>
       </c>
     </row>
@@ -956,12 +956,12 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>890</v>
+        <v>776</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:02.000Z</t>
+          <t>2026-07-10T04:47:36.000Z</t>
         </is>
       </c>
     </row>
@@ -985,12 +985,12 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1155</v>
+        <v>1066</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:02.000Z</t>
+          <t>2026-07-10T04:47:37.000Z</t>
         </is>
       </c>
     </row>
@@ -1014,12 +1014,12 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>1133</v>
+        <v>931</v>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:03.000Z</t>
+          <t>2026-07-10T04:47:38.000Z</t>
         </is>
       </c>
     </row>
@@ -1043,12 +1043,12 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>728</v>
+        <v>330</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:04.000Z</t>
+          <t>2026-07-10T04:47:39.000Z</t>
         </is>
       </c>
     </row>
@@ -1072,12 +1072,12 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>568</v>
+        <v>367</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:05.000Z</t>
+          <t>2026-07-10T04:47:40.000Z</t>
         </is>
       </c>
     </row>
@@ -1101,12 +1101,12 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>639</v>
+        <v>555</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:06.000Z</t>
+          <t>2026-07-10T04:47:40.000Z</t>
         </is>
       </c>
     </row>
@@ -1130,12 +1130,12 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>554</v>
+        <v>397</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:06.000Z</t>
+          <t>2026-07-10T04:47:41.000Z</t>
         </is>
       </c>
     </row>
@@ -1159,12 +1159,12 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>168</v>
+        <v>1096</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:07.000Z</t>
+          <t>2026-07-10T04:47:42.000Z</t>
         </is>
       </c>
     </row>
@@ -1188,12 +1188,12 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>968</v>
+        <v>945</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:08.000Z</t>
+          <t>2026-07-10T04:47:43.000Z</t>
         </is>
       </c>
     </row>
@@ -1217,12 +1217,12 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>467</v>
+        <v>1070</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:09.000Z</t>
+          <t>2026-07-10T04:47:44.000Z</t>
         </is>
       </c>
     </row>
@@ -1246,12 +1246,12 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>807</v>
+        <v>340</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:10.000Z</t>
+          <t>2026-07-10T04:47:44.000Z</t>
         </is>
       </c>
     </row>
@@ -1275,12 +1275,12 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>697</v>
+        <v>193</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:10.000Z</t>
+          <t>2026-07-10T04:47:45.000Z</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>104</v>
+        <v>1056</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:11.000Z</t>
+          <t>2026-07-10T04:47:46.000Z</t>
         </is>
       </c>
     </row>
@@ -1333,12 +1333,12 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>906</v>
+        <v>1103</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:12.000Z</t>
+          <t>2026-07-10T04:47:47.000Z</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>1134</v>
+        <v>711</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:13.000Z</t>
+          <t>2026-07-10T04:47:48.000Z</t>
         </is>
       </c>
     </row>
@@ -1391,12 +1391,12 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>949</v>
+        <v>125</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:14.000Z</t>
+          <t>2026-07-10T04:47:48.000Z</t>
         </is>
       </c>
     </row>
@@ -1420,12 +1420,12 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>333</v>
+        <v>158</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:14.000Z</t>
+          <t>2026-07-10T04:47:49.000Z</t>
         </is>
       </c>
     </row>
@@ -1449,12 +1449,12 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>149</v>
+        <v>568</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:15.000Z</t>
+          <t>2026-07-10T04:47:50.000Z</t>
         </is>
       </c>
     </row>
@@ -1478,12 +1478,12 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>332</v>
+        <v>1039</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:16.000Z</t>
+          <t>2026-07-10T04:47:51.000Z</t>
         </is>
       </c>
     </row>
@@ -1507,12 +1507,12 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>811</v>
+        <v>1152</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:17.000Z</t>
+          <t>2026-07-10T04:47:52.000Z</t>
         </is>
       </c>
     </row>
@@ -1536,12 +1536,12 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>138</v>
+        <v>711</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:18.000Z</t>
+          <t>2026-07-10T04:47:52.000Z</t>
         </is>
       </c>
     </row>
@@ -1565,12 +1565,12 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>150</v>
+        <v>410</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:18.000Z</t>
+          <t>2026-07-10T04:47:53.000Z</t>
         </is>
       </c>
     </row>
@@ -1594,12 +1594,12 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>158</v>
+        <v>944</v>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:19.000Z</t>
+          <t>2026-07-10T04:47:54.000Z</t>
         </is>
       </c>
     </row>
@@ -1623,12 +1623,12 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>889</v>
+        <v>1146</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:20.000Z</t>
+          <t>2026-07-10T04:47:55.000Z</t>
         </is>
       </c>
     </row>
@@ -1652,12 +1652,12 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>600</v>
+        <v>876</v>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:21.000Z</t>
+          <t>2026-07-10T04:47:56.000Z</t>
         </is>
       </c>
     </row>
@@ -1681,12 +1681,12 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>882</v>
+        <v>1178</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:22.000Z</t>
+          <t>2026-07-10T04:47:56.000Z</t>
         </is>
       </c>
     </row>
@@ -1710,12 +1710,12 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>260</v>
+        <v>114</v>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:22.000Z</t>
+          <t>2026-07-10T04:47:57.000Z</t>
         </is>
       </c>
     </row>
@@ -1739,12 +1739,12 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>114</v>
+        <v>388</v>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:23.000Z</t>
+          <t>2026-07-10T04:47:58.000Z</t>
         </is>
       </c>
     </row>
@@ -1768,12 +1768,12 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>1122</v>
+        <v>497</v>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:24.000Z</t>
+          <t>2026-07-10T04:47:59.000Z</t>
         </is>
       </c>
     </row>
@@ -1797,12 +1797,12 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>226</v>
+        <v>492</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:25.000Z</t>
+          <t>2026-07-10T04:48:00.000Z</t>
         </is>
       </c>
     </row>
@@ -1826,12 +1826,12 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>1131</v>
+        <v>934</v>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:26.000Z</t>
+          <t>2026-07-10T04:48:00.000Z</t>
         </is>
       </c>
     </row>
@@ -1855,12 +1855,12 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>157</v>
+        <v>718</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:26.000Z</t>
+          <t>2026-07-10T04:48:01.000Z</t>
         </is>
       </c>
     </row>
@@ -1884,12 +1884,12 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>526</v>
+        <v>571</v>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:27.000Z</t>
+          <t>2026-07-10T04:48:02.000Z</t>
         </is>
       </c>
     </row>
@@ -1913,12 +1913,12 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>613</v>
+        <v>991</v>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:28.000Z</t>
+          <t>2026-07-10T04:48:03.000Z</t>
         </is>
       </c>
     </row>
@@ -1942,12 +1942,12 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>905</v>
+        <v>781</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:29.000Z</t>
+          <t>2026-07-10T04:48:04.000Z</t>
         </is>
       </c>
     </row>
@@ -1971,12 +1971,12 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>739</v>
+        <v>689</v>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:30.000Z</t>
+          <t>2026-07-10T04:48:04.000Z</t>
         </is>
       </c>
     </row>
@@ -2000,12 +2000,12 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>697</v>
+        <v>725</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:30.000Z</t>
+          <t>2026-07-10T04:48:05.000Z</t>
         </is>
       </c>
     </row>
@@ -2029,12 +2029,12 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>360</v>
+        <v>489</v>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:31.000Z</t>
+          <t>2026-07-10T04:48:06.000Z</t>
         </is>
       </c>
     </row>
@@ -2058,12 +2058,12 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>782</v>
+        <v>588</v>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:32.000Z</t>
+          <t>2026-07-10T04:48:07.000Z</t>
         </is>
       </c>
     </row>
@@ -2087,12 +2087,12 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>1123</v>
+        <v>303</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:33.000Z</t>
+          <t>2026-07-10T04:48:08.000Z</t>
         </is>
       </c>
     </row>
@@ -2116,12 +2116,12 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>324</v>
+        <v>1020</v>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:34.000Z</t>
+          <t>2026-07-10T04:48:08.000Z</t>
         </is>
       </c>
     </row>
@@ -2145,12 +2145,12 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>152</v>
+        <v>946</v>
       </c>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:34.000Z</t>
+          <t>2026-07-10T04:48:09.000Z</t>
         </is>
       </c>
     </row>
@@ -2174,12 +2174,12 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>526</v>
+        <v>480</v>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:35.000Z</t>
+          <t>2026-07-10T04:48:10.000Z</t>
         </is>
       </c>
     </row>
@@ -2203,12 +2203,12 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>755</v>
+        <v>889</v>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:36.000Z</t>
+          <t>2026-07-10T04:48:11.000Z</t>
         </is>
       </c>
     </row>
@@ -2232,12 +2232,12 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>909</v>
+        <v>355</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:37.000Z</t>
+          <t>2026-07-10T04:48:12.000Z</t>
         </is>
       </c>
     </row>
@@ -2261,12 +2261,12 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>571</v>
+        <v>967</v>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:38.000Z</t>
+          <t>2026-07-10T04:48:12.000Z</t>
         </is>
       </c>
     </row>
@@ -2290,12 +2290,12 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>1174</v>
+        <v>759</v>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:38.000Z</t>
+          <t>2026-07-10T04:48:13.000Z</t>
         </is>
       </c>
     </row>
@@ -2319,12 +2319,12 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>144</v>
+        <v>997</v>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:39.000Z</t>
+          <t>2026-07-10T04:48:14.000Z</t>
         </is>
       </c>
     </row>
@@ -2348,12 +2348,12 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>652</v>
+        <v>313</v>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:40.000Z</t>
+          <t>2026-07-10T04:48:15.000Z</t>
         </is>
       </c>
     </row>
@@ -2377,12 +2377,12 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>1044</v>
+        <v>832</v>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:41.000Z</t>
+          <t>2026-07-10T04:48:16.000Z</t>
         </is>
       </c>
     </row>
@@ -2406,12 +2406,12 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>109</v>
+        <v>896</v>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:42.000Z</t>
+          <t>2026-07-10T04:48:16.000Z</t>
         </is>
       </c>
     </row>
@@ -2435,12 +2435,12 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>963</v>
+        <v>808</v>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:42.000Z</t>
+          <t>2026-07-10T04:48:17.000Z</t>
         </is>
       </c>
     </row>
@@ -2464,12 +2464,12 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>774</v>
+        <v>353</v>
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:43.000Z</t>
+          <t>2026-07-10T04:48:18.000Z</t>
         </is>
       </c>
     </row>
@@ -2493,12 +2493,12 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>566</v>
+        <v>799</v>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:44.000Z</t>
+          <t>2026-07-10T04:48:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2522,12 +2522,12 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>1176</v>
+        <v>803</v>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:45.000Z</t>
+          <t>2026-07-10T04:48:20.000Z</t>
         </is>
       </c>
     </row>
@@ -2551,12 +2551,12 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>670</v>
+        <v>605</v>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:46.000Z</t>
+          <t>2026-07-10T04:48:20.000Z</t>
         </is>
       </c>
     </row>
@@ -2580,12 +2580,12 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>1079</v>
+        <v>989</v>
       </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:46.000Z</t>
+          <t>2026-07-10T04:48:21.000Z</t>
         </is>
       </c>
     </row>
@@ -2609,12 +2609,12 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>185</v>
+        <v>512</v>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:47.000Z</t>
+          <t>2026-07-10T04:48:22.000Z</t>
         </is>
       </c>
     </row>
@@ -2638,12 +2638,12 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>1171</v>
+        <v>986</v>
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:48.000Z</t>
+          <t>2026-07-10T04:48:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2667,12 +2667,12 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>501</v>
+        <v>585</v>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:49.000Z</t>
+          <t>2026-07-10T04:48:24.000Z</t>
         </is>
       </c>
     </row>
@@ -2696,12 +2696,12 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>246</v>
+        <v>168</v>
       </c>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:50.000Z</t>
+          <t>2026-07-10T04:48:24.000Z</t>
         </is>
       </c>
     </row>
@@ -2725,12 +2725,12 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>757</v>
+        <v>106</v>
       </c>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:50.000Z</t>
+          <t>2026-07-10T04:48:25.000Z</t>
         </is>
       </c>
     </row>
@@ -2754,12 +2754,12 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>812</v>
+        <v>317</v>
       </c>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:51.000Z</t>
+          <t>2026-07-10T04:48:26.000Z</t>
         </is>
       </c>
     </row>
@@ -2783,12 +2783,12 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>458</v>
+        <v>847</v>
       </c>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:52.000Z</t>
+          <t>2026-07-10T04:48:27.000Z</t>
         </is>
       </c>
     </row>
@@ -2812,12 +2812,12 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>843</v>
+        <v>1012</v>
       </c>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:53.000Z</t>
+          <t>2026-07-10T04:48:28.000Z</t>
         </is>
       </c>
     </row>
@@ -2841,12 +2841,12 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>359</v>
+        <v>1162</v>
       </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:54.000Z</t>
+          <t>2026-07-10T04:48:28.000Z</t>
         </is>
       </c>
     </row>
@@ -2870,12 +2870,12 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>614</v>
+        <v>559</v>
       </c>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:54.000Z</t>
+          <t>2026-07-10T04:48:29.000Z</t>
         </is>
       </c>
     </row>
@@ -2899,12 +2899,12 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>483</v>
+        <v>839</v>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:55.000Z</t>
+          <t>2026-07-10T04:48:30.000Z</t>
         </is>
       </c>
     </row>
@@ -2928,12 +2928,12 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>758</v>
+        <v>405</v>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:56.000Z</t>
+          <t>2026-07-10T04:48:31.000Z</t>
         </is>
       </c>
     </row>
@@ -2957,12 +2957,12 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>988</v>
+        <v>84</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:57.000Z</t>
+          <t>2026-07-10T04:48:32.000Z</t>
         </is>
       </c>
     </row>
@@ -2986,12 +2986,12 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>566</v>
+        <v>754</v>
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:58.000Z</t>
+          <t>2026-07-10T04:48:32.000Z</t>
         </is>
       </c>
     </row>
@@ -3015,12 +3015,12 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>406</v>
+        <v>906</v>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:58.000Z</t>
+          <t>2026-07-10T04:48:33.000Z</t>
         </is>
       </c>
     </row>
@@ -3044,12 +3044,12 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>773</v>
+        <v>498</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026-07-10T04:32:59.000Z</t>
+          <t>2026-07-10T04:48:34.000Z</t>
         </is>
       </c>
     </row>
@@ -3073,12 +3073,12 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>856</v>
+        <v>295</v>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:00.000Z</t>
+          <t>2026-07-10T04:48:35.000Z</t>
         </is>
       </c>
     </row>
@@ -3102,12 +3102,12 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>653</v>
+        <v>1151</v>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:01.000Z</t>
+          <t>2026-07-10T04:48:36.000Z</t>
         </is>
       </c>
     </row>
@@ -3131,12 +3131,12 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>1091</v>
+        <v>513</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:02.000Z</t>
+          <t>2026-07-10T04:48:36.000Z</t>
         </is>
       </c>
     </row>
@@ -3160,12 +3160,12 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>1153</v>
+        <v>664</v>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:02.000Z</t>
+          <t>2026-07-10T04:48:37.000Z</t>
         </is>
       </c>
     </row>
@@ -3189,12 +3189,12 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>976</v>
+        <v>714</v>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:03.000Z</t>
+          <t>2026-07-10T04:48:38.000Z</t>
         </is>
       </c>
     </row>
@@ -3218,12 +3218,12 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>618</v>
+        <v>814</v>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:04.000Z</t>
+          <t>2026-07-10T04:48:39.000Z</t>
         </is>
       </c>
     </row>
@@ -3247,12 +3247,12 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>123</v>
+        <v>747</v>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:05.000Z</t>
+          <t>2026-07-10T04:48:40.000Z</t>
         </is>
       </c>
     </row>
@@ -3276,12 +3276,12 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>636</v>
+        <v>896</v>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:06.000Z</t>
+          <t>2026-07-10T04:48:40.000Z</t>
         </is>
       </c>
     </row>
@@ -3305,12 +3305,12 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>1116</v>
+        <v>652</v>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:06.000Z</t>
+          <t>2026-07-10T04:48:41.000Z</t>
         </is>
       </c>
     </row>
@@ -3334,12 +3334,12 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>818</v>
+        <v>512</v>
       </c>
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:07.000Z</t>
+          <t>2026-07-10T04:48:42.000Z</t>
         </is>
       </c>
     </row>
@@ -3363,12 +3363,12 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>879</v>
+        <v>656</v>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:08.000Z</t>
+          <t>2026-07-10T04:48:43.000Z</t>
         </is>
       </c>
     </row>
@@ -3392,12 +3392,12 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>985</v>
+        <v>610</v>
       </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:09.000Z</t>
+          <t>2026-07-10T04:48:44.000Z</t>
         </is>
       </c>
     </row>
@@ -3421,12 +3421,12 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>483</v>
+        <v>705</v>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:10.000Z</t>
+          <t>2026-07-10T04:48:44.000Z</t>
         </is>
       </c>
     </row>
@@ -3450,12 +3450,12 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>1015</v>
+        <v>207</v>
       </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:10.000Z</t>
+          <t>2026-07-10T04:48:45.000Z</t>
         </is>
       </c>
     </row>
@@ -3479,12 +3479,12 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>761</v>
+        <v>152</v>
       </c>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:11.000Z</t>
+          <t>2026-07-10T04:48:46.000Z</t>
         </is>
       </c>
     </row>
@@ -3508,12 +3508,12 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>645</v>
+        <v>166</v>
       </c>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:12.000Z</t>
+          <t>2026-07-10T04:48:47.000Z</t>
         </is>
       </c>
     </row>
@@ -3537,12 +3537,12 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>1136</v>
+        <v>909</v>
       </c>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:13.000Z</t>
+          <t>2026-07-10T04:48:48.000Z</t>
         </is>
       </c>
     </row>
@@ -3566,12 +3566,12 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>235</v>
+        <v>792</v>
       </c>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:14.000Z</t>
+          <t>2026-07-10T04:48:48.000Z</t>
         </is>
       </c>
     </row>
@@ -3595,12 +3595,12 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>1031</v>
+        <v>664</v>
       </c>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:14.000Z</t>
+          <t>2026-07-10T04:48:49.000Z</t>
         </is>
       </c>
     </row>
@@ -3624,12 +3624,12 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>188</v>
+        <v>262</v>
       </c>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:15.000Z</t>
+          <t>2026-07-10T04:48:50.000Z</t>
         </is>
       </c>
     </row>
@@ -3653,12 +3653,12 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>696</v>
+        <v>154</v>
       </c>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:16.000Z</t>
+          <t>2026-07-10T04:48:51.000Z</t>
         </is>
       </c>
     </row>
@@ -3682,12 +3682,12 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>542</v>
+        <v>549</v>
       </c>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:17.000Z</t>
+          <t>2026-07-10T04:48:52.000Z</t>
         </is>
       </c>
     </row>
@@ -3711,12 +3711,12 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>1100</v>
+        <v>629</v>
       </c>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:18.000Z</t>
+          <t>2026-07-10T04:48:52.000Z</t>
         </is>
       </c>
     </row>
@@ -3740,12 +3740,12 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>264</v>
+        <v>229</v>
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:18.000Z</t>
+          <t>2026-07-10T04:48:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3769,12 +3769,12 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>1043</v>
+        <v>266</v>
       </c>
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:19.000Z</t>
+          <t>2026-07-10T04:48:54.000Z</t>
         </is>
       </c>
     </row>
@@ -3798,12 +3798,12 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>1065</v>
+        <v>426</v>
       </c>
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:20.000Z</t>
+          <t>2026-07-10T04:48:55.000Z</t>
         </is>
       </c>
     </row>
@@ -3827,12 +3827,12 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>193</v>
+        <v>87</v>
       </c>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:21.000Z</t>
+          <t>2026-07-10T04:48:56.000Z</t>
         </is>
       </c>
     </row>
@@ -3856,12 +3856,12 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>125</v>
+        <v>1003</v>
       </c>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:22.000Z</t>
+          <t>2026-07-10T04:48:56.000Z</t>
         </is>
       </c>
     </row>
@@ -3885,12 +3885,12 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>205</v>
+        <v>264</v>
       </c>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:22.000Z</t>
+          <t>2026-07-10T04:48:57.000Z</t>
         </is>
       </c>
     </row>
@@ -3914,12 +3914,12 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>625</v>
+        <v>1161</v>
       </c>
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:23.000Z</t>
+          <t>2026-07-10T04:48:58.000Z</t>
         </is>
       </c>
     </row>
@@ -3943,12 +3943,12 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>957</v>
+        <v>325</v>
       </c>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:24.000Z</t>
+          <t>2026-07-10T04:48:59.000Z</t>
         </is>
       </c>
     </row>
@@ -3972,12 +3972,12 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>847</v>
+        <v>534</v>
       </c>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:25.000Z</t>
+          <t>2026-07-10T04:49:00.000Z</t>
         </is>
       </c>
     </row>
@@ -4001,12 +4001,12 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>325</v>
+        <v>1034</v>
       </c>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:26.000Z</t>
+          <t>2026-07-10T04:49:00.000Z</t>
         </is>
       </c>
     </row>
@@ -4030,12 +4030,12 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>171</v>
+        <v>999</v>
       </c>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:26.000Z</t>
+          <t>2026-07-10T04:49:01.000Z</t>
         </is>
       </c>
     </row>
@@ -4059,12 +4059,12 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>671</v>
+        <v>1147</v>
       </c>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:27.000Z</t>
+          <t>2026-07-10T04:49:02.000Z</t>
         </is>
       </c>
     </row>
@@ -4088,12 +4088,12 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>1056</v>
+        <v>1127</v>
       </c>
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:28.000Z</t>
+          <t>2026-07-10T04:49:03.000Z</t>
         </is>
       </c>
     </row>
@@ -4117,12 +4117,12 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>144</v>
+        <v>780</v>
       </c>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:29.000Z</t>
+          <t>2026-07-10T04:49:04.000Z</t>
         </is>
       </c>
     </row>
@@ -4146,12 +4146,12 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>536</v>
+        <v>1011</v>
       </c>
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:30.000Z</t>
+          <t>2026-07-10T04:49:04.000Z</t>
         </is>
       </c>
     </row>
@@ -4175,12 +4175,12 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>659</v>
+        <v>1027</v>
       </c>
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:30.000Z</t>
+          <t>2026-07-10T04:49:05.000Z</t>
         </is>
       </c>
     </row>
@@ -4204,12 +4204,12 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>489</v>
+        <v>805</v>
       </c>
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:31.000Z</t>
+          <t>2026-07-10T04:49:06.000Z</t>
         </is>
       </c>
     </row>
@@ -4233,12 +4233,12 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>722</v>
+        <v>801</v>
       </c>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:32.000Z</t>
+          <t>2026-07-10T04:49:07.000Z</t>
         </is>
       </c>
     </row>
@@ -4262,12 +4262,12 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>623</v>
+        <v>1148</v>
       </c>
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:33.000Z</t>
+          <t>2026-07-10T04:49:08.000Z</t>
         </is>
       </c>
     </row>
@@ -4291,12 +4291,12 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>710</v>
+        <v>701</v>
       </c>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:34.000Z</t>
+          <t>2026-07-10T04:49:08.000Z</t>
         </is>
       </c>
     </row>
@@ -4320,12 +4320,12 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>469</v>
+        <v>784</v>
       </c>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:34.000Z</t>
+          <t>2026-07-10T04:49:09.000Z</t>
         </is>
       </c>
     </row>
@@ -4349,12 +4349,12 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>1011</v>
+        <v>664</v>
       </c>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:35.000Z</t>
+          <t>2026-07-10T04:49:10.000Z</t>
         </is>
       </c>
     </row>
@@ -4378,12 +4378,12 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>156</v>
+        <v>932</v>
       </c>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:36.000Z</t>
+          <t>2026-07-10T04:49:11.000Z</t>
         </is>
       </c>
     </row>
@@ -4407,12 +4407,12 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>467</v>
+        <v>1188</v>
       </c>
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:37.000Z</t>
+          <t>2026-07-10T04:49:12.000Z</t>
         </is>
       </c>
     </row>
@@ -4436,12 +4436,12 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>364</v>
+        <v>694</v>
       </c>
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:38.000Z</t>
+          <t>2026-07-10T04:49:12.000Z</t>
         </is>
       </c>
     </row>
@@ -4465,12 +4465,12 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>228</v>
+        <v>469</v>
       </c>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:38.000Z</t>
+          <t>2026-07-10T04:49:13.000Z</t>
         </is>
       </c>
     </row>
@@ -4494,12 +4494,12 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>202</v>
+        <v>806</v>
       </c>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:39.000Z</t>
+          <t>2026-07-10T04:49:14.000Z</t>
         </is>
       </c>
     </row>
@@ -4523,12 +4523,12 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>535</v>
+        <v>338</v>
       </c>
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:40.000Z</t>
+          <t>2026-07-10T04:49:15.000Z</t>
         </is>
       </c>
     </row>
@@ -4552,12 +4552,12 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>292</v>
+        <v>424</v>
       </c>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:41.000Z</t>
+          <t>2026-07-10T04:49:16.000Z</t>
         </is>
       </c>
     </row>
@@ -4581,12 +4581,12 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>566</v>
+        <v>810</v>
       </c>
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:42.000Z</t>
+          <t>2026-07-10T04:49:16.000Z</t>
         </is>
       </c>
     </row>
@@ -4610,12 +4610,12 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>694</v>
+        <v>144</v>
       </c>
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:42.000Z</t>
+          <t>2026-07-10T04:49:17.000Z</t>
         </is>
       </c>
     </row>
@@ -4639,12 +4639,12 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>773</v>
+        <v>962</v>
       </c>
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:43.000Z</t>
+          <t>2026-07-10T04:49:18.000Z</t>
         </is>
       </c>
     </row>
@@ -4668,12 +4668,12 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>413</v>
+        <v>332</v>
       </c>
       <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:44.000Z</t>
+          <t>2026-07-10T04:49:19.000Z</t>
         </is>
       </c>
     </row>
@@ -4697,12 +4697,12 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>922</v>
+        <v>883</v>
       </c>
       <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:45.000Z</t>
+          <t>2026-07-10T04:49:20.000Z</t>
         </is>
       </c>
     </row>
@@ -4726,12 +4726,12 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>458</v>
+        <v>697</v>
       </c>
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:46.000Z</t>
+          <t>2026-07-10T04:49:20.000Z</t>
         </is>
       </c>
     </row>
@@ -4755,12 +4755,12 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>450</v>
+        <v>895</v>
       </c>
       <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:46.000Z</t>
+          <t>2026-07-10T04:49:21.000Z</t>
         </is>
       </c>
     </row>
@@ -4784,12 +4784,12 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>735</v>
+        <v>1186</v>
       </c>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:47.000Z</t>
+          <t>2026-07-10T04:49:22.000Z</t>
         </is>
       </c>
     </row>
@@ -4813,12 +4813,12 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>1200</v>
+        <v>266</v>
       </c>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:48.000Z</t>
+          <t>2026-07-10T04:49:23.000Z</t>
         </is>
       </c>
     </row>
@@ -4842,12 +4842,12 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>229</v>
+        <v>1189</v>
       </c>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:49.000Z</t>
+          <t>2026-07-10T04:49:24.000Z</t>
         </is>
       </c>
     </row>
@@ -4871,12 +4871,12 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>497</v>
+        <v>294</v>
       </c>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:50.000Z</t>
+          <t>2026-07-10T04:49:24.000Z</t>
         </is>
       </c>
     </row>
@@ -4900,12 +4900,12 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>422</v>
+        <v>269</v>
       </c>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:50.000Z</t>
+          <t>2026-07-10T04:49:25.000Z</t>
         </is>
       </c>
     </row>
@@ -4929,12 +4929,12 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>513</v>
+        <v>956</v>
       </c>
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:51.000Z</t>
+          <t>2026-07-10T04:49:26.000Z</t>
         </is>
       </c>
     </row>
@@ -4958,12 +4958,12 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>1185</v>
+        <v>867</v>
       </c>
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:52.000Z</t>
+          <t>2026-07-10T04:49:27.000Z</t>
         </is>
       </c>
     </row>
@@ -4987,12 +4987,12 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>460</v>
+        <v>200</v>
       </c>
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:53.000Z</t>
+          <t>2026-07-10T04:49:28.000Z</t>
         </is>
       </c>
     </row>
@@ -5016,12 +5016,12 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>1126</v>
+        <v>1116</v>
       </c>
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:54.000Z</t>
+          <t>2026-07-10T04:49:28.000Z</t>
         </is>
       </c>
     </row>
@@ -5045,12 +5045,12 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>448</v>
+        <v>488</v>
       </c>
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:54.000Z</t>
+          <t>2026-07-10T04:49:29.000Z</t>
         </is>
       </c>
     </row>
@@ -5074,12 +5074,12 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>962</v>
+        <v>283</v>
       </c>
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:55.000Z</t>
+          <t>2026-07-10T04:49:30.000Z</t>
         </is>
       </c>
     </row>
@@ -5103,12 +5103,12 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>738</v>
+        <v>313</v>
       </c>
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:56.000Z</t>
+          <t>2026-07-10T04:49:31.000Z</t>
         </is>
       </c>
     </row>
@@ -5132,12 +5132,12 @@
         </is>
       </c>
       <c r="E161" t="n">
-        <v>887</v>
+        <v>82</v>
       </c>
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:57.000Z</t>
+          <t>2026-07-10T04:49:32.000Z</t>
         </is>
       </c>
     </row>
@@ -5161,12 +5161,12 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>652</v>
+        <v>207</v>
       </c>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:58.000Z</t>
+          <t>2026-07-10T04:49:32.000Z</t>
         </is>
       </c>
     </row>
@@ -5190,12 +5190,12 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>188</v>
+        <v>1129</v>
       </c>
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:58.000Z</t>
+          <t>2026-07-10T04:49:33.000Z</t>
         </is>
       </c>
     </row>
@@ -5219,12 +5219,12 @@
         </is>
       </c>
       <c r="E164" t="n">
-        <v>899</v>
+        <v>395</v>
       </c>
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
-          <t>2026-07-10T04:33:59.000Z</t>
+          <t>2026-07-10T04:49:34.000Z</t>
         </is>
       </c>
     </row>
@@ -5248,12 +5248,12 @@
         </is>
       </c>
       <c r="E165" t="n">
-        <v>767</v>
+        <v>1179</v>
       </c>
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:00.000Z</t>
+          <t>2026-07-10T04:49:35.000Z</t>
         </is>
       </c>
     </row>
@@ -5277,12 +5277,12 @@
         </is>
       </c>
       <c r="E166" t="n">
-        <v>450</v>
+        <v>1058</v>
       </c>
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:01.000Z</t>
+          <t>2026-07-10T04:49:36.000Z</t>
         </is>
       </c>
     </row>
@@ -5306,12 +5306,12 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>589</v>
+        <v>271</v>
       </c>
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:02.000Z</t>
+          <t>2026-07-10T04:49:36.000Z</t>
         </is>
       </c>
     </row>
@@ -5335,12 +5335,12 @@
         </is>
       </c>
       <c r="E168" t="n">
-        <v>757</v>
+        <v>276</v>
       </c>
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:02.000Z</t>
+          <t>2026-07-10T04:49:37.000Z</t>
         </is>
       </c>
     </row>
@@ -5364,12 +5364,12 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>1162</v>
+        <v>934</v>
       </c>
       <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:03.000Z</t>
+          <t>2026-07-10T04:49:38.000Z</t>
         </is>
       </c>
     </row>
@@ -5393,12 +5393,12 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>1166</v>
+        <v>96</v>
       </c>
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:04.000Z</t>
+          <t>2026-07-10T04:49:39.000Z</t>
         </is>
       </c>
     </row>
@@ -5422,12 +5422,12 @@
         </is>
       </c>
       <c r="E171" t="n">
-        <v>1112</v>
+        <v>649</v>
       </c>
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:05.000Z</t>
+          <t>2026-07-10T04:49:40.000Z</t>
         </is>
       </c>
     </row>
@@ -5451,12 +5451,12 @@
         </is>
       </c>
       <c r="E172" t="n">
-        <v>121</v>
+        <v>745</v>
       </c>
       <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:06.000Z</t>
+          <t>2026-07-10T04:49:40.000Z</t>
         </is>
       </c>
     </row>
@@ -5480,12 +5480,12 @@
         </is>
       </c>
       <c r="E173" t="n">
-        <v>264</v>
+        <v>678</v>
       </c>
       <c r="F173" t="inlineStr"/>
       <c r="G173" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:06.000Z</t>
+          <t>2026-07-10T04:49:41.000Z</t>
         </is>
       </c>
     </row>
@@ -5509,12 +5509,12 @@
         </is>
       </c>
       <c r="E174" t="n">
-        <v>499</v>
+        <v>1030</v>
       </c>
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:07.000Z</t>
+          <t>2026-07-10T04:49:42.000Z</t>
         </is>
       </c>
     </row>
@@ -5538,12 +5538,12 @@
         </is>
       </c>
       <c r="E175" t="n">
-        <v>776</v>
+        <v>796</v>
       </c>
       <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:08.000Z</t>
+          <t>2026-07-10T04:49:43.000Z</t>
         </is>
       </c>
     </row>
@@ -5567,12 +5567,12 @@
         </is>
       </c>
       <c r="E176" t="n">
-        <v>657</v>
+        <v>263</v>
       </c>
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:09.000Z</t>
+          <t>2026-07-10T04:49:44.000Z</t>
         </is>
       </c>
     </row>
@@ -5596,12 +5596,12 @@
         </is>
       </c>
       <c r="E177" t="n">
-        <v>353</v>
+        <v>1014</v>
       </c>
       <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:10.000Z</t>
+          <t>2026-07-10T04:49:44.000Z</t>
         </is>
       </c>
     </row>
@@ -5625,12 +5625,12 @@
         </is>
       </c>
       <c r="E178" t="n">
-        <v>878</v>
+        <v>905</v>
       </c>
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:10.000Z</t>
+          <t>2026-07-10T04:49:45.000Z</t>
         </is>
       </c>
     </row>
@@ -5654,12 +5654,12 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>861</v>
+        <v>180</v>
       </c>
       <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:11.000Z</t>
+          <t>2026-07-10T04:49:46.000Z</t>
         </is>
       </c>
     </row>
@@ -5683,12 +5683,12 @@
         </is>
       </c>
       <c r="E180" t="n">
-        <v>162</v>
+        <v>812</v>
       </c>
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:12.000Z</t>
+          <t>2026-07-10T04:49:47.000Z</t>
         </is>
       </c>
     </row>
@@ -5712,12 +5712,12 @@
         </is>
       </c>
       <c r="E181" t="n">
-        <v>228</v>
+        <v>1176</v>
       </c>
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:13.000Z</t>
+          <t>2026-07-10T04:49:48.000Z</t>
         </is>
       </c>
     </row>
@@ -5741,12 +5741,12 @@
         </is>
       </c>
       <c r="E182" t="n">
-        <v>925</v>
+        <v>241</v>
       </c>
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:14.000Z</t>
+          <t>2026-07-10T04:49:48.000Z</t>
         </is>
       </c>
     </row>
@@ -5770,12 +5770,12 @@
         </is>
       </c>
       <c r="E183" t="n">
-        <v>242</v>
+        <v>577</v>
       </c>
       <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:14.000Z</t>
+          <t>2026-07-10T04:49:49.000Z</t>
         </is>
       </c>
     </row>
@@ -5799,12 +5799,12 @@
         </is>
       </c>
       <c r="E184" t="n">
-        <v>689</v>
+        <v>617</v>
       </c>
       <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:15.000Z</t>
+          <t>2026-07-10T04:49:50.000Z</t>
         </is>
       </c>
     </row>
@@ -5828,12 +5828,12 @@
         </is>
       </c>
       <c r="E185" t="n">
-        <v>349</v>
+        <v>1098</v>
       </c>
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:16.000Z</t>
+          <t>2026-07-10T04:49:51.000Z</t>
         </is>
       </c>
     </row>
@@ -5857,12 +5857,12 @@
         </is>
       </c>
       <c r="E186" t="n">
-        <v>747</v>
+        <v>818</v>
       </c>
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:17.000Z</t>
+          <t>2026-07-10T04:49:52.000Z</t>
         </is>
       </c>
     </row>
@@ -5886,12 +5886,12 @@
         </is>
       </c>
       <c r="E187" t="n">
-        <v>567</v>
+        <v>287</v>
       </c>
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:18.000Z</t>
+          <t>2026-07-10T04:49:52.000Z</t>
         </is>
       </c>
     </row>
@@ -5915,12 +5915,12 @@
         </is>
       </c>
       <c r="E188" t="n">
-        <v>192</v>
+        <v>817</v>
       </c>
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:18.000Z</t>
+          <t>2026-07-10T04:49:53.000Z</t>
         </is>
       </c>
     </row>
@@ -5944,12 +5944,12 @@
         </is>
       </c>
       <c r="E189" t="n">
-        <v>211</v>
+        <v>769</v>
       </c>
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:19.000Z</t>
+          <t>2026-07-10T04:49:54.000Z</t>
         </is>
       </c>
     </row>
@@ -5973,12 +5973,12 @@
         </is>
       </c>
       <c r="E190" t="n">
-        <v>621</v>
+        <v>462</v>
       </c>
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:20.000Z</t>
+          <t>2026-07-10T04:49:55.000Z</t>
         </is>
       </c>
     </row>
@@ -6002,12 +6002,12 @@
         </is>
       </c>
       <c r="E191" t="n">
-        <v>343</v>
+        <v>759</v>
       </c>
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:21.000Z</t>
+          <t>2026-07-10T04:49:56.000Z</t>
         </is>
       </c>
     </row>
@@ -6031,12 +6031,12 @@
         </is>
       </c>
       <c r="E192" t="n">
-        <v>896</v>
+        <v>1029</v>
       </c>
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:22.000Z</t>
+          <t>2026-07-10T04:49:56.000Z</t>
         </is>
       </c>
     </row>
@@ -6060,12 +6060,12 @@
         </is>
       </c>
       <c r="E193" t="n">
-        <v>513</v>
+        <v>509</v>
       </c>
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:22.000Z</t>
+          <t>2026-07-10T04:49:57.000Z</t>
         </is>
       </c>
     </row>
@@ -6089,12 +6089,12 @@
         </is>
       </c>
       <c r="E194" t="n">
-        <v>134</v>
+        <v>357</v>
       </c>
       <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:23.000Z</t>
+          <t>2026-07-10T04:49:58.000Z</t>
         </is>
       </c>
     </row>
@@ -6118,12 +6118,12 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>150</v>
+        <v>729</v>
       </c>
       <c r="F195" t="inlineStr"/>
       <c r="G195" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:24.000Z</t>
+          <t>2026-07-10T04:49:59.000Z</t>
         </is>
       </c>
     </row>
@@ -6147,12 +6147,12 @@
         </is>
       </c>
       <c r="E196" t="n">
-        <v>849</v>
+        <v>660</v>
       </c>
       <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:25.000Z</t>
+          <t>2026-07-10T04:50:00.000Z</t>
         </is>
       </c>
     </row>
@@ -6176,12 +6176,12 @@
         </is>
       </c>
       <c r="E197" t="n">
-        <v>903</v>
+        <v>359</v>
       </c>
       <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:26.000Z</t>
+          <t>2026-07-10T04:50:00.000Z</t>
         </is>
       </c>
     </row>
@@ -6205,12 +6205,12 @@
         </is>
       </c>
       <c r="E198" t="n">
-        <v>179</v>
+        <v>942</v>
       </c>
       <c r="F198" t="inlineStr"/>
       <c r="G198" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:26.000Z</t>
+          <t>2026-07-10T04:50:01.000Z</t>
         </is>
       </c>
     </row>
@@ -6234,12 +6234,12 @@
         </is>
       </c>
       <c r="E199" t="n">
-        <v>1046</v>
+        <v>219</v>
       </c>
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:27.000Z</t>
+          <t>2026-07-10T04:50:02.000Z</t>
         </is>
       </c>
     </row>
@@ -6263,12 +6263,12 @@
         </is>
       </c>
       <c r="E200" t="n">
-        <v>251</v>
+        <v>1179</v>
       </c>
       <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:28.000Z</t>
+          <t>2026-07-10T04:50:03.000Z</t>
         </is>
       </c>
     </row>
@@ -6292,12 +6292,12 @@
         </is>
       </c>
       <c r="E201" t="n">
-        <v>305</v>
+        <v>1183</v>
       </c>
       <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:29.000Z</t>
+          <t>2026-07-10T04:50:04.000Z</t>
         </is>
       </c>
     </row>
@@ -6321,12 +6321,12 @@
         </is>
       </c>
       <c r="E202" t="n">
-        <v>881</v>
+        <v>763</v>
       </c>
       <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:30.000Z</t>
+          <t>2026-07-10T04:50:04.000Z</t>
         </is>
       </c>
     </row>
@@ -6350,12 +6350,12 @@
         </is>
       </c>
       <c r="E203" t="n">
-        <v>803</v>
+        <v>685</v>
       </c>
       <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:30.000Z</t>
+          <t>2026-07-10T04:50:05.000Z</t>
         </is>
       </c>
     </row>
@@ -6379,12 +6379,12 @@
         </is>
       </c>
       <c r="E204" t="n">
-        <v>623</v>
+        <v>109</v>
       </c>
       <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:31.000Z</t>
+          <t>2026-07-10T04:50:06.000Z</t>
         </is>
       </c>
     </row>
@@ -6408,12 +6408,12 @@
         </is>
       </c>
       <c r="E205" t="n">
-        <v>723</v>
+        <v>563</v>
       </c>
       <c r="F205" t="inlineStr"/>
       <c r="G205" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:32.000Z</t>
+          <t>2026-07-10T04:50:07.000Z</t>
         </is>
       </c>
     </row>
@@ -6437,12 +6437,12 @@
         </is>
       </c>
       <c r="E206" t="n">
-        <v>986</v>
+        <v>315</v>
       </c>
       <c r="F206" t="inlineStr"/>
       <c r="G206" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:33.000Z</t>
+          <t>2026-07-10T04:50:08.000Z</t>
         </is>
       </c>
     </row>
@@ -6466,12 +6466,12 @@
         </is>
       </c>
       <c r="E207" t="n">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="F207" t="inlineStr"/>
       <c r="G207" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:34.000Z</t>
+          <t>2026-07-10T04:50:08.000Z</t>
         </is>
       </c>
     </row>
@@ -6495,12 +6495,12 @@
         </is>
       </c>
       <c r="E208" t="n">
-        <v>1036</v>
+        <v>205</v>
       </c>
       <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:34.000Z</t>
+          <t>2026-07-10T04:50:09.000Z</t>
         </is>
       </c>
     </row>
@@ -6524,12 +6524,12 @@
         </is>
       </c>
       <c r="E209" t="n">
-        <v>632</v>
+        <v>326</v>
       </c>
       <c r="F209" t="inlineStr"/>
       <c r="G209" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:35.000Z</t>
+          <t>2026-07-10T04:50:10.000Z</t>
         </is>
       </c>
     </row>
@@ -6553,12 +6553,12 @@
         </is>
       </c>
       <c r="E210" t="n">
-        <v>526</v>
+        <v>854</v>
       </c>
       <c r="F210" t="inlineStr"/>
       <c r="G210" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:36.000Z</t>
+          <t>2026-07-10T04:50:11.000Z</t>
         </is>
       </c>
     </row>
@@ -6582,12 +6582,12 @@
         </is>
       </c>
       <c r="E211" t="n">
-        <v>446</v>
+        <v>916</v>
       </c>
       <c r="F211" t="inlineStr"/>
       <c r="G211" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:37.000Z</t>
+          <t>2026-07-10T04:50:12.000Z</t>
         </is>
       </c>
     </row>
@@ -6611,12 +6611,12 @@
         </is>
       </c>
       <c r="E212" t="n">
-        <v>1132</v>
+        <v>755</v>
       </c>
       <c r="F212" t="inlineStr"/>
       <c r="G212" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:38.000Z</t>
+          <t>2026-07-10T04:50:12.000Z</t>
         </is>
       </c>
     </row>
@@ -6640,12 +6640,12 @@
         </is>
       </c>
       <c r="E213" t="n">
-        <v>1151</v>
+        <v>839</v>
       </c>
       <c r="F213" t="inlineStr"/>
       <c r="G213" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:38.000Z</t>
+          <t>2026-07-10T04:50:13.000Z</t>
         </is>
       </c>
     </row>
@@ -6669,12 +6669,12 @@
         </is>
       </c>
       <c r="E214" t="n">
-        <v>952</v>
+        <v>772</v>
       </c>
       <c r="F214" t="inlineStr"/>
       <c r="G214" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:39.000Z</t>
+          <t>2026-07-10T04:50:14.000Z</t>
         </is>
       </c>
     </row>
@@ -6698,12 +6698,12 @@
         </is>
       </c>
       <c r="E215" t="n">
-        <v>713</v>
+        <v>892</v>
       </c>
       <c r="F215" t="inlineStr"/>
       <c r="G215" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:40.000Z</t>
+          <t>2026-07-10T04:50:15.000Z</t>
         </is>
       </c>
     </row>
@@ -6727,12 +6727,12 @@
         </is>
       </c>
       <c r="E216" t="n">
-        <v>406</v>
+        <v>623</v>
       </c>
       <c r="F216" t="inlineStr"/>
       <c r="G216" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:41.000Z</t>
+          <t>2026-07-10T04:50:16.000Z</t>
         </is>
       </c>
     </row>
@@ -6756,12 +6756,12 @@
         </is>
       </c>
       <c r="E217" t="n">
-        <v>332</v>
+        <v>401</v>
       </c>
       <c r="F217" t="inlineStr"/>
       <c r="G217" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:42.000Z</t>
+          <t>2026-07-10T04:50:16.000Z</t>
         </is>
       </c>
     </row>
@@ -6785,12 +6785,12 @@
         </is>
       </c>
       <c r="E218" t="n">
-        <v>231</v>
+        <v>395</v>
       </c>
       <c r="F218" t="inlineStr"/>
       <c r="G218" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:42.000Z</t>
+          <t>2026-07-10T04:50:17.000Z</t>
         </is>
       </c>
     </row>
@@ -6814,12 +6814,12 @@
         </is>
       </c>
       <c r="E219" t="n">
-        <v>590</v>
+        <v>927</v>
       </c>
       <c r="F219" t="inlineStr"/>
       <c r="G219" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:43.000Z</t>
+          <t>2026-07-10T04:50:18.000Z</t>
         </is>
       </c>
     </row>
@@ -6843,12 +6843,12 @@
         </is>
       </c>
       <c r="E220" t="n">
-        <v>279</v>
+        <v>1158</v>
       </c>
       <c r="F220" t="inlineStr"/>
       <c r="G220" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:44.000Z</t>
+          <t>2026-07-10T04:50:19.000Z</t>
         </is>
       </c>
     </row>
@@ -6872,12 +6872,12 @@
         </is>
       </c>
       <c r="E221" t="n">
-        <v>529</v>
+        <v>1107</v>
       </c>
       <c r="F221" t="inlineStr"/>
       <c r="G221" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:45.000Z</t>
+          <t>2026-07-10T04:50:20.000Z</t>
         </is>
       </c>
     </row>
@@ -6901,12 +6901,12 @@
         </is>
       </c>
       <c r="E222" t="n">
-        <v>1132</v>
+        <v>523</v>
       </c>
       <c r="F222" t="inlineStr"/>
       <c r="G222" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:46.000Z</t>
+          <t>2026-07-10T04:50:20.000Z</t>
         </is>
       </c>
     </row>
@@ -6930,12 +6930,12 @@
         </is>
       </c>
       <c r="E223" t="n">
-        <v>380</v>
+        <v>367</v>
       </c>
       <c r="F223" t="inlineStr"/>
       <c r="G223" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:46.000Z</t>
+          <t>2026-07-10T04:50:21.000Z</t>
         </is>
       </c>
     </row>
@@ -6959,12 +6959,12 @@
         </is>
       </c>
       <c r="E224" t="n">
-        <v>736</v>
+        <v>1088</v>
       </c>
       <c r="F224" t="inlineStr"/>
       <c r="G224" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:47.000Z</t>
+          <t>2026-07-10T04:50:22.000Z</t>
         </is>
       </c>
     </row>
@@ -6988,12 +6988,12 @@
         </is>
       </c>
       <c r="E225" t="n">
-        <v>244</v>
+        <v>502</v>
       </c>
       <c r="F225" t="inlineStr"/>
       <c r="G225" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:48.000Z</t>
+          <t>2026-07-10T04:50:23.000Z</t>
         </is>
       </c>
     </row>
@@ -7017,12 +7017,12 @@
         </is>
       </c>
       <c r="E226" t="n">
-        <v>1185</v>
+        <v>1106</v>
       </c>
       <c r="F226" t="inlineStr"/>
       <c r="G226" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:49.000Z</t>
+          <t>2026-07-10T04:50:24.000Z</t>
         </is>
       </c>
     </row>
@@ -7046,12 +7046,12 @@
         </is>
       </c>
       <c r="E227" t="n">
-        <v>887</v>
+        <v>228</v>
       </c>
       <c r="F227" t="inlineStr"/>
       <c r="G227" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:50.000Z</t>
+          <t>2026-07-10T04:50:24.000Z</t>
         </is>
       </c>
     </row>
@@ -7075,12 +7075,12 @@
         </is>
       </c>
       <c r="E228" t="n">
-        <v>398</v>
+        <v>258</v>
       </c>
       <c r="F228" t="inlineStr"/>
       <c r="G228" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:50.000Z</t>
+          <t>2026-07-10T04:50:25.000Z</t>
         </is>
       </c>
     </row>
@@ -7104,12 +7104,12 @@
         </is>
       </c>
       <c r="E229" t="n">
-        <v>954</v>
+        <v>346</v>
       </c>
       <c r="F229" t="inlineStr"/>
       <c r="G229" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:51.000Z</t>
+          <t>2026-07-10T04:50:26.000Z</t>
         </is>
       </c>
     </row>
@@ -7133,12 +7133,12 @@
         </is>
       </c>
       <c r="E230" t="n">
-        <v>522</v>
+        <v>735</v>
       </c>
       <c r="F230" t="inlineStr"/>
       <c r="G230" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:52.000Z</t>
+          <t>2026-07-10T04:50:27.000Z</t>
         </is>
       </c>
     </row>
@@ -7162,12 +7162,12 @@
         </is>
       </c>
       <c r="E231" t="n">
-        <v>106</v>
+        <v>618</v>
       </c>
       <c r="F231" t="inlineStr"/>
       <c r="G231" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:53.000Z</t>
+          <t>2026-07-10T04:50:28.000Z</t>
         </is>
       </c>
     </row>
@@ -7191,12 +7191,12 @@
         </is>
       </c>
       <c r="E232" t="n">
-        <v>431</v>
+        <v>727</v>
       </c>
       <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:54.000Z</t>
+          <t>2026-07-10T04:50:28.000Z</t>
         </is>
       </c>
     </row>
@@ -7220,12 +7220,12 @@
         </is>
       </c>
       <c r="E233" t="n">
-        <v>98</v>
+        <v>998</v>
       </c>
       <c r="F233" t="inlineStr"/>
       <c r="G233" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:54.000Z</t>
+          <t>2026-07-10T04:50:29.000Z</t>
         </is>
       </c>
     </row>
@@ -7249,12 +7249,12 @@
         </is>
       </c>
       <c r="E234" t="n">
-        <v>126</v>
+        <v>247</v>
       </c>
       <c r="F234" t="inlineStr"/>
       <c r="G234" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:55.000Z</t>
+          <t>2026-07-10T04:50:30.000Z</t>
         </is>
       </c>
     </row>
@@ -7278,12 +7278,12 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>1050</v>
+        <v>564</v>
       </c>
       <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:56.000Z</t>
+          <t>2026-07-10T04:50:31.000Z</t>
         </is>
       </c>
     </row>
@@ -7307,12 +7307,12 @@
         </is>
       </c>
       <c r="E236" t="n">
-        <v>541</v>
+        <v>968</v>
       </c>
       <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:57.000Z</t>
+          <t>2026-07-10T04:50:32.000Z</t>
         </is>
       </c>
     </row>
@@ -7336,12 +7336,12 @@
         </is>
       </c>
       <c r="E237" t="n">
-        <v>695</v>
+        <v>944</v>
       </c>
       <c r="F237" t="inlineStr"/>
       <c r="G237" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:58.000Z</t>
+          <t>2026-07-10T04:50:32.000Z</t>
         </is>
       </c>
     </row>
@@ -7365,12 +7365,12 @@
         </is>
       </c>
       <c r="E238" t="n">
-        <v>1190</v>
+        <v>316</v>
       </c>
       <c r="F238" t="inlineStr"/>
       <c r="G238" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:58.000Z</t>
+          <t>2026-07-10T04:50:33.000Z</t>
         </is>
       </c>
     </row>
@@ -7394,12 +7394,12 @@
         </is>
       </c>
       <c r="E239" t="n">
-        <v>232</v>
+        <v>1178</v>
       </c>
       <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
-          <t>2026-07-10T04:34:59.000Z</t>
+          <t>2026-07-10T04:50:34.000Z</t>
         </is>
       </c>
     </row>
@@ -7423,12 +7423,12 @@
         </is>
       </c>
       <c r="E240" t="n">
-        <v>490</v>
+        <v>784</v>
       </c>
       <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:00.000Z</t>
+          <t>2026-07-10T04:50:35.000Z</t>
         </is>
       </c>
     </row>
@@ -7452,12 +7452,12 @@
         </is>
       </c>
       <c r="E241" t="n">
-        <v>481</v>
+        <v>457</v>
       </c>
       <c r="F241" t="inlineStr"/>
       <c r="G241" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:01.000Z</t>
+          <t>2026-07-10T04:50:36.000Z</t>
         </is>
       </c>
     </row>
@@ -7481,12 +7481,12 @@
         </is>
       </c>
       <c r="E242" t="n">
-        <v>886</v>
+        <v>646</v>
       </c>
       <c r="F242" t="inlineStr"/>
       <c r="G242" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:02.000Z</t>
+          <t>2026-07-10T04:50:36.000Z</t>
         </is>
       </c>
     </row>
@@ -7510,12 +7510,12 @@
         </is>
       </c>
       <c r="E243" t="n">
-        <v>91</v>
+        <v>1161</v>
       </c>
       <c r="F243" t="inlineStr"/>
       <c r="G243" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:02.000Z</t>
+          <t>2026-07-10T04:50:37.000Z</t>
         </is>
       </c>
     </row>
@@ -7539,12 +7539,12 @@
         </is>
       </c>
       <c r="E244" t="n">
-        <v>223</v>
+        <v>821</v>
       </c>
       <c r="F244" t="inlineStr"/>
       <c r="G244" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:03.000Z</t>
+          <t>2026-07-10T04:50:38.000Z</t>
         </is>
       </c>
     </row>
@@ -7568,12 +7568,12 @@
         </is>
       </c>
       <c r="E245" t="n">
-        <v>1164</v>
+        <v>1057</v>
       </c>
       <c r="F245" t="inlineStr"/>
       <c r="G245" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:04.000Z</t>
+          <t>2026-07-10T04:50:39.000Z</t>
         </is>
       </c>
     </row>
@@ -7597,12 +7597,12 @@
         </is>
       </c>
       <c r="E246" t="n">
-        <v>825</v>
+        <v>677</v>
       </c>
       <c r="F246" t="inlineStr"/>
       <c r="G246" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:05.000Z</t>
+          <t>2026-07-10T04:50:40.000Z</t>
         </is>
       </c>
     </row>
@@ -7626,12 +7626,12 @@
         </is>
       </c>
       <c r="E247" t="n">
-        <v>450</v>
+        <v>775</v>
       </c>
       <c r="F247" t="inlineStr"/>
       <c r="G247" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:06.000Z</t>
+          <t>2026-07-10T04:50:40.000Z</t>
         </is>
       </c>
     </row>
@@ -7655,12 +7655,12 @@
         </is>
       </c>
       <c r="E248" t="n">
-        <v>799</v>
+        <v>178</v>
       </c>
       <c r="F248" t="inlineStr"/>
       <c r="G248" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:06.000Z</t>
+          <t>2026-07-10T04:50:41.000Z</t>
         </is>
       </c>
     </row>
@@ -7684,12 +7684,12 @@
         </is>
       </c>
       <c r="E249" t="n">
-        <v>1000</v>
+        <v>240</v>
       </c>
       <c r="F249" t="inlineStr"/>
       <c r="G249" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:07.000Z</t>
+          <t>2026-07-10T04:50:42.000Z</t>
         </is>
       </c>
     </row>
@@ -7713,12 +7713,12 @@
         </is>
       </c>
       <c r="E250" t="n">
-        <v>1094</v>
+        <v>1010</v>
       </c>
       <c r="F250" t="inlineStr"/>
       <c r="G250" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:08.000Z</t>
+          <t>2026-07-10T04:50:43.000Z</t>
         </is>
       </c>
     </row>
@@ -7742,12 +7742,12 @@
         </is>
       </c>
       <c r="E251" t="n">
-        <v>1024</v>
+        <v>952</v>
       </c>
       <c r="F251" t="inlineStr"/>
       <c r="G251" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:09.000Z</t>
+          <t>2026-07-10T04:50:44.000Z</t>
         </is>
       </c>
     </row>
@@ -7771,12 +7771,12 @@
         </is>
       </c>
       <c r="E252" t="n">
-        <v>306</v>
+        <v>983</v>
       </c>
       <c r="F252" t="inlineStr"/>
       <c r="G252" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:10.000Z</t>
+          <t>2026-07-10T04:50:44.000Z</t>
         </is>
       </c>
     </row>
@@ -7800,12 +7800,12 @@
         </is>
       </c>
       <c r="E253" t="n">
-        <v>121</v>
+        <v>767</v>
       </c>
       <c r="F253" t="inlineStr"/>
       <c r="G253" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:10.000Z</t>
+          <t>2026-07-10T04:50:45.000Z</t>
         </is>
       </c>
     </row>
@@ -7829,12 +7829,12 @@
         </is>
       </c>
       <c r="E254" t="n">
-        <v>887</v>
+        <v>552</v>
       </c>
       <c r="F254" t="inlineStr"/>
       <c r="G254" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:11.000Z</t>
+          <t>2026-07-10T04:50:46.000Z</t>
         </is>
       </c>
     </row>
@@ -7858,12 +7858,12 @@
         </is>
       </c>
       <c r="E255" t="n">
-        <v>738</v>
+        <v>729</v>
       </c>
       <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:12.000Z</t>
+          <t>2026-07-10T04:50:47.000Z</t>
         </is>
       </c>
     </row>
@@ -7887,12 +7887,12 @@
         </is>
       </c>
       <c r="E256" t="n">
-        <v>659</v>
+        <v>1075</v>
       </c>
       <c r="F256" t="inlineStr"/>
       <c r="G256" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:13.000Z</t>
+          <t>2026-07-10T04:50:48.000Z</t>
         </is>
       </c>
     </row>
@@ -7916,12 +7916,12 @@
         </is>
       </c>
       <c r="E257" t="n">
-        <v>657</v>
+        <v>163</v>
       </c>
       <c r="F257" t="inlineStr"/>
       <c r="G257" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:14.000Z</t>
+          <t>2026-07-10T04:50:48.000Z</t>
         </is>
       </c>
     </row>
@@ -7945,12 +7945,12 @@
         </is>
       </c>
       <c r="E258" t="n">
-        <v>158</v>
+        <v>244</v>
       </c>
       <c r="F258" t="inlineStr"/>
       <c r="G258" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:14.000Z</t>
+          <t>2026-07-10T04:50:49.000Z</t>
         </is>
       </c>
     </row>
@@ -7974,12 +7974,12 @@
         </is>
       </c>
       <c r="E259" t="n">
-        <v>626</v>
+        <v>333</v>
       </c>
       <c r="F259" t="inlineStr"/>
       <c r="G259" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:15.000Z</t>
+          <t>2026-07-10T04:50:50.000Z</t>
         </is>
       </c>
     </row>
@@ -8003,12 +8003,12 @@
         </is>
       </c>
       <c r="E260" t="n">
-        <v>507</v>
+        <v>1038</v>
       </c>
       <c r="F260" t="inlineStr"/>
       <c r="G260" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:16.000Z</t>
+          <t>2026-07-10T04:50:51.000Z</t>
         </is>
       </c>
     </row>
@@ -8032,12 +8032,12 @@
         </is>
       </c>
       <c r="E261" t="n">
-        <v>270</v>
+        <v>364</v>
       </c>
       <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:17.000Z</t>
+          <t>2026-07-10T04:50:52.000Z</t>
         </is>
       </c>
     </row>
@@ -8061,12 +8061,12 @@
         </is>
       </c>
       <c r="E262" t="n">
-        <v>307</v>
+        <v>1036</v>
       </c>
       <c r="F262" t="inlineStr"/>
       <c r="G262" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:18.000Z</t>
+          <t>2026-07-10T04:50:52.000Z</t>
         </is>
       </c>
     </row>
@@ -8090,12 +8090,12 @@
         </is>
       </c>
       <c r="E263" t="n">
-        <v>553</v>
+        <v>823</v>
       </c>
       <c r="F263" t="inlineStr"/>
       <c r="G263" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:18.000Z</t>
+          <t>2026-07-10T04:50:53.000Z</t>
         </is>
       </c>
     </row>
@@ -8119,12 +8119,12 @@
         </is>
       </c>
       <c r="E264" t="n">
-        <v>919</v>
+        <v>994</v>
       </c>
       <c r="F264" t="inlineStr"/>
       <c r="G264" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:19.000Z</t>
+          <t>2026-07-10T04:50:54.000Z</t>
         </is>
       </c>
     </row>
@@ -8148,12 +8148,12 @@
         </is>
       </c>
       <c r="E265" t="n">
-        <v>842</v>
+        <v>174</v>
       </c>
       <c r="F265" t="inlineStr"/>
       <c r="G265" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:20.000Z</t>
+          <t>2026-07-10T04:50:55.000Z</t>
         </is>
       </c>
     </row>
@@ -8177,12 +8177,12 @@
         </is>
       </c>
       <c r="E266" t="n">
-        <v>134</v>
+        <v>607</v>
       </c>
       <c r="F266" t="inlineStr"/>
       <c r="G266" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:21.000Z</t>
+          <t>2026-07-10T04:50:56.000Z</t>
         </is>
       </c>
     </row>
@@ -8206,12 +8206,12 @@
         </is>
       </c>
       <c r="E267" t="n">
-        <v>441</v>
+        <v>1003</v>
       </c>
       <c r="F267" t="inlineStr"/>
       <c r="G267" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:22.000Z</t>
+          <t>2026-07-10T04:50:56.000Z</t>
         </is>
       </c>
     </row>
@@ -8235,12 +8235,12 @@
         </is>
       </c>
       <c r="E268" t="n">
-        <v>738</v>
+        <v>804</v>
       </c>
       <c r="F268" t="inlineStr"/>
       <c r="G268" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:22.000Z</t>
+          <t>2026-07-10T04:50:57.000Z</t>
         </is>
       </c>
     </row>
@@ -8264,12 +8264,12 @@
         </is>
       </c>
       <c r="E269" t="n">
-        <v>1164</v>
+        <v>1183</v>
       </c>
       <c r="F269" t="inlineStr"/>
       <c r="G269" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:23.000Z</t>
+          <t>2026-07-10T04:50:58.000Z</t>
         </is>
       </c>
     </row>
@@ -8293,12 +8293,12 @@
         </is>
       </c>
       <c r="E270" t="n">
-        <v>932</v>
+        <v>1093</v>
       </c>
       <c r="F270" t="inlineStr"/>
       <c r="G270" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:24.000Z</t>
+          <t>2026-07-10T04:50:59.000Z</t>
         </is>
       </c>
     </row>
@@ -8322,12 +8322,12 @@
         </is>
       </c>
       <c r="E271" t="n">
-        <v>721</v>
+        <v>937</v>
       </c>
       <c r="F271" t="inlineStr"/>
       <c r="G271" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:25.000Z</t>
+          <t>2026-07-10T04:51:00.000Z</t>
         </is>
       </c>
     </row>
@@ -8351,12 +8351,12 @@
         </is>
       </c>
       <c r="E272" t="n">
-        <v>785</v>
+        <v>556</v>
       </c>
       <c r="F272" t="inlineStr"/>
       <c r="G272" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:26.000Z</t>
+          <t>2026-07-10T04:51:00.000Z</t>
         </is>
       </c>
     </row>
@@ -8380,12 +8380,12 @@
         </is>
       </c>
       <c r="E273" t="n">
-        <v>464</v>
+        <v>947</v>
       </c>
       <c r="F273" t="inlineStr"/>
       <c r="G273" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:26.000Z</t>
+          <t>2026-07-10T04:51:01.000Z</t>
         </is>
       </c>
     </row>
@@ -8409,12 +8409,12 @@
         </is>
       </c>
       <c r="E274" t="n">
-        <v>464</v>
+        <v>446</v>
       </c>
       <c r="F274" t="inlineStr"/>
       <c r="G274" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:27.000Z</t>
+          <t>2026-07-10T04:51:02.000Z</t>
         </is>
       </c>
     </row>
@@ -8438,12 +8438,12 @@
         </is>
       </c>
       <c r="E275" t="n">
-        <v>614</v>
+        <v>361</v>
       </c>
       <c r="F275" t="inlineStr"/>
       <c r="G275" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:28.000Z</t>
+          <t>2026-07-10T04:51:03.000Z</t>
         </is>
       </c>
     </row>
@@ -8467,12 +8467,12 @@
         </is>
       </c>
       <c r="E276" t="n">
-        <v>295</v>
+        <v>343</v>
       </c>
       <c r="F276" t="inlineStr"/>
       <c r="G276" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:29.000Z</t>
+          <t>2026-07-10T04:51:04.000Z</t>
         </is>
       </c>
     </row>
@@ -8496,12 +8496,12 @@
         </is>
       </c>
       <c r="E277" t="n">
-        <v>193</v>
+        <v>93</v>
       </c>
       <c r="F277" t="inlineStr"/>
       <c r="G277" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:30.000Z</t>
+          <t>2026-07-10T04:51:04.000Z</t>
         </is>
       </c>
     </row>
@@ -8525,12 +8525,12 @@
         </is>
       </c>
       <c r="E278" t="n">
-        <v>447</v>
+        <v>334</v>
       </c>
       <c r="F278" t="inlineStr"/>
       <c r="G278" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:30.000Z</t>
+          <t>2026-07-10T04:51:05.000Z</t>
         </is>
       </c>
     </row>
@@ -8554,12 +8554,12 @@
         </is>
       </c>
       <c r="E279" t="n">
-        <v>388</v>
+        <v>856</v>
       </c>
       <c r="F279" t="inlineStr"/>
       <c r="G279" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:31.000Z</t>
+          <t>2026-07-10T04:51:06.000Z</t>
         </is>
       </c>
     </row>
@@ -8583,12 +8583,12 @@
         </is>
       </c>
       <c r="E280" t="n">
-        <v>813</v>
+        <v>774</v>
       </c>
       <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:32.000Z</t>
+          <t>2026-07-10T04:51:07.000Z</t>
         </is>
       </c>
     </row>
@@ -8612,12 +8612,12 @@
         </is>
       </c>
       <c r="E281" t="n">
-        <v>536</v>
+        <v>476</v>
       </c>
       <c r="F281" t="inlineStr"/>
       <c r="G281" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:33.000Z</t>
+          <t>2026-07-10T04:51:08.000Z</t>
         </is>
       </c>
     </row>
@@ -8641,12 +8641,12 @@
         </is>
       </c>
       <c r="E282" t="n">
-        <v>923</v>
+        <v>252</v>
       </c>
       <c r="F282" t="inlineStr"/>
       <c r="G282" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:34.000Z</t>
+          <t>2026-07-10T04:51:08.000Z</t>
         </is>
       </c>
     </row>
@@ -8670,12 +8670,12 @@
         </is>
       </c>
       <c r="E283" t="n">
-        <v>790</v>
+        <v>215</v>
       </c>
       <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:34.000Z</t>
+          <t>2026-07-10T04:51:09.000Z</t>
         </is>
       </c>
     </row>
@@ -8699,12 +8699,12 @@
         </is>
       </c>
       <c r="E284" t="n">
-        <v>723</v>
+        <v>803</v>
       </c>
       <c r="F284" t="inlineStr"/>
       <c r="G284" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:35.000Z</t>
+          <t>2026-07-10T04:51:10.000Z</t>
         </is>
       </c>
     </row>
@@ -8728,12 +8728,12 @@
         </is>
       </c>
       <c r="E285" t="n">
-        <v>582</v>
+        <v>862</v>
       </c>
       <c r="F285" t="inlineStr"/>
       <c r="G285" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:36.000Z</t>
+          <t>2026-07-10T04:51:11.000Z</t>
         </is>
       </c>
     </row>
@@ -8757,12 +8757,12 @@
         </is>
       </c>
       <c r="E286" t="n">
-        <v>886</v>
+        <v>444</v>
       </c>
       <c r="F286" t="inlineStr"/>
       <c r="G286" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:37.000Z</t>
+          <t>2026-07-10T04:51:12.000Z</t>
         </is>
       </c>
     </row>
@@ -8786,12 +8786,12 @@
         </is>
       </c>
       <c r="E287" t="n">
-        <v>665</v>
+        <v>322</v>
       </c>
       <c r="F287" t="inlineStr"/>
       <c r="G287" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:38.000Z</t>
+          <t>2026-07-10T04:51:12.000Z</t>
         </is>
       </c>
     </row>
@@ -8815,12 +8815,12 @@
         </is>
       </c>
       <c r="E288" t="n">
-        <v>679</v>
+        <v>381</v>
       </c>
       <c r="F288" t="inlineStr"/>
       <c r="G288" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:38.000Z</t>
+          <t>2026-07-10T04:51:13.000Z</t>
         </is>
       </c>
     </row>
@@ -8844,12 +8844,12 @@
         </is>
       </c>
       <c r="E289" t="n">
-        <v>207</v>
+        <v>457</v>
       </c>
       <c r="F289" t="inlineStr"/>
       <c r="G289" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:39.000Z</t>
+          <t>2026-07-10T04:51:14.000Z</t>
         </is>
       </c>
     </row>
@@ -8873,12 +8873,12 @@
         </is>
       </c>
       <c r="E290" t="n">
-        <v>601</v>
+        <v>83</v>
       </c>
       <c r="F290" t="inlineStr"/>
       <c r="G290" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:40.000Z</t>
+          <t>2026-07-10T04:51:15.000Z</t>
         </is>
       </c>
     </row>
@@ -8902,12 +8902,12 @@
         </is>
       </c>
       <c r="E291" t="n">
-        <v>919</v>
+        <v>362</v>
       </c>
       <c r="F291" t="inlineStr"/>
       <c r="G291" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:41.000Z</t>
+          <t>2026-07-10T04:51:16.000Z</t>
         </is>
       </c>
     </row>
@@ -8931,12 +8931,12 @@
         </is>
       </c>
       <c r="E292" t="n">
-        <v>440</v>
+        <v>490</v>
       </c>
       <c r="F292" t="inlineStr"/>
       <c r="G292" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:42.000Z</t>
+          <t>2026-07-10T04:51:16.000Z</t>
         </is>
       </c>
     </row>
@@ -8960,12 +8960,12 @@
         </is>
       </c>
       <c r="E293" t="n">
-        <v>212</v>
+        <v>283</v>
       </c>
       <c r="F293" t="inlineStr"/>
       <c r="G293" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:42.000Z</t>
+          <t>2026-07-10T04:51:17.000Z</t>
         </is>
       </c>
     </row>
@@ -8989,12 +8989,12 @@
         </is>
       </c>
       <c r="E294" t="n">
-        <v>360</v>
+        <v>1009</v>
       </c>
       <c r="F294" t="inlineStr"/>
       <c r="G294" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:43.000Z</t>
+          <t>2026-07-10T04:51:18.000Z</t>
         </is>
       </c>
     </row>
@@ -9018,12 +9018,12 @@
         </is>
       </c>
       <c r="E295" t="n">
-        <v>450</v>
+        <v>834</v>
       </c>
       <c r="F295" t="inlineStr"/>
       <c r="G295" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:44.000Z</t>
+          <t>2026-07-10T04:51:19.000Z</t>
         </is>
       </c>
     </row>
@@ -9047,12 +9047,12 @@
         </is>
       </c>
       <c r="E296" t="n">
-        <v>398</v>
+        <v>661</v>
       </c>
       <c r="F296" t="inlineStr"/>
       <c r="G296" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:45.000Z</t>
+          <t>2026-07-10T04:51:20.000Z</t>
         </is>
       </c>
     </row>
@@ -9076,12 +9076,12 @@
         </is>
       </c>
       <c r="E297" t="n">
-        <v>808</v>
+        <v>251</v>
       </c>
       <c r="F297" t="inlineStr"/>
       <c r="G297" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:46.000Z</t>
+          <t>2026-07-10T04:51:20.000Z</t>
         </is>
       </c>
     </row>
@@ -9105,12 +9105,12 @@
         </is>
       </c>
       <c r="E298" t="n">
-        <v>1097</v>
+        <v>329</v>
       </c>
       <c r="F298" t="inlineStr"/>
       <c r="G298" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:46.000Z</t>
+          <t>2026-07-10T04:51:21.000Z</t>
         </is>
       </c>
     </row>
@@ -9134,12 +9134,12 @@
         </is>
       </c>
       <c r="E299" t="n">
-        <v>290</v>
+        <v>928</v>
       </c>
       <c r="F299" t="inlineStr"/>
       <c r="G299" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:47.000Z</t>
+          <t>2026-07-10T04:51:22.000Z</t>
         </is>
       </c>
     </row>
@@ -9163,12 +9163,12 @@
         </is>
       </c>
       <c r="E300" t="n">
-        <v>963</v>
+        <v>569</v>
       </c>
       <c r="F300" t="inlineStr"/>
       <c r="G300" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:48.000Z</t>
+          <t>2026-07-10T04:51:23.000Z</t>
         </is>
       </c>
     </row>
@@ -9192,12 +9192,12 @@
         </is>
       </c>
       <c r="E301" t="n">
-        <v>1099</v>
+        <v>531</v>
       </c>
       <c r="F301" t="inlineStr"/>
       <c r="G301" t="inlineStr">
         <is>
-          <t>2026-07-10T04:35:49.000Z</t>
+          <t>2026-07-10T04:51:24.000Z</t>
         </is>
       </c>
     </row>
@@ -9325,7 +9325,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-10T04:31:49.000Z</t>
+          <t>2026-07-10T04:47:24.000Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploy Test Reports — 1200 Tests All PASSED 5ed32c55a64b2de032133a5d6a87de7dcb8bbc8a
</commit_message>
<xml_diff>
--- a/reports/latest/Appium_Report.xlsx
+++ b/reports/latest/Appium_Report.xlsx
@@ -521,12 +521,12 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1095</v>
+        <v>473</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:24.000Z</t>
+          <t>2026-07-10T04:53:49.000Z</t>
         </is>
       </c>
     </row>
@@ -550,12 +550,12 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>499</v>
+        <v>799</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:25.000Z</t>
+          <t>2026-07-10T04:53:50.000Z</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>725</v>
+        <v>775</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:26.000Z</t>
+          <t>2026-07-10T04:53:50.000Z</t>
         </is>
       </c>
     </row>
@@ -608,12 +608,12 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>773</v>
+        <v>189</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:27.000Z</t>
+          <t>2026-07-10T04:53:51.000Z</t>
         </is>
       </c>
     </row>
@@ -637,12 +637,12 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>615</v>
+        <v>415</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:28.000Z</t>
+          <t>2026-07-10T04:53:52.000Z</t>
         </is>
       </c>
     </row>
@@ -666,12 +666,12 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1171</v>
+        <v>486</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:28.000Z</t>
+          <t>2026-07-10T04:53:53.000Z</t>
         </is>
       </c>
     </row>
@@ -695,12 +695,12 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>328</v>
+        <v>1079</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:29.000Z</t>
+          <t>2026-07-10T04:53:54.000Z</t>
         </is>
       </c>
     </row>
@@ -724,12 +724,12 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>151</v>
+        <v>724</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:30.000Z</t>
+          <t>2026-07-10T04:53:54.000Z</t>
         </is>
       </c>
     </row>
@@ -753,12 +753,12 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>747</v>
+        <v>339</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:31.000Z</t>
+          <t>2026-07-10T04:53:55.000Z</t>
         </is>
       </c>
     </row>
@@ -782,12 +782,12 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>241</v>
+        <v>140</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:32.000Z</t>
+          <t>2026-07-10T04:53:56.000Z</t>
         </is>
       </c>
     </row>
@@ -811,12 +811,12 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>664</v>
+        <v>1065</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:32.000Z</t>
+          <t>2026-07-10T04:53:57.000Z</t>
         </is>
       </c>
     </row>
@@ -840,12 +840,12 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1029</v>
+        <v>185</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:33.000Z</t>
+          <t>2026-07-10T04:53:58.000Z</t>
         </is>
       </c>
     </row>
@@ -869,12 +869,12 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>705</v>
+        <v>378</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:34.000Z</t>
+          <t>2026-07-10T04:53:58.000Z</t>
         </is>
       </c>
     </row>
@@ -898,12 +898,12 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>411</v>
+        <v>912</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:35.000Z</t>
+          <t>2026-07-10T04:53:59.000Z</t>
         </is>
       </c>
     </row>
@@ -927,12 +927,12 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>682</v>
+        <v>651</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:36.000Z</t>
+          <t>2026-07-10T04:54:00.000Z</t>
         </is>
       </c>
     </row>
@@ -956,12 +956,12 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>776</v>
+        <v>91</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:36.000Z</t>
+          <t>2026-07-10T04:54:01.000Z</t>
         </is>
       </c>
     </row>
@@ -985,12 +985,12 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1066</v>
+        <v>874</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:37.000Z</t>
+          <t>2026-07-10T04:54:02.000Z</t>
         </is>
       </c>
     </row>
@@ -1014,12 +1014,12 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>931</v>
+        <v>700</v>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:38.000Z</t>
+          <t>2026-07-10T04:54:02.000Z</t>
         </is>
       </c>
     </row>
@@ -1043,12 +1043,12 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>330</v>
+        <v>234</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:39.000Z</t>
+          <t>2026-07-10T04:54:03.000Z</t>
         </is>
       </c>
     </row>
@@ -1072,12 +1072,12 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>367</v>
+        <v>855</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:40.000Z</t>
+          <t>2026-07-10T04:54:04.000Z</t>
         </is>
       </c>
     </row>
@@ -1101,12 +1101,12 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>555</v>
+        <v>410</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:40.000Z</t>
+          <t>2026-07-10T04:54:05.000Z</t>
         </is>
       </c>
     </row>
@@ -1130,12 +1130,12 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>397</v>
+        <v>801</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:41.000Z</t>
+          <t>2026-07-10T04:54:06.000Z</t>
         </is>
       </c>
     </row>
@@ -1159,12 +1159,12 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1096</v>
+        <v>882</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:42.000Z</t>
+          <t>2026-07-10T04:54:06.000Z</t>
         </is>
       </c>
     </row>
@@ -1188,12 +1188,12 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>945</v>
+        <v>394</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:43.000Z</t>
+          <t>2026-07-10T04:54:07.000Z</t>
         </is>
       </c>
     </row>
@@ -1217,12 +1217,12 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>1070</v>
+        <v>299</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:44.000Z</t>
+          <t>2026-07-10T04:54:08.000Z</t>
         </is>
       </c>
     </row>
@@ -1246,12 +1246,12 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>340</v>
+        <v>758</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:44.000Z</t>
+          <t>2026-07-10T04:54:09.000Z</t>
         </is>
       </c>
     </row>
@@ -1275,12 +1275,12 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>193</v>
+        <v>283</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:45.000Z</t>
+          <t>2026-07-10T04:54:10.000Z</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>1056</v>
+        <v>951</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:46.000Z</t>
+          <t>2026-07-10T04:54:10.000Z</t>
         </is>
       </c>
     </row>
@@ -1333,12 +1333,12 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1103</v>
+        <v>848</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:47.000Z</t>
+          <t>2026-07-10T04:54:11.000Z</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>711</v>
+        <v>96</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:48.000Z</t>
+          <t>2026-07-10T04:54:12.000Z</t>
         </is>
       </c>
     </row>
@@ -1391,12 +1391,12 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:48.000Z</t>
+          <t>2026-07-10T04:54:13.000Z</t>
         </is>
       </c>
     </row>
@@ -1420,12 +1420,12 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>158</v>
+        <v>1135</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:49.000Z</t>
+          <t>2026-07-10T04:54:14.000Z</t>
         </is>
       </c>
     </row>
@@ -1449,12 +1449,12 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>568</v>
+        <v>529</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:50.000Z</t>
+          <t>2026-07-10T04:54:14.000Z</t>
         </is>
       </c>
     </row>
@@ -1478,12 +1478,12 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>1039</v>
+        <v>956</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:51.000Z</t>
+          <t>2026-07-10T04:54:15.000Z</t>
         </is>
       </c>
     </row>
@@ -1507,12 +1507,12 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>1152</v>
+        <v>233</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:52.000Z</t>
+          <t>2026-07-10T04:54:16.000Z</t>
         </is>
       </c>
     </row>
@@ -1536,12 +1536,12 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>711</v>
+        <v>480</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:52.000Z</t>
+          <t>2026-07-10T04:54:17.000Z</t>
         </is>
       </c>
     </row>
@@ -1565,12 +1565,12 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>410</v>
+        <v>773</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:53.000Z</t>
+          <t>2026-07-10T04:54:18.000Z</t>
         </is>
       </c>
     </row>
@@ -1594,12 +1594,12 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>944</v>
+        <v>1037</v>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:54.000Z</t>
+          <t>2026-07-10T04:54:18.000Z</t>
         </is>
       </c>
     </row>
@@ -1623,12 +1623,12 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>1146</v>
+        <v>520</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:55.000Z</t>
+          <t>2026-07-10T04:54:19.000Z</t>
         </is>
       </c>
     </row>
@@ -1652,12 +1652,12 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>876</v>
+        <v>203</v>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:56.000Z</t>
+          <t>2026-07-10T04:54:20.000Z</t>
         </is>
       </c>
     </row>
@@ -1681,12 +1681,12 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1178</v>
+        <v>955</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:56.000Z</t>
+          <t>2026-07-10T04:54:21.000Z</t>
         </is>
       </c>
     </row>
@@ -1710,12 +1710,12 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>114</v>
+        <v>1037</v>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:57.000Z</t>
+          <t>2026-07-10T04:54:22.000Z</t>
         </is>
       </c>
     </row>
@@ -1739,12 +1739,12 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>388</v>
+        <v>735</v>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:58.000Z</t>
+          <t>2026-07-10T04:54:22.000Z</t>
         </is>
       </c>
     </row>
@@ -1768,12 +1768,12 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>497</v>
+        <v>1050</v>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:59.000Z</t>
+          <t>2026-07-10T04:54:23.000Z</t>
         </is>
       </c>
     </row>
@@ -1797,12 +1797,12 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>492</v>
+        <v>1041</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:00.000Z</t>
+          <t>2026-07-10T04:54:24.000Z</t>
         </is>
       </c>
     </row>
@@ -1826,12 +1826,12 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>934</v>
+        <v>297</v>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:00.000Z</t>
+          <t>2026-07-10T04:54:25.000Z</t>
         </is>
       </c>
     </row>
@@ -1855,12 +1855,12 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>718</v>
+        <v>660</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:01.000Z</t>
+          <t>2026-07-10T04:54:26.000Z</t>
         </is>
       </c>
     </row>
@@ -1884,12 +1884,12 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>571</v>
+        <v>946</v>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:02.000Z</t>
+          <t>2026-07-10T04:54:26.000Z</t>
         </is>
       </c>
     </row>
@@ -1913,12 +1913,12 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>991</v>
+        <v>943</v>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:03.000Z</t>
+          <t>2026-07-10T04:54:27.000Z</t>
         </is>
       </c>
     </row>
@@ -1942,12 +1942,12 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>781</v>
+        <v>1080</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:04.000Z</t>
+          <t>2026-07-10T04:54:28.000Z</t>
         </is>
       </c>
     </row>
@@ -1971,12 +1971,12 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:04.000Z</t>
+          <t>2026-07-10T04:54:29.000Z</t>
         </is>
       </c>
     </row>
@@ -2000,12 +2000,12 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>725</v>
+        <v>1075</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:05.000Z</t>
+          <t>2026-07-10T04:54:30.000Z</t>
         </is>
       </c>
     </row>
@@ -2029,12 +2029,12 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>489</v>
+        <v>872</v>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:06.000Z</t>
+          <t>2026-07-10T04:54:30.000Z</t>
         </is>
       </c>
     </row>
@@ -2058,12 +2058,12 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>588</v>
+        <v>726</v>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:07.000Z</t>
+          <t>2026-07-10T04:54:31.000Z</t>
         </is>
       </c>
     </row>
@@ -2087,12 +2087,12 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>303</v>
+        <v>580</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:08.000Z</t>
+          <t>2026-07-10T04:54:32.000Z</t>
         </is>
       </c>
     </row>
@@ -2116,12 +2116,12 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>1020</v>
+        <v>104</v>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:08.000Z</t>
+          <t>2026-07-10T04:54:33.000Z</t>
         </is>
       </c>
     </row>
@@ -2145,12 +2145,12 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>946</v>
+        <v>664</v>
       </c>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:09.000Z</t>
+          <t>2026-07-10T04:54:34.000Z</t>
         </is>
       </c>
     </row>
@@ -2174,12 +2174,12 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>480</v>
+        <v>857</v>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:10.000Z</t>
+          <t>2026-07-10T04:54:34.000Z</t>
         </is>
       </c>
     </row>
@@ -2203,12 +2203,12 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>889</v>
+        <v>1129</v>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:11.000Z</t>
+          <t>2026-07-10T04:54:35.000Z</t>
         </is>
       </c>
     </row>
@@ -2232,12 +2232,12 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>355</v>
+        <v>376</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:12.000Z</t>
+          <t>2026-07-10T04:54:36.000Z</t>
         </is>
       </c>
     </row>
@@ -2261,12 +2261,12 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>967</v>
+        <v>149</v>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:12.000Z</t>
+          <t>2026-07-10T04:54:37.000Z</t>
         </is>
       </c>
     </row>
@@ -2290,12 +2290,12 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>759</v>
+        <v>1086</v>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:13.000Z</t>
+          <t>2026-07-10T04:54:38.000Z</t>
         </is>
       </c>
     </row>
@@ -2319,12 +2319,12 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>997</v>
+        <v>1074</v>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:14.000Z</t>
+          <t>2026-07-10T04:54:38.000Z</t>
         </is>
       </c>
     </row>
@@ -2348,12 +2348,12 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>313</v>
+        <v>1136</v>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:15.000Z</t>
+          <t>2026-07-10T04:54:39.000Z</t>
         </is>
       </c>
     </row>
@@ -2377,12 +2377,12 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>832</v>
+        <v>891</v>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:16.000Z</t>
+          <t>2026-07-10T04:54:40.000Z</t>
         </is>
       </c>
     </row>
@@ -2406,12 +2406,12 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>896</v>
+        <v>608</v>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:16.000Z</t>
+          <t>2026-07-10T04:54:41.000Z</t>
         </is>
       </c>
     </row>
@@ -2435,12 +2435,12 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>808</v>
+        <v>741</v>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:17.000Z</t>
+          <t>2026-07-10T04:54:42.000Z</t>
         </is>
       </c>
     </row>
@@ -2464,12 +2464,12 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>353</v>
+        <v>83</v>
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:18.000Z</t>
+          <t>2026-07-10T04:54:42.000Z</t>
         </is>
       </c>
     </row>
@@ -2493,12 +2493,12 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>799</v>
+        <v>327</v>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:19.000Z</t>
+          <t>2026-07-10T04:54:43.000Z</t>
         </is>
       </c>
     </row>
@@ -2522,12 +2522,12 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>803</v>
+        <v>513</v>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:20.000Z</t>
+          <t>2026-07-10T04:54:44.000Z</t>
         </is>
       </c>
     </row>
@@ -2551,12 +2551,12 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>605</v>
+        <v>805</v>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:20.000Z</t>
+          <t>2026-07-10T04:54:45.000Z</t>
         </is>
       </c>
     </row>
@@ -2580,12 +2580,12 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>989</v>
+        <v>720</v>
       </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:21.000Z</t>
+          <t>2026-07-10T04:54:46.000Z</t>
         </is>
       </c>
     </row>
@@ -2609,12 +2609,12 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>512</v>
+        <v>446</v>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:22.000Z</t>
+          <t>2026-07-10T04:54:46.000Z</t>
         </is>
       </c>
     </row>
@@ -2638,12 +2638,12 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>986</v>
+        <v>693</v>
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:23.000Z</t>
+          <t>2026-07-10T04:54:47.000Z</t>
         </is>
       </c>
     </row>
@@ -2667,12 +2667,12 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>585</v>
+        <v>89</v>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:24.000Z</t>
+          <t>2026-07-10T04:54:48.000Z</t>
         </is>
       </c>
     </row>
@@ -2696,12 +2696,12 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>168</v>
+        <v>733</v>
       </c>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:24.000Z</t>
+          <t>2026-07-10T04:54:49.000Z</t>
         </is>
       </c>
     </row>
@@ -2725,12 +2725,12 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>106</v>
+        <v>1096</v>
       </c>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:25.000Z</t>
+          <t>2026-07-10T04:54:50.000Z</t>
         </is>
       </c>
     </row>
@@ -2754,12 +2754,12 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>317</v>
+        <v>129</v>
       </c>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:26.000Z</t>
+          <t>2026-07-10T04:54:50.000Z</t>
         </is>
       </c>
     </row>
@@ -2783,12 +2783,12 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>847</v>
+        <v>404</v>
       </c>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:27.000Z</t>
+          <t>2026-07-10T04:54:51.000Z</t>
         </is>
       </c>
     </row>
@@ -2812,12 +2812,12 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>1012</v>
+        <v>153</v>
       </c>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:28.000Z</t>
+          <t>2026-07-10T04:54:52.000Z</t>
         </is>
       </c>
     </row>
@@ -2841,12 +2841,12 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>1162</v>
+        <v>1088</v>
       </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:28.000Z</t>
+          <t>2026-07-10T04:54:53.000Z</t>
         </is>
       </c>
     </row>
@@ -2870,12 +2870,12 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>559</v>
+        <v>260</v>
       </c>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:29.000Z</t>
+          <t>2026-07-10T04:54:54.000Z</t>
         </is>
       </c>
     </row>
@@ -2899,12 +2899,12 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>839</v>
+        <v>1122</v>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:30.000Z</t>
+          <t>2026-07-10T04:54:54.000Z</t>
         </is>
       </c>
     </row>
@@ -2928,12 +2928,12 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>405</v>
+        <v>611</v>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:31.000Z</t>
+          <t>2026-07-10T04:54:55.000Z</t>
         </is>
       </c>
     </row>
@@ -2957,12 +2957,12 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>84</v>
+        <v>368</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:32.000Z</t>
+          <t>2026-07-10T04:54:56.000Z</t>
         </is>
       </c>
     </row>
@@ -2986,12 +2986,12 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>754</v>
+        <v>874</v>
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:32.000Z</t>
+          <t>2026-07-10T04:54:57.000Z</t>
         </is>
       </c>
     </row>
@@ -3015,12 +3015,12 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>906</v>
+        <v>972</v>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:33.000Z</t>
+          <t>2026-07-10T04:54:58.000Z</t>
         </is>
       </c>
     </row>
@@ -3044,12 +3044,12 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>498</v>
+        <v>904</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:34.000Z</t>
+          <t>2026-07-10T04:54:58.000Z</t>
         </is>
       </c>
     </row>
@@ -3073,12 +3073,12 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>295</v>
+        <v>1169</v>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:35.000Z</t>
+          <t>2026-07-10T04:54:59.000Z</t>
         </is>
       </c>
     </row>
@@ -3102,12 +3102,12 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>1151</v>
+        <v>1128</v>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:36.000Z</t>
+          <t>2026-07-10T04:55:00.000Z</t>
         </is>
       </c>
     </row>
@@ -3131,12 +3131,12 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>513</v>
+        <v>805</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:36.000Z</t>
+          <t>2026-07-10T04:55:01.000Z</t>
         </is>
       </c>
     </row>
@@ -3160,12 +3160,12 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>664</v>
+        <v>749</v>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:37.000Z</t>
+          <t>2026-07-10T04:55:02.000Z</t>
         </is>
       </c>
     </row>
@@ -3189,12 +3189,12 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>714</v>
+        <v>483</v>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:38.000Z</t>
+          <t>2026-07-10T04:55:02.000Z</t>
         </is>
       </c>
     </row>
@@ -3218,12 +3218,12 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>814</v>
+        <v>152</v>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:39.000Z</t>
+          <t>2026-07-10T04:55:03.000Z</t>
         </is>
       </c>
     </row>
@@ -3247,12 +3247,12 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>747</v>
+        <v>143</v>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:40.000Z</t>
+          <t>2026-07-10T04:55:04.000Z</t>
         </is>
       </c>
     </row>
@@ -3276,12 +3276,12 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>896</v>
+        <v>879</v>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:40.000Z</t>
+          <t>2026-07-10T04:55:05.000Z</t>
         </is>
       </c>
     </row>
@@ -3305,12 +3305,12 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>652</v>
+        <v>176</v>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:41.000Z</t>
+          <t>2026-07-10T04:55:06.000Z</t>
         </is>
       </c>
     </row>
@@ -3334,12 +3334,12 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>512</v>
+        <v>628</v>
       </c>
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:42.000Z</t>
+          <t>2026-07-10T04:55:06.000Z</t>
         </is>
       </c>
     </row>
@@ -3363,12 +3363,12 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>656</v>
+        <v>300</v>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:43.000Z</t>
+          <t>2026-07-10T04:55:07.000Z</t>
         </is>
       </c>
     </row>
@@ -3392,12 +3392,12 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:44.000Z</t>
+          <t>2026-07-10T04:55:08.000Z</t>
         </is>
       </c>
     </row>
@@ -3421,12 +3421,12 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>705</v>
+        <v>1039</v>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:44.000Z</t>
+          <t>2026-07-10T04:55:09.000Z</t>
         </is>
       </c>
     </row>
@@ -3450,12 +3450,12 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>207</v>
+        <v>504</v>
       </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:45.000Z</t>
+          <t>2026-07-10T04:55:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3479,12 +3479,12 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>152</v>
+        <v>741</v>
       </c>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:46.000Z</t>
+          <t>2026-07-10T04:55:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3508,12 +3508,12 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>166</v>
+        <v>1006</v>
       </c>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:47.000Z</t>
+          <t>2026-07-10T04:55:11.000Z</t>
         </is>
       </c>
     </row>
@@ -3537,12 +3537,12 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>909</v>
+        <v>638</v>
       </c>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:48.000Z</t>
+          <t>2026-07-10T04:55:12.000Z</t>
         </is>
       </c>
     </row>
@@ -3566,12 +3566,12 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>792</v>
+        <v>143</v>
       </c>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:48.000Z</t>
+          <t>2026-07-10T04:55:13.000Z</t>
         </is>
       </c>
     </row>
@@ -3595,12 +3595,12 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>664</v>
+        <v>424</v>
       </c>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:49.000Z</t>
+          <t>2026-07-10T04:55:14.000Z</t>
         </is>
       </c>
     </row>
@@ -3624,12 +3624,12 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>262</v>
+        <v>610</v>
       </c>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:50.000Z</t>
+          <t>2026-07-10T04:55:14.000Z</t>
         </is>
       </c>
     </row>
@@ -3653,12 +3653,12 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>154</v>
+        <v>455</v>
       </c>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:51.000Z</t>
+          <t>2026-07-10T04:55:15.000Z</t>
         </is>
       </c>
     </row>
@@ -3682,12 +3682,12 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>549</v>
+        <v>416</v>
       </c>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:52.000Z</t>
+          <t>2026-07-10T04:55:16.000Z</t>
         </is>
       </c>
     </row>
@@ -3711,12 +3711,12 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>629</v>
+        <v>445</v>
       </c>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:52.000Z</t>
+          <t>2026-07-10T04:55:17.000Z</t>
         </is>
       </c>
     </row>
@@ -3740,12 +3740,12 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>229</v>
+        <v>410</v>
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:53.000Z</t>
+          <t>2026-07-10T04:55:18.000Z</t>
         </is>
       </c>
     </row>
@@ -3769,12 +3769,12 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>266</v>
+        <v>1150</v>
       </c>
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:54.000Z</t>
+          <t>2026-07-10T04:55:18.000Z</t>
         </is>
       </c>
     </row>
@@ -3798,12 +3798,12 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>426</v>
+        <v>699</v>
       </c>
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:55.000Z</t>
+          <t>2026-07-10T04:55:19.000Z</t>
         </is>
       </c>
     </row>
@@ -3827,12 +3827,12 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>87</v>
+        <v>511</v>
       </c>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:56.000Z</t>
+          <t>2026-07-10T04:55:20.000Z</t>
         </is>
       </c>
     </row>
@@ -3856,12 +3856,12 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>1003</v>
+        <v>1029</v>
       </c>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:56.000Z</t>
+          <t>2026-07-10T04:55:21.000Z</t>
         </is>
       </c>
     </row>
@@ -3885,12 +3885,12 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>264</v>
+        <v>389</v>
       </c>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:57.000Z</t>
+          <t>2026-07-10T04:55:22.000Z</t>
         </is>
       </c>
     </row>
@@ -3914,12 +3914,12 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>1161</v>
+        <v>289</v>
       </c>
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:58.000Z</t>
+          <t>2026-07-10T04:55:22.000Z</t>
         </is>
       </c>
     </row>
@@ -3943,12 +3943,12 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>325</v>
+        <v>727</v>
       </c>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2026-07-10T04:48:59.000Z</t>
+          <t>2026-07-10T04:55:23.000Z</t>
         </is>
       </c>
     </row>
@@ -3972,12 +3972,12 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>534</v>
+        <v>204</v>
       </c>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:00.000Z</t>
+          <t>2026-07-10T04:55:24.000Z</t>
         </is>
       </c>
     </row>
@@ -4001,12 +4001,12 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>1034</v>
+        <v>1054</v>
       </c>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:00.000Z</t>
+          <t>2026-07-10T04:55:25.000Z</t>
         </is>
       </c>
     </row>
@@ -4030,12 +4030,12 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>999</v>
+        <v>410</v>
       </c>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:01.000Z</t>
+          <t>2026-07-10T04:55:26.000Z</t>
         </is>
       </c>
     </row>
@@ -4059,12 +4059,12 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>1147</v>
+        <v>1144</v>
       </c>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:02.000Z</t>
+          <t>2026-07-10T04:55:26.000Z</t>
         </is>
       </c>
     </row>
@@ -4088,12 +4088,12 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>1127</v>
+        <v>997</v>
       </c>
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:03.000Z</t>
+          <t>2026-07-10T04:55:27.000Z</t>
         </is>
       </c>
     </row>
@@ -4117,12 +4117,12 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>780</v>
+        <v>414</v>
       </c>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:04.000Z</t>
+          <t>2026-07-10T04:55:28.000Z</t>
         </is>
       </c>
     </row>
@@ -4146,12 +4146,12 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>1011</v>
+        <v>191</v>
       </c>
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:04.000Z</t>
+          <t>2026-07-10T04:55:29.000Z</t>
         </is>
       </c>
     </row>
@@ -4175,12 +4175,12 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>1027</v>
+        <v>307</v>
       </c>
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:05.000Z</t>
+          <t>2026-07-10T04:55:30.000Z</t>
         </is>
       </c>
     </row>
@@ -4204,12 +4204,12 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>805</v>
+        <v>323</v>
       </c>
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:06.000Z</t>
+          <t>2026-07-10T04:55:30.000Z</t>
         </is>
       </c>
     </row>
@@ -4233,12 +4233,12 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>801</v>
+        <v>257</v>
       </c>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:07.000Z</t>
+          <t>2026-07-10T04:55:31.000Z</t>
         </is>
       </c>
     </row>
@@ -4262,12 +4262,12 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>1148</v>
+        <v>477</v>
       </c>
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:08.000Z</t>
+          <t>2026-07-10T04:55:32.000Z</t>
         </is>
       </c>
     </row>
@@ -4291,12 +4291,12 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>701</v>
+        <v>672</v>
       </c>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:08.000Z</t>
+          <t>2026-07-10T04:55:33.000Z</t>
         </is>
       </c>
     </row>
@@ -4320,12 +4320,12 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>784</v>
+        <v>899</v>
       </c>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:09.000Z</t>
+          <t>2026-07-10T04:55:34.000Z</t>
         </is>
       </c>
     </row>
@@ -4349,12 +4349,12 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>664</v>
+        <v>151</v>
       </c>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:10.000Z</t>
+          <t>2026-07-10T04:55:34.000Z</t>
         </is>
       </c>
     </row>
@@ -4378,12 +4378,12 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>932</v>
+        <v>1033</v>
       </c>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:11.000Z</t>
+          <t>2026-07-10T04:55:35.000Z</t>
         </is>
       </c>
     </row>
@@ -4407,12 +4407,12 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>1188</v>
+        <v>390</v>
       </c>
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:12.000Z</t>
+          <t>2026-07-10T04:55:36.000Z</t>
         </is>
       </c>
     </row>
@@ -4436,12 +4436,12 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>694</v>
+        <v>423</v>
       </c>
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:12.000Z</t>
+          <t>2026-07-10T04:55:37.000Z</t>
         </is>
       </c>
     </row>
@@ -4465,12 +4465,12 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>469</v>
+        <v>803</v>
       </c>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:13.000Z</t>
+          <t>2026-07-10T04:55:38.000Z</t>
         </is>
       </c>
     </row>
@@ -4494,12 +4494,12 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>806</v>
+        <v>940</v>
       </c>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:14.000Z</t>
+          <t>2026-07-10T04:55:38.000Z</t>
         </is>
       </c>
     </row>
@@ -4523,12 +4523,12 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>338</v>
+        <v>523</v>
       </c>
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:15.000Z</t>
+          <t>2026-07-10T04:55:39.000Z</t>
         </is>
       </c>
     </row>
@@ -4552,12 +4552,12 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>424</v>
+        <v>1060</v>
       </c>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:16.000Z</t>
+          <t>2026-07-10T04:55:40.000Z</t>
         </is>
       </c>
     </row>
@@ -4581,12 +4581,12 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>810</v>
+        <v>664</v>
       </c>
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:16.000Z</t>
+          <t>2026-07-10T04:55:41.000Z</t>
         </is>
       </c>
     </row>
@@ -4610,12 +4610,12 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>144</v>
+        <v>506</v>
       </c>
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:17.000Z</t>
+          <t>2026-07-10T04:55:42.000Z</t>
         </is>
       </c>
     </row>
@@ -4639,12 +4639,12 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>962</v>
+        <v>634</v>
       </c>
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:18.000Z</t>
+          <t>2026-07-10T04:55:42.000Z</t>
         </is>
       </c>
     </row>
@@ -4668,12 +4668,12 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>332</v>
+        <v>702</v>
       </c>
       <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:19.000Z</t>
+          <t>2026-07-10T04:55:43.000Z</t>
         </is>
       </c>
     </row>
@@ -4697,12 +4697,12 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>883</v>
+        <v>1082</v>
       </c>
       <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:20.000Z</t>
+          <t>2026-07-10T04:55:44.000Z</t>
         </is>
       </c>
     </row>
@@ -4726,12 +4726,12 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>697</v>
+        <v>1174</v>
       </c>
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:20.000Z</t>
+          <t>2026-07-10T04:55:45.000Z</t>
         </is>
       </c>
     </row>
@@ -4755,12 +4755,12 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>895</v>
+        <v>576</v>
       </c>
       <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:21.000Z</t>
+          <t>2026-07-10T04:55:46.000Z</t>
         </is>
       </c>
     </row>
@@ -4784,12 +4784,12 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>1186</v>
+        <v>284</v>
       </c>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:22.000Z</t>
+          <t>2026-07-10T04:55:46.000Z</t>
         </is>
       </c>
     </row>
@@ -4813,12 +4813,12 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>266</v>
+        <v>764</v>
       </c>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:23.000Z</t>
+          <t>2026-07-10T04:55:47.000Z</t>
         </is>
       </c>
     </row>
@@ -4842,12 +4842,12 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>1189</v>
+        <v>635</v>
       </c>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:24.000Z</t>
+          <t>2026-07-10T04:55:48.000Z</t>
         </is>
       </c>
     </row>
@@ -4871,12 +4871,12 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>294</v>
+        <v>1048</v>
       </c>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:24.000Z</t>
+          <t>2026-07-10T04:55:49.000Z</t>
         </is>
       </c>
     </row>
@@ -4900,12 +4900,12 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>269</v>
+        <v>562</v>
       </c>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:25.000Z</t>
+          <t>2026-07-10T04:55:50.000Z</t>
         </is>
       </c>
     </row>
@@ -4929,12 +4929,12 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>956</v>
+        <v>332</v>
       </c>
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:26.000Z</t>
+          <t>2026-07-10T04:55:50.000Z</t>
         </is>
       </c>
     </row>
@@ -4958,12 +4958,12 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>867</v>
+        <v>1199</v>
       </c>
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:27.000Z</t>
+          <t>2026-07-10T04:55:51.000Z</t>
         </is>
       </c>
     </row>
@@ -4987,12 +4987,12 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>200</v>
+        <v>977</v>
       </c>
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:28.000Z</t>
+          <t>2026-07-10T04:55:52.000Z</t>
         </is>
       </c>
     </row>
@@ -5016,12 +5016,12 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>1116</v>
+        <v>659</v>
       </c>
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:28.000Z</t>
+          <t>2026-07-10T04:55:53.000Z</t>
         </is>
       </c>
     </row>
@@ -5045,12 +5045,12 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>488</v>
+        <v>431</v>
       </c>
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:29.000Z</t>
+          <t>2026-07-10T04:55:54.000Z</t>
         </is>
       </c>
     </row>
@@ -5074,12 +5074,12 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>283</v>
+        <v>471</v>
       </c>
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:30.000Z</t>
+          <t>2026-07-10T04:55:54.000Z</t>
         </is>
       </c>
     </row>
@@ -5103,12 +5103,12 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>313</v>
+        <v>570</v>
       </c>
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:31.000Z</t>
+          <t>2026-07-10T04:55:55.000Z</t>
         </is>
       </c>
     </row>
@@ -5132,12 +5132,12 @@
         </is>
       </c>
       <c r="E161" t="n">
-        <v>82</v>
+        <v>857</v>
       </c>
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:32.000Z</t>
+          <t>2026-07-10T04:55:56.000Z</t>
         </is>
       </c>
     </row>
@@ -5161,12 +5161,12 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>207</v>
+        <v>224</v>
       </c>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:32.000Z</t>
+          <t>2026-07-10T04:55:57.000Z</t>
         </is>
       </c>
     </row>
@@ -5190,12 +5190,12 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>1129</v>
+        <v>898</v>
       </c>
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:33.000Z</t>
+          <t>2026-07-10T04:55:58.000Z</t>
         </is>
       </c>
     </row>
@@ -5219,12 +5219,12 @@
         </is>
       </c>
       <c r="E164" t="n">
-        <v>395</v>
+        <v>347</v>
       </c>
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:34.000Z</t>
+          <t>2026-07-10T04:55:58.000Z</t>
         </is>
       </c>
     </row>
@@ -5248,12 +5248,12 @@
         </is>
       </c>
       <c r="E165" t="n">
-        <v>1179</v>
+        <v>415</v>
       </c>
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:35.000Z</t>
+          <t>2026-07-10T04:55:59.000Z</t>
         </is>
       </c>
     </row>
@@ -5277,12 +5277,12 @@
         </is>
       </c>
       <c r="E166" t="n">
-        <v>1058</v>
+        <v>394</v>
       </c>
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:36.000Z</t>
+          <t>2026-07-10T04:56:00.000Z</t>
         </is>
       </c>
     </row>
@@ -5306,12 +5306,12 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>271</v>
+        <v>931</v>
       </c>
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:36.000Z</t>
+          <t>2026-07-10T04:56:01.000Z</t>
         </is>
       </c>
     </row>
@@ -5335,12 +5335,12 @@
         </is>
       </c>
       <c r="E168" t="n">
-        <v>276</v>
+        <v>335</v>
       </c>
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:37.000Z</t>
+          <t>2026-07-10T04:56:02.000Z</t>
         </is>
       </c>
     </row>
@@ -5364,12 +5364,12 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>934</v>
+        <v>609</v>
       </c>
       <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:38.000Z</t>
+          <t>2026-07-10T04:56:02.000Z</t>
         </is>
       </c>
     </row>
@@ -5393,12 +5393,12 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>96</v>
+        <v>1164</v>
       </c>
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:39.000Z</t>
+          <t>2026-07-10T04:56:03.000Z</t>
         </is>
       </c>
     </row>
@@ -5422,12 +5422,12 @@
         </is>
       </c>
       <c r="E171" t="n">
-        <v>649</v>
+        <v>760</v>
       </c>
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:40.000Z</t>
+          <t>2026-07-10T04:56:04.000Z</t>
         </is>
       </c>
     </row>
@@ -5451,12 +5451,12 @@
         </is>
       </c>
       <c r="E172" t="n">
-        <v>745</v>
+        <v>634</v>
       </c>
       <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:40.000Z</t>
+          <t>2026-07-10T04:56:05.000Z</t>
         </is>
       </c>
     </row>
@@ -5480,12 +5480,12 @@
         </is>
       </c>
       <c r="E173" t="n">
-        <v>678</v>
+        <v>740</v>
       </c>
       <c r="F173" t="inlineStr"/>
       <c r="G173" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:41.000Z</t>
+          <t>2026-07-10T04:56:06.000Z</t>
         </is>
       </c>
     </row>
@@ -5509,12 +5509,12 @@
         </is>
       </c>
       <c r="E174" t="n">
-        <v>1030</v>
+        <v>669</v>
       </c>
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:42.000Z</t>
+          <t>2026-07-10T04:56:06.000Z</t>
         </is>
       </c>
     </row>
@@ -5538,12 +5538,12 @@
         </is>
       </c>
       <c r="E175" t="n">
-        <v>796</v>
+        <v>1013</v>
       </c>
       <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:43.000Z</t>
+          <t>2026-07-10T04:56:07.000Z</t>
         </is>
       </c>
     </row>
@@ -5567,12 +5567,12 @@
         </is>
       </c>
       <c r="E176" t="n">
-        <v>263</v>
+        <v>150</v>
       </c>
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:44.000Z</t>
+          <t>2026-07-10T04:56:08.000Z</t>
         </is>
       </c>
     </row>
@@ -5596,12 +5596,12 @@
         </is>
       </c>
       <c r="E177" t="n">
-        <v>1014</v>
+        <v>583</v>
       </c>
       <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:44.000Z</t>
+          <t>2026-07-10T04:56:09.000Z</t>
         </is>
       </c>
     </row>
@@ -5625,12 +5625,12 @@
         </is>
       </c>
       <c r="E178" t="n">
-        <v>905</v>
+        <v>1136</v>
       </c>
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:45.000Z</t>
+          <t>2026-07-10T04:56:10.000Z</t>
         </is>
       </c>
     </row>
@@ -5654,12 +5654,12 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>180</v>
+        <v>1085</v>
       </c>
       <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:46.000Z</t>
+          <t>2026-07-10T04:56:10.000Z</t>
         </is>
       </c>
     </row>
@@ -5683,12 +5683,12 @@
         </is>
       </c>
       <c r="E180" t="n">
-        <v>812</v>
+        <v>630</v>
       </c>
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:47.000Z</t>
+          <t>2026-07-10T04:56:11.000Z</t>
         </is>
       </c>
     </row>
@@ -5712,12 +5712,12 @@
         </is>
       </c>
       <c r="E181" t="n">
-        <v>1176</v>
+        <v>201</v>
       </c>
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:48.000Z</t>
+          <t>2026-07-10T04:56:12.000Z</t>
         </is>
       </c>
     </row>
@@ -5741,12 +5741,12 @@
         </is>
       </c>
       <c r="E182" t="n">
-        <v>241</v>
+        <v>460</v>
       </c>
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:48.000Z</t>
+          <t>2026-07-10T04:56:13.000Z</t>
         </is>
       </c>
     </row>
@@ -5770,12 +5770,12 @@
         </is>
       </c>
       <c r="E183" t="n">
-        <v>577</v>
+        <v>695</v>
       </c>
       <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:49.000Z</t>
+          <t>2026-07-10T04:56:14.000Z</t>
         </is>
       </c>
     </row>
@@ -5799,12 +5799,12 @@
         </is>
       </c>
       <c r="E184" t="n">
-        <v>617</v>
+        <v>877</v>
       </c>
       <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:50.000Z</t>
+          <t>2026-07-10T04:56:14.000Z</t>
         </is>
       </c>
     </row>
@@ -5828,12 +5828,12 @@
         </is>
       </c>
       <c r="E185" t="n">
-        <v>1098</v>
+        <v>209</v>
       </c>
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:51.000Z</t>
+          <t>2026-07-10T04:56:15.000Z</t>
         </is>
       </c>
     </row>
@@ -5857,12 +5857,12 @@
         </is>
       </c>
       <c r="E186" t="n">
-        <v>818</v>
+        <v>364</v>
       </c>
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:52.000Z</t>
+          <t>2026-07-10T04:56:16.000Z</t>
         </is>
       </c>
     </row>
@@ -5886,12 +5886,12 @@
         </is>
       </c>
       <c r="E187" t="n">
-        <v>287</v>
+        <v>141</v>
       </c>
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:52.000Z</t>
+          <t>2026-07-10T04:56:17.000Z</t>
         </is>
       </c>
     </row>
@@ -5915,12 +5915,12 @@
         </is>
       </c>
       <c r="E188" t="n">
-        <v>817</v>
+        <v>645</v>
       </c>
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:53.000Z</t>
+          <t>2026-07-10T04:56:18.000Z</t>
         </is>
       </c>
     </row>
@@ -5944,12 +5944,12 @@
         </is>
       </c>
       <c r="E189" t="n">
-        <v>769</v>
+        <v>617</v>
       </c>
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:54.000Z</t>
+          <t>2026-07-10T04:56:18.000Z</t>
         </is>
       </c>
     </row>
@@ -5973,12 +5973,12 @@
         </is>
       </c>
       <c r="E190" t="n">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:55.000Z</t>
+          <t>2026-07-10T04:56:19.000Z</t>
         </is>
       </c>
     </row>
@@ -6002,12 +6002,12 @@
         </is>
       </c>
       <c r="E191" t="n">
-        <v>759</v>
+        <v>225</v>
       </c>
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:56.000Z</t>
+          <t>2026-07-10T04:56:20.000Z</t>
         </is>
       </c>
     </row>
@@ -6031,12 +6031,12 @@
         </is>
       </c>
       <c r="E192" t="n">
-        <v>1029</v>
+        <v>1037</v>
       </c>
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:56.000Z</t>
+          <t>2026-07-10T04:56:21.000Z</t>
         </is>
       </c>
     </row>
@@ -6060,12 +6060,12 @@
         </is>
       </c>
       <c r="E193" t="n">
-        <v>509</v>
+        <v>865</v>
       </c>
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:57.000Z</t>
+          <t>2026-07-10T04:56:22.000Z</t>
         </is>
       </c>
     </row>
@@ -6089,12 +6089,12 @@
         </is>
       </c>
       <c r="E194" t="n">
-        <v>357</v>
+        <v>864</v>
       </c>
       <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:58.000Z</t>
+          <t>2026-07-10T04:56:22.000Z</t>
         </is>
       </c>
     </row>
@@ -6118,12 +6118,12 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>729</v>
+        <v>1076</v>
       </c>
       <c r="F195" t="inlineStr"/>
       <c r="G195" t="inlineStr">
         <is>
-          <t>2026-07-10T04:49:59.000Z</t>
+          <t>2026-07-10T04:56:23.000Z</t>
         </is>
       </c>
     </row>
@@ -6147,12 +6147,12 @@
         </is>
       </c>
       <c r="E196" t="n">
-        <v>660</v>
+        <v>793</v>
       </c>
       <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:00.000Z</t>
+          <t>2026-07-10T04:56:24.000Z</t>
         </is>
       </c>
     </row>
@@ -6176,12 +6176,12 @@
         </is>
       </c>
       <c r="E197" t="n">
-        <v>359</v>
+        <v>750</v>
       </c>
       <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:00.000Z</t>
+          <t>2026-07-10T04:56:25.000Z</t>
         </is>
       </c>
     </row>
@@ -6205,12 +6205,12 @@
         </is>
       </c>
       <c r="E198" t="n">
-        <v>942</v>
+        <v>943</v>
       </c>
       <c r="F198" t="inlineStr"/>
       <c r="G198" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:01.000Z</t>
+          <t>2026-07-10T04:56:26.000Z</t>
         </is>
       </c>
     </row>
@@ -6234,12 +6234,12 @@
         </is>
       </c>
       <c r="E199" t="n">
-        <v>219</v>
+        <v>666</v>
       </c>
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:02.000Z</t>
+          <t>2026-07-10T04:56:26.000Z</t>
         </is>
       </c>
     </row>
@@ -6263,12 +6263,12 @@
         </is>
       </c>
       <c r="E200" t="n">
-        <v>1179</v>
+        <v>618</v>
       </c>
       <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:03.000Z</t>
+          <t>2026-07-10T04:56:27.000Z</t>
         </is>
       </c>
     </row>
@@ -6292,12 +6292,12 @@
         </is>
       </c>
       <c r="E201" t="n">
-        <v>1183</v>
+        <v>436</v>
       </c>
       <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:04.000Z</t>
+          <t>2026-07-10T04:56:28.000Z</t>
         </is>
       </c>
     </row>
@@ -6321,12 +6321,12 @@
         </is>
       </c>
       <c r="E202" t="n">
-        <v>763</v>
+        <v>926</v>
       </c>
       <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:04.000Z</t>
+          <t>2026-07-10T04:56:29.000Z</t>
         </is>
       </c>
     </row>
@@ -6350,12 +6350,12 @@
         </is>
       </c>
       <c r="E203" t="n">
-        <v>685</v>
+        <v>214</v>
       </c>
       <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:05.000Z</t>
+          <t>2026-07-10T04:56:30.000Z</t>
         </is>
       </c>
     </row>
@@ -6379,12 +6379,12 @@
         </is>
       </c>
       <c r="E204" t="n">
-        <v>109</v>
+        <v>570</v>
       </c>
       <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:06.000Z</t>
+          <t>2026-07-10T04:56:30.000Z</t>
         </is>
       </c>
     </row>
@@ -6408,12 +6408,12 @@
         </is>
       </c>
       <c r="E205" t="n">
-        <v>563</v>
+        <v>1043</v>
       </c>
       <c r="F205" t="inlineStr"/>
       <c r="G205" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:07.000Z</t>
+          <t>2026-07-10T04:56:31.000Z</t>
         </is>
       </c>
     </row>
@@ -6437,12 +6437,12 @@
         </is>
       </c>
       <c r="E206" t="n">
-        <v>315</v>
+        <v>872</v>
       </c>
       <c r="F206" t="inlineStr"/>
       <c r="G206" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:08.000Z</t>
+          <t>2026-07-10T04:56:32.000Z</t>
         </is>
       </c>
     </row>
@@ -6466,12 +6466,12 @@
         </is>
       </c>
       <c r="E207" t="n">
-        <v>720</v>
+        <v>120</v>
       </c>
       <c r="F207" t="inlineStr"/>
       <c r="G207" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:08.000Z</t>
+          <t>2026-07-10T04:56:33.000Z</t>
         </is>
       </c>
     </row>
@@ -6495,12 +6495,12 @@
         </is>
       </c>
       <c r="E208" t="n">
-        <v>205</v>
+        <v>1104</v>
       </c>
       <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:09.000Z</t>
+          <t>2026-07-10T04:56:34.000Z</t>
         </is>
       </c>
     </row>
@@ -6524,12 +6524,12 @@
         </is>
       </c>
       <c r="E209" t="n">
-        <v>326</v>
+        <v>244</v>
       </c>
       <c r="F209" t="inlineStr"/>
       <c r="G209" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:10.000Z</t>
+          <t>2026-07-10T04:56:34.000Z</t>
         </is>
       </c>
     </row>
@@ -6553,12 +6553,12 @@
         </is>
       </c>
       <c r="E210" t="n">
-        <v>854</v>
+        <v>906</v>
       </c>
       <c r="F210" t="inlineStr"/>
       <c r="G210" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:11.000Z</t>
+          <t>2026-07-10T04:56:35.000Z</t>
         </is>
       </c>
     </row>
@@ -6582,12 +6582,12 @@
         </is>
       </c>
       <c r="E211" t="n">
-        <v>916</v>
+        <v>961</v>
       </c>
       <c r="F211" t="inlineStr"/>
       <c r="G211" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:12.000Z</t>
+          <t>2026-07-10T04:56:36.000Z</t>
         </is>
       </c>
     </row>
@@ -6611,12 +6611,12 @@
         </is>
       </c>
       <c r="E212" t="n">
-        <v>755</v>
+        <v>801</v>
       </c>
       <c r="F212" t="inlineStr"/>
       <c r="G212" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:12.000Z</t>
+          <t>2026-07-10T04:56:37.000Z</t>
         </is>
       </c>
     </row>
@@ -6640,12 +6640,12 @@
         </is>
       </c>
       <c r="E213" t="n">
-        <v>839</v>
+        <v>85</v>
       </c>
       <c r="F213" t="inlineStr"/>
       <c r="G213" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:13.000Z</t>
+          <t>2026-07-10T04:56:38.000Z</t>
         </is>
       </c>
     </row>
@@ -6669,12 +6669,12 @@
         </is>
       </c>
       <c r="E214" t="n">
-        <v>772</v>
+        <v>662</v>
       </c>
       <c r="F214" t="inlineStr"/>
       <c r="G214" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:14.000Z</t>
+          <t>2026-07-10T04:56:38.000Z</t>
         </is>
       </c>
     </row>
@@ -6698,12 +6698,12 @@
         </is>
       </c>
       <c r="E215" t="n">
-        <v>892</v>
+        <v>269</v>
       </c>
       <c r="F215" t="inlineStr"/>
       <c r="G215" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:15.000Z</t>
+          <t>2026-07-10T04:56:39.000Z</t>
         </is>
       </c>
     </row>
@@ -6727,12 +6727,12 @@
         </is>
       </c>
       <c r="E216" t="n">
-        <v>623</v>
+        <v>107</v>
       </c>
       <c r="F216" t="inlineStr"/>
       <c r="G216" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:16.000Z</t>
+          <t>2026-07-10T04:56:40.000Z</t>
         </is>
       </c>
     </row>
@@ -6756,12 +6756,12 @@
         </is>
       </c>
       <c r="E217" t="n">
-        <v>401</v>
+        <v>206</v>
       </c>
       <c r="F217" t="inlineStr"/>
       <c r="G217" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:16.000Z</t>
+          <t>2026-07-10T04:56:41.000Z</t>
         </is>
       </c>
     </row>
@@ -6785,12 +6785,12 @@
         </is>
       </c>
       <c r="E218" t="n">
-        <v>395</v>
+        <v>787</v>
       </c>
       <c r="F218" t="inlineStr"/>
       <c r="G218" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:17.000Z</t>
+          <t>2026-07-10T04:56:42.000Z</t>
         </is>
       </c>
     </row>
@@ -6814,12 +6814,12 @@
         </is>
       </c>
       <c r="E219" t="n">
-        <v>927</v>
+        <v>471</v>
       </c>
       <c r="F219" t="inlineStr"/>
       <c r="G219" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:18.000Z</t>
+          <t>2026-07-10T04:56:42.000Z</t>
         </is>
       </c>
     </row>
@@ -6843,12 +6843,12 @@
         </is>
       </c>
       <c r="E220" t="n">
-        <v>1158</v>
+        <v>1088</v>
       </c>
       <c r="F220" t="inlineStr"/>
       <c r="G220" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:19.000Z</t>
+          <t>2026-07-10T04:56:43.000Z</t>
         </is>
       </c>
     </row>
@@ -6872,12 +6872,12 @@
         </is>
       </c>
       <c r="E221" t="n">
-        <v>1107</v>
+        <v>1054</v>
       </c>
       <c r="F221" t="inlineStr"/>
       <c r="G221" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:20.000Z</t>
+          <t>2026-07-10T04:56:44.000Z</t>
         </is>
       </c>
     </row>
@@ -6901,12 +6901,12 @@
         </is>
       </c>
       <c r="E222" t="n">
-        <v>523</v>
+        <v>189</v>
       </c>
       <c r="F222" t="inlineStr"/>
       <c r="G222" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:20.000Z</t>
+          <t>2026-07-10T04:56:45.000Z</t>
         </is>
       </c>
     </row>
@@ -6930,12 +6930,12 @@
         </is>
       </c>
       <c r="E223" t="n">
-        <v>367</v>
+        <v>1156</v>
       </c>
       <c r="F223" t="inlineStr"/>
       <c r="G223" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:21.000Z</t>
+          <t>2026-07-10T04:56:46.000Z</t>
         </is>
       </c>
     </row>
@@ -6959,12 +6959,12 @@
         </is>
       </c>
       <c r="E224" t="n">
-        <v>1088</v>
+        <v>890</v>
       </c>
       <c r="F224" t="inlineStr"/>
       <c r="G224" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:22.000Z</t>
+          <t>2026-07-10T04:56:46.000Z</t>
         </is>
       </c>
     </row>
@@ -6988,12 +6988,12 @@
         </is>
       </c>
       <c r="E225" t="n">
-        <v>502</v>
+        <v>745</v>
       </c>
       <c r="F225" t="inlineStr"/>
       <c r="G225" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:23.000Z</t>
+          <t>2026-07-10T04:56:47.000Z</t>
         </is>
       </c>
     </row>
@@ -7017,12 +7017,12 @@
         </is>
       </c>
       <c r="E226" t="n">
-        <v>1106</v>
+        <v>542</v>
       </c>
       <c r="F226" t="inlineStr"/>
       <c r="G226" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:24.000Z</t>
+          <t>2026-07-10T04:56:48.000Z</t>
         </is>
       </c>
     </row>
@@ -7046,12 +7046,12 @@
         </is>
       </c>
       <c r="E227" t="n">
-        <v>228</v>
+        <v>420</v>
       </c>
       <c r="F227" t="inlineStr"/>
       <c r="G227" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:24.000Z</t>
+          <t>2026-07-10T04:56:49.000Z</t>
         </is>
       </c>
     </row>
@@ -7075,12 +7075,12 @@
         </is>
       </c>
       <c r="E228" t="n">
-        <v>258</v>
+        <v>773</v>
       </c>
       <c r="F228" t="inlineStr"/>
       <c r="G228" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:25.000Z</t>
+          <t>2026-07-10T04:56:50.000Z</t>
         </is>
       </c>
     </row>
@@ -7104,12 +7104,12 @@
         </is>
       </c>
       <c r="E229" t="n">
-        <v>346</v>
+        <v>108</v>
       </c>
       <c r="F229" t="inlineStr"/>
       <c r="G229" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:26.000Z</t>
+          <t>2026-07-10T04:56:50.000Z</t>
         </is>
       </c>
     </row>
@@ -7133,12 +7133,12 @@
         </is>
       </c>
       <c r="E230" t="n">
-        <v>735</v>
+        <v>1040</v>
       </c>
       <c r="F230" t="inlineStr"/>
       <c r="G230" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:27.000Z</t>
+          <t>2026-07-10T04:56:51.000Z</t>
         </is>
       </c>
     </row>
@@ -7162,12 +7162,12 @@
         </is>
       </c>
       <c r="E231" t="n">
-        <v>618</v>
+        <v>404</v>
       </c>
       <c r="F231" t="inlineStr"/>
       <c r="G231" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:28.000Z</t>
+          <t>2026-07-10T04:56:52.000Z</t>
         </is>
       </c>
     </row>
@@ -7191,12 +7191,12 @@
         </is>
       </c>
       <c r="E232" t="n">
-        <v>727</v>
+        <v>929</v>
       </c>
       <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:28.000Z</t>
+          <t>2026-07-10T04:56:53.000Z</t>
         </is>
       </c>
     </row>
@@ -7220,12 +7220,12 @@
         </is>
       </c>
       <c r="E233" t="n">
-        <v>998</v>
+        <v>881</v>
       </c>
       <c r="F233" t="inlineStr"/>
       <c r="G233" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:29.000Z</t>
+          <t>2026-07-10T04:56:54.000Z</t>
         </is>
       </c>
     </row>
@@ -7249,12 +7249,12 @@
         </is>
       </c>
       <c r="E234" t="n">
-        <v>247</v>
+        <v>1079</v>
       </c>
       <c r="F234" t="inlineStr"/>
       <c r="G234" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:30.000Z</t>
+          <t>2026-07-10T04:56:54.000Z</t>
         </is>
       </c>
     </row>
@@ -7278,12 +7278,12 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>564</v>
+        <v>248</v>
       </c>
       <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:31.000Z</t>
+          <t>2026-07-10T04:56:55.000Z</t>
         </is>
       </c>
     </row>
@@ -7307,12 +7307,12 @@
         </is>
       </c>
       <c r="E236" t="n">
-        <v>968</v>
+        <v>416</v>
       </c>
       <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:32.000Z</t>
+          <t>2026-07-10T04:56:56.000Z</t>
         </is>
       </c>
     </row>
@@ -7336,12 +7336,12 @@
         </is>
       </c>
       <c r="E237" t="n">
-        <v>944</v>
+        <v>754</v>
       </c>
       <c r="F237" t="inlineStr"/>
       <c r="G237" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:32.000Z</t>
+          <t>2026-07-10T04:56:57.000Z</t>
         </is>
       </c>
     </row>
@@ -7365,12 +7365,12 @@
         </is>
       </c>
       <c r="E238" t="n">
-        <v>316</v>
+        <v>165</v>
       </c>
       <c r="F238" t="inlineStr"/>
       <c r="G238" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:33.000Z</t>
+          <t>2026-07-10T04:56:58.000Z</t>
         </is>
       </c>
     </row>
@@ -7394,12 +7394,12 @@
         </is>
       </c>
       <c r="E239" t="n">
-        <v>1178</v>
+        <v>97</v>
       </c>
       <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:34.000Z</t>
+          <t>2026-07-10T04:56:58.000Z</t>
         </is>
       </c>
     </row>
@@ -7423,12 +7423,12 @@
         </is>
       </c>
       <c r="E240" t="n">
-        <v>784</v>
+        <v>297</v>
       </c>
       <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:35.000Z</t>
+          <t>2026-07-10T04:56:59.000Z</t>
         </is>
       </c>
     </row>
@@ -7452,12 +7452,12 @@
         </is>
       </c>
       <c r="E241" t="n">
-        <v>457</v>
+        <v>124</v>
       </c>
       <c r="F241" t="inlineStr"/>
       <c r="G241" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:36.000Z</t>
+          <t>2026-07-10T04:57:00.000Z</t>
         </is>
       </c>
     </row>
@@ -7481,12 +7481,12 @@
         </is>
       </c>
       <c r="E242" t="n">
-        <v>646</v>
+        <v>1177</v>
       </c>
       <c r="F242" t="inlineStr"/>
       <c r="G242" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:36.000Z</t>
+          <t>2026-07-10T04:57:01.000Z</t>
         </is>
       </c>
     </row>
@@ -7510,12 +7510,12 @@
         </is>
       </c>
       <c r="E243" t="n">
-        <v>1161</v>
+        <v>789</v>
       </c>
       <c r="F243" t="inlineStr"/>
       <c r="G243" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:37.000Z</t>
+          <t>2026-07-10T04:57:02.000Z</t>
         </is>
       </c>
     </row>
@@ -7539,12 +7539,12 @@
         </is>
       </c>
       <c r="E244" t="n">
-        <v>821</v>
+        <v>82</v>
       </c>
       <c r="F244" t="inlineStr"/>
       <c r="G244" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:38.000Z</t>
+          <t>2026-07-10T04:57:02.000Z</t>
         </is>
       </c>
     </row>
@@ -7568,12 +7568,12 @@
         </is>
       </c>
       <c r="E245" t="n">
-        <v>1057</v>
+        <v>120</v>
       </c>
       <c r="F245" t="inlineStr"/>
       <c r="G245" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:39.000Z</t>
+          <t>2026-07-10T04:57:03.000Z</t>
         </is>
       </c>
     </row>
@@ -7597,12 +7597,12 @@
         </is>
       </c>
       <c r="E246" t="n">
-        <v>677</v>
+        <v>288</v>
       </c>
       <c r="F246" t="inlineStr"/>
       <c r="G246" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:40.000Z</t>
+          <t>2026-07-10T04:57:04.000Z</t>
         </is>
       </c>
     </row>
@@ -7626,12 +7626,12 @@
         </is>
       </c>
       <c r="E247" t="n">
-        <v>775</v>
+        <v>933</v>
       </c>
       <c r="F247" t="inlineStr"/>
       <c r="G247" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:40.000Z</t>
+          <t>2026-07-10T04:57:05.000Z</t>
         </is>
       </c>
     </row>
@@ -7655,12 +7655,12 @@
         </is>
       </c>
       <c r="E248" t="n">
-        <v>178</v>
+        <v>968</v>
       </c>
       <c r="F248" t="inlineStr"/>
       <c r="G248" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:41.000Z</t>
+          <t>2026-07-10T04:57:06.000Z</t>
         </is>
       </c>
     </row>
@@ -7684,12 +7684,12 @@
         </is>
       </c>
       <c r="E249" t="n">
-        <v>240</v>
+        <v>377</v>
       </c>
       <c r="F249" t="inlineStr"/>
       <c r="G249" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:42.000Z</t>
+          <t>2026-07-10T04:57:06.000Z</t>
         </is>
       </c>
     </row>
@@ -7713,12 +7713,12 @@
         </is>
       </c>
       <c r="E250" t="n">
-        <v>1010</v>
+        <v>831</v>
       </c>
       <c r="F250" t="inlineStr"/>
       <c r="G250" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:43.000Z</t>
+          <t>2026-07-10T04:57:07.000Z</t>
         </is>
       </c>
     </row>
@@ -7742,12 +7742,12 @@
         </is>
       </c>
       <c r="E251" t="n">
-        <v>952</v>
+        <v>803</v>
       </c>
       <c r="F251" t="inlineStr"/>
       <c r="G251" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:44.000Z</t>
+          <t>2026-07-10T04:57:08.000Z</t>
         </is>
       </c>
     </row>
@@ -7771,12 +7771,12 @@
         </is>
       </c>
       <c r="E252" t="n">
-        <v>983</v>
+        <v>539</v>
       </c>
       <c r="F252" t="inlineStr"/>
       <c r="G252" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:44.000Z</t>
+          <t>2026-07-10T04:57:09.000Z</t>
         </is>
       </c>
     </row>
@@ -7800,12 +7800,12 @@
         </is>
       </c>
       <c r="E253" t="n">
-        <v>767</v>
+        <v>1116</v>
       </c>
       <c r="F253" t="inlineStr"/>
       <c r="G253" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:45.000Z</t>
+          <t>2026-07-10T04:57:10.000Z</t>
         </is>
       </c>
     </row>
@@ -7829,12 +7829,12 @@
         </is>
       </c>
       <c r="E254" t="n">
-        <v>552</v>
+        <v>1056</v>
       </c>
       <c r="F254" t="inlineStr"/>
       <c r="G254" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:46.000Z</t>
+          <t>2026-07-10T04:57:10.000Z</t>
         </is>
       </c>
     </row>
@@ -7858,12 +7858,12 @@
         </is>
       </c>
       <c r="E255" t="n">
-        <v>729</v>
+        <v>107</v>
       </c>
       <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:47.000Z</t>
+          <t>2026-07-10T04:57:11.000Z</t>
         </is>
       </c>
     </row>
@@ -7887,12 +7887,12 @@
         </is>
       </c>
       <c r="E256" t="n">
-        <v>1075</v>
+        <v>1073</v>
       </c>
       <c r="F256" t="inlineStr"/>
       <c r="G256" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:48.000Z</t>
+          <t>2026-07-10T04:57:12.000Z</t>
         </is>
       </c>
     </row>
@@ -7916,12 +7916,12 @@
         </is>
       </c>
       <c r="E257" t="n">
-        <v>163</v>
+        <v>541</v>
       </c>
       <c r="F257" t="inlineStr"/>
       <c r="G257" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:48.000Z</t>
+          <t>2026-07-10T04:57:13.000Z</t>
         </is>
       </c>
     </row>
@@ -7945,12 +7945,12 @@
         </is>
       </c>
       <c r="E258" t="n">
-        <v>244</v>
+        <v>949</v>
       </c>
       <c r="F258" t="inlineStr"/>
       <c r="G258" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:49.000Z</t>
+          <t>2026-07-10T04:57:14.000Z</t>
         </is>
       </c>
     </row>
@@ -7974,12 +7974,12 @@
         </is>
       </c>
       <c r="E259" t="n">
-        <v>333</v>
+        <v>91</v>
       </c>
       <c r="F259" t="inlineStr"/>
       <c r="G259" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:50.000Z</t>
+          <t>2026-07-10T04:57:14.000Z</t>
         </is>
       </c>
     </row>
@@ -8003,12 +8003,12 @@
         </is>
       </c>
       <c r="E260" t="n">
-        <v>1038</v>
+        <v>461</v>
       </c>
       <c r="F260" t="inlineStr"/>
       <c r="G260" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:51.000Z</t>
+          <t>2026-07-10T04:57:15.000Z</t>
         </is>
       </c>
     </row>
@@ -8032,12 +8032,12 @@
         </is>
       </c>
       <c r="E261" t="n">
-        <v>364</v>
+        <v>488</v>
       </c>
       <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:52.000Z</t>
+          <t>2026-07-10T04:57:16.000Z</t>
         </is>
       </c>
     </row>
@@ -8061,12 +8061,12 @@
         </is>
       </c>
       <c r="E262" t="n">
-        <v>1036</v>
+        <v>782</v>
       </c>
       <c r="F262" t="inlineStr"/>
       <c r="G262" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:52.000Z</t>
+          <t>2026-07-10T04:57:17.000Z</t>
         </is>
       </c>
     </row>
@@ -8090,12 +8090,12 @@
         </is>
       </c>
       <c r="E263" t="n">
-        <v>823</v>
+        <v>863</v>
       </c>
       <c r="F263" t="inlineStr"/>
       <c r="G263" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:53.000Z</t>
+          <t>2026-07-10T04:57:18.000Z</t>
         </is>
       </c>
     </row>
@@ -8119,12 +8119,12 @@
         </is>
       </c>
       <c r="E264" t="n">
-        <v>994</v>
+        <v>445</v>
       </c>
       <c r="F264" t="inlineStr"/>
       <c r="G264" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:54.000Z</t>
+          <t>2026-07-10T04:57:18.000Z</t>
         </is>
       </c>
     </row>
@@ -8148,12 +8148,12 @@
         </is>
       </c>
       <c r="E265" t="n">
-        <v>174</v>
+        <v>134</v>
       </c>
       <c r="F265" t="inlineStr"/>
       <c r="G265" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:55.000Z</t>
+          <t>2026-07-10T04:57:19.000Z</t>
         </is>
       </c>
     </row>
@@ -8177,12 +8177,12 @@
         </is>
       </c>
       <c r="E266" t="n">
-        <v>607</v>
+        <v>933</v>
       </c>
       <c r="F266" t="inlineStr"/>
       <c r="G266" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:56.000Z</t>
+          <t>2026-07-10T04:57:20.000Z</t>
         </is>
       </c>
     </row>
@@ -8206,12 +8206,12 @@
         </is>
       </c>
       <c r="E267" t="n">
-        <v>1003</v>
+        <v>902</v>
       </c>
       <c r="F267" t="inlineStr"/>
       <c r="G267" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:56.000Z</t>
+          <t>2026-07-10T04:57:21.000Z</t>
         </is>
       </c>
     </row>
@@ -8235,12 +8235,12 @@
         </is>
       </c>
       <c r="E268" t="n">
-        <v>804</v>
+        <v>94</v>
       </c>
       <c r="F268" t="inlineStr"/>
       <c r="G268" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:57.000Z</t>
+          <t>2026-07-10T04:57:22.000Z</t>
         </is>
       </c>
     </row>
@@ -8264,12 +8264,12 @@
         </is>
       </c>
       <c r="E269" t="n">
-        <v>1183</v>
+        <v>990</v>
       </c>
       <c r="F269" t="inlineStr"/>
       <c r="G269" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:58.000Z</t>
+          <t>2026-07-10T04:57:22.000Z</t>
         </is>
       </c>
     </row>
@@ -8293,12 +8293,12 @@
         </is>
       </c>
       <c r="E270" t="n">
-        <v>1093</v>
+        <v>343</v>
       </c>
       <c r="F270" t="inlineStr"/>
       <c r="G270" t="inlineStr">
         <is>
-          <t>2026-07-10T04:50:59.000Z</t>
+          <t>2026-07-10T04:57:23.000Z</t>
         </is>
       </c>
     </row>
@@ -8322,12 +8322,12 @@
         </is>
       </c>
       <c r="E271" t="n">
-        <v>937</v>
+        <v>333</v>
       </c>
       <c r="F271" t="inlineStr"/>
       <c r="G271" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:00.000Z</t>
+          <t>2026-07-10T04:57:24.000Z</t>
         </is>
       </c>
     </row>
@@ -8351,12 +8351,12 @@
         </is>
       </c>
       <c r="E272" t="n">
-        <v>556</v>
+        <v>905</v>
       </c>
       <c r="F272" t="inlineStr"/>
       <c r="G272" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:00.000Z</t>
+          <t>2026-07-10T04:57:25.000Z</t>
         </is>
       </c>
     </row>
@@ -8380,12 +8380,12 @@
         </is>
       </c>
       <c r="E273" t="n">
-        <v>947</v>
+        <v>891</v>
       </c>
       <c r="F273" t="inlineStr"/>
       <c r="G273" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:01.000Z</t>
+          <t>2026-07-10T04:57:26.000Z</t>
         </is>
       </c>
     </row>
@@ -8409,12 +8409,12 @@
         </is>
       </c>
       <c r="E274" t="n">
-        <v>446</v>
+        <v>329</v>
       </c>
       <c r="F274" t="inlineStr"/>
       <c r="G274" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:02.000Z</t>
+          <t>2026-07-10T04:57:26.000Z</t>
         </is>
       </c>
     </row>
@@ -8438,12 +8438,12 @@
         </is>
       </c>
       <c r="E275" t="n">
-        <v>361</v>
+        <v>242</v>
       </c>
       <c r="F275" t="inlineStr"/>
       <c r="G275" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:03.000Z</t>
+          <t>2026-07-10T04:57:27.000Z</t>
         </is>
       </c>
     </row>
@@ -8467,12 +8467,12 @@
         </is>
       </c>
       <c r="E276" t="n">
-        <v>343</v>
+        <v>716</v>
       </c>
       <c r="F276" t="inlineStr"/>
       <c r="G276" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:04.000Z</t>
+          <t>2026-07-10T04:57:28.000Z</t>
         </is>
       </c>
     </row>
@@ -8496,12 +8496,12 @@
         </is>
       </c>
       <c r="E277" t="n">
-        <v>93</v>
+        <v>1088</v>
       </c>
       <c r="F277" t="inlineStr"/>
       <c r="G277" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:04.000Z</t>
+          <t>2026-07-10T04:57:29.000Z</t>
         </is>
       </c>
     </row>
@@ -8525,12 +8525,12 @@
         </is>
       </c>
       <c r="E278" t="n">
-        <v>334</v>
+        <v>366</v>
       </c>
       <c r="F278" t="inlineStr"/>
       <c r="G278" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:05.000Z</t>
+          <t>2026-07-10T04:57:30.000Z</t>
         </is>
       </c>
     </row>
@@ -8554,12 +8554,12 @@
         </is>
       </c>
       <c r="E279" t="n">
-        <v>856</v>
+        <v>357</v>
       </c>
       <c r="F279" t="inlineStr"/>
       <c r="G279" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:06.000Z</t>
+          <t>2026-07-10T04:57:30.000Z</t>
         </is>
       </c>
     </row>
@@ -8583,12 +8583,12 @@
         </is>
       </c>
       <c r="E280" t="n">
-        <v>774</v>
+        <v>401</v>
       </c>
       <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:07.000Z</t>
+          <t>2026-07-10T04:57:31.000Z</t>
         </is>
       </c>
     </row>
@@ -8612,12 +8612,12 @@
         </is>
       </c>
       <c r="E281" t="n">
-        <v>476</v>
+        <v>312</v>
       </c>
       <c r="F281" t="inlineStr"/>
       <c r="G281" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:08.000Z</t>
+          <t>2026-07-10T04:57:32.000Z</t>
         </is>
       </c>
     </row>
@@ -8641,12 +8641,12 @@
         </is>
       </c>
       <c r="E282" t="n">
-        <v>252</v>
+        <v>269</v>
       </c>
       <c r="F282" t="inlineStr"/>
       <c r="G282" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:08.000Z</t>
+          <t>2026-07-10T04:57:33.000Z</t>
         </is>
       </c>
     </row>
@@ -8670,12 +8670,12 @@
         </is>
       </c>
       <c r="E283" t="n">
-        <v>215</v>
+        <v>502</v>
       </c>
       <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:09.000Z</t>
+          <t>2026-07-10T04:57:34.000Z</t>
         </is>
       </c>
     </row>
@@ -8699,12 +8699,12 @@
         </is>
       </c>
       <c r="E284" t="n">
-        <v>803</v>
+        <v>522</v>
       </c>
       <c r="F284" t="inlineStr"/>
       <c r="G284" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:10.000Z</t>
+          <t>2026-07-10T04:57:34.000Z</t>
         </is>
       </c>
     </row>
@@ -8728,12 +8728,12 @@
         </is>
       </c>
       <c r="E285" t="n">
-        <v>862</v>
+        <v>1117</v>
       </c>
       <c r="F285" t="inlineStr"/>
       <c r="G285" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:11.000Z</t>
+          <t>2026-07-10T04:57:35.000Z</t>
         </is>
       </c>
     </row>
@@ -8757,12 +8757,12 @@
         </is>
       </c>
       <c r="E286" t="n">
-        <v>444</v>
+        <v>229</v>
       </c>
       <c r="F286" t="inlineStr"/>
       <c r="G286" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:12.000Z</t>
+          <t>2026-07-10T04:57:36.000Z</t>
         </is>
       </c>
     </row>
@@ -8786,12 +8786,12 @@
         </is>
       </c>
       <c r="E287" t="n">
-        <v>322</v>
+        <v>836</v>
       </c>
       <c r="F287" t="inlineStr"/>
       <c r="G287" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:12.000Z</t>
+          <t>2026-07-10T04:57:37.000Z</t>
         </is>
       </c>
     </row>
@@ -8815,12 +8815,12 @@
         </is>
       </c>
       <c r="E288" t="n">
-        <v>381</v>
+        <v>963</v>
       </c>
       <c r="F288" t="inlineStr"/>
       <c r="G288" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:13.000Z</t>
+          <t>2026-07-10T04:57:38.000Z</t>
         </is>
       </c>
     </row>
@@ -8844,12 +8844,12 @@
         </is>
       </c>
       <c r="E289" t="n">
-        <v>457</v>
+        <v>1014</v>
       </c>
       <c r="F289" t="inlineStr"/>
       <c r="G289" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:14.000Z</t>
+          <t>2026-07-10T04:57:38.000Z</t>
         </is>
       </c>
     </row>
@@ -8873,12 +8873,12 @@
         </is>
       </c>
       <c r="E290" t="n">
-        <v>83</v>
+        <v>941</v>
       </c>
       <c r="F290" t="inlineStr"/>
       <c r="G290" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:15.000Z</t>
+          <t>2026-07-10T04:57:39.000Z</t>
         </is>
       </c>
     </row>
@@ -8902,12 +8902,12 @@
         </is>
       </c>
       <c r="E291" t="n">
-        <v>362</v>
+        <v>1098</v>
       </c>
       <c r="F291" t="inlineStr"/>
       <c r="G291" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:16.000Z</t>
+          <t>2026-07-10T04:57:40.000Z</t>
         </is>
       </c>
     </row>
@@ -8931,12 +8931,12 @@
         </is>
       </c>
       <c r="E292" t="n">
-        <v>490</v>
+        <v>1128</v>
       </c>
       <c r="F292" t="inlineStr"/>
       <c r="G292" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:16.000Z</t>
+          <t>2026-07-10T04:57:41.000Z</t>
         </is>
       </c>
     </row>
@@ -8960,12 +8960,12 @@
         </is>
       </c>
       <c r="E293" t="n">
-        <v>283</v>
+        <v>1141</v>
       </c>
       <c r="F293" t="inlineStr"/>
       <c r="G293" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:17.000Z</t>
+          <t>2026-07-10T04:57:42.000Z</t>
         </is>
       </c>
     </row>
@@ -8989,12 +8989,12 @@
         </is>
       </c>
       <c r="E294" t="n">
-        <v>1009</v>
+        <v>204</v>
       </c>
       <c r="F294" t="inlineStr"/>
       <c r="G294" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:18.000Z</t>
+          <t>2026-07-10T04:57:42.000Z</t>
         </is>
       </c>
     </row>
@@ -9018,12 +9018,12 @@
         </is>
       </c>
       <c r="E295" t="n">
-        <v>834</v>
+        <v>536</v>
       </c>
       <c r="F295" t="inlineStr"/>
       <c r="G295" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:19.000Z</t>
+          <t>2026-07-10T04:57:43.000Z</t>
         </is>
       </c>
     </row>
@@ -9047,12 +9047,12 @@
         </is>
       </c>
       <c r="E296" t="n">
-        <v>661</v>
+        <v>1000</v>
       </c>
       <c r="F296" t="inlineStr"/>
       <c r="G296" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:20.000Z</t>
+          <t>2026-07-10T04:57:44.000Z</t>
         </is>
       </c>
     </row>
@@ -9076,12 +9076,12 @@
         </is>
       </c>
       <c r="E297" t="n">
-        <v>251</v>
+        <v>573</v>
       </c>
       <c r="F297" t="inlineStr"/>
       <c r="G297" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:20.000Z</t>
+          <t>2026-07-10T04:57:45.000Z</t>
         </is>
       </c>
     </row>
@@ -9105,12 +9105,12 @@
         </is>
       </c>
       <c r="E298" t="n">
-        <v>329</v>
+        <v>1100</v>
       </c>
       <c r="F298" t="inlineStr"/>
       <c r="G298" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:21.000Z</t>
+          <t>2026-07-10T04:57:46.000Z</t>
         </is>
       </c>
     </row>
@@ -9134,12 +9134,12 @@
         </is>
       </c>
       <c r="E299" t="n">
-        <v>928</v>
+        <v>851</v>
       </c>
       <c r="F299" t="inlineStr"/>
       <c r="G299" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:22.000Z</t>
+          <t>2026-07-10T04:57:46.000Z</t>
         </is>
       </c>
     </row>
@@ -9163,12 +9163,12 @@
         </is>
       </c>
       <c r="E300" t="n">
-        <v>569</v>
+        <v>564</v>
       </c>
       <c r="F300" t="inlineStr"/>
       <c r="G300" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:23.000Z</t>
+          <t>2026-07-10T04:57:47.000Z</t>
         </is>
       </c>
     </row>
@@ -9192,12 +9192,12 @@
         </is>
       </c>
       <c r="E301" t="n">
-        <v>531</v>
+        <v>253</v>
       </c>
       <c r="F301" t="inlineStr"/>
       <c r="G301" t="inlineStr">
         <is>
-          <t>2026-07-10T04:51:24.000Z</t>
+          <t>2026-07-10T04:57:48.000Z</t>
         </is>
       </c>
     </row>
@@ -9325,7 +9325,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-10T04:47:24.000Z</t>
+          <t>2026-07-10T04:53:48.000Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploy Test Reports — 1200 Tests All PASSED 256f12e869c7d1509c2a133de803ef43f406a143
</commit_message>
<xml_diff>
--- a/reports/latest/Appium_Report.xlsx
+++ b/reports/latest/Appium_Report.xlsx
@@ -521,12 +521,12 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>473</v>
+        <v>312</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-10T04:53:49.000Z</t>
+          <t>2026-07-10T05:24:38.000Z</t>
         </is>
       </c>
     </row>
@@ -550,12 +550,12 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>799</v>
+        <v>666</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-10T04:53:50.000Z</t>
+          <t>2026-07-10T05:24:38.000Z</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>775</v>
+        <v>817</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-10T04:53:50.000Z</t>
+          <t>2026-07-10T05:24:39.000Z</t>
         </is>
       </c>
     </row>
@@ -608,12 +608,12 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>189</v>
+        <v>134</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-10T04:53:51.000Z</t>
+          <t>2026-07-10T05:24:40.000Z</t>
         </is>
       </c>
     </row>
@@ -637,12 +637,12 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>415</v>
+        <v>950</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-10T04:53:52.000Z</t>
+          <t>2026-07-10T05:24:41.000Z</t>
         </is>
       </c>
     </row>
@@ -666,12 +666,12 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>486</v>
+        <v>1141</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-10T04:53:53.000Z</t>
+          <t>2026-07-10T05:24:42.000Z</t>
         </is>
       </c>
     </row>
@@ -695,12 +695,12 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1079</v>
+        <v>231</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-07-10T04:53:54.000Z</t>
+          <t>2026-07-10T05:24:42.000Z</t>
         </is>
       </c>
     </row>
@@ -724,12 +724,12 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>724</v>
+        <v>1166</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-07-10T04:53:54.000Z</t>
+          <t>2026-07-10T05:24:43.000Z</t>
         </is>
       </c>
     </row>
@@ -753,12 +753,12 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>339</v>
+        <v>1041</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-07-10T04:53:55.000Z</t>
+          <t>2026-07-10T05:24:44.000Z</t>
         </is>
       </c>
     </row>
@@ -782,12 +782,12 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>140</v>
+        <v>472</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-07-10T04:53:56.000Z</t>
+          <t>2026-07-10T05:24:45.000Z</t>
         </is>
       </c>
     </row>
@@ -811,12 +811,12 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1065</v>
+        <v>122</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-10T04:53:57.000Z</t>
+          <t>2026-07-10T05:24:46.000Z</t>
         </is>
       </c>
     </row>
@@ -840,12 +840,12 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>185</v>
+        <v>1188</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-07-10T04:53:58.000Z</t>
+          <t>2026-07-10T05:24:46.000Z</t>
         </is>
       </c>
     </row>
@@ -869,12 +869,12 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>378</v>
+        <v>972</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-10T04:53:58.000Z</t>
+          <t>2026-07-10T05:24:47.000Z</t>
         </is>
       </c>
     </row>
@@ -898,12 +898,12 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>912</v>
+        <v>902</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-10T04:53:59.000Z</t>
+          <t>2026-07-10T05:24:48.000Z</t>
         </is>
       </c>
     </row>
@@ -927,12 +927,12 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>651</v>
+        <v>807</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:00.000Z</t>
+          <t>2026-07-10T05:24:49.000Z</t>
         </is>
       </c>
     </row>
@@ -956,12 +956,12 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>91</v>
+        <v>1103</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:01.000Z</t>
+          <t>2026-07-10T05:24:50.000Z</t>
         </is>
       </c>
     </row>
@@ -985,12 +985,12 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>874</v>
+        <v>109</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:02.000Z</t>
+          <t>2026-07-10T05:24:50.000Z</t>
         </is>
       </c>
     </row>
@@ -1014,12 +1014,12 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>700</v>
+        <v>677</v>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:02.000Z</t>
+          <t>2026-07-10T05:24:51.000Z</t>
         </is>
       </c>
     </row>
@@ -1043,12 +1043,12 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>234</v>
+        <v>515</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:03.000Z</t>
+          <t>2026-07-10T05:24:52.000Z</t>
         </is>
       </c>
     </row>
@@ -1072,12 +1072,12 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>855</v>
+        <v>143</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:04.000Z</t>
+          <t>2026-07-10T05:24:53.000Z</t>
         </is>
       </c>
     </row>
@@ -1101,12 +1101,12 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>410</v>
+        <v>935</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:05.000Z</t>
+          <t>2026-07-10T05:24:54.000Z</t>
         </is>
       </c>
     </row>
@@ -1130,12 +1130,12 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>801</v>
+        <v>235</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:06.000Z</t>
+          <t>2026-07-10T05:24:54.000Z</t>
         </is>
       </c>
     </row>
@@ -1159,12 +1159,12 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>882</v>
+        <v>421</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:06.000Z</t>
+          <t>2026-07-10T05:24:55.000Z</t>
         </is>
       </c>
     </row>
@@ -1188,12 +1188,12 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>394</v>
+        <v>580</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:07.000Z</t>
+          <t>2026-07-10T05:24:56.000Z</t>
         </is>
       </c>
     </row>
@@ -1217,12 +1217,12 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:08.000Z</t>
+          <t>2026-07-10T05:24:57.000Z</t>
         </is>
       </c>
     </row>
@@ -1246,12 +1246,12 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>758</v>
+        <v>844</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:09.000Z</t>
+          <t>2026-07-10T05:24:58.000Z</t>
         </is>
       </c>
     </row>
@@ -1275,12 +1275,12 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>283</v>
+        <v>114</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:10.000Z</t>
+          <t>2026-07-10T05:24:58.000Z</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>951</v>
+        <v>227</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:10.000Z</t>
+          <t>2026-07-10T05:24:59.000Z</t>
         </is>
       </c>
     </row>
@@ -1333,12 +1333,12 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>848</v>
+        <v>991</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:11.000Z</t>
+          <t>2026-07-10T05:25:00.000Z</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>96</v>
+        <v>1035</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:12.000Z</t>
+          <t>2026-07-10T05:25:01.000Z</t>
         </is>
       </c>
     </row>
@@ -1391,12 +1391,12 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>141</v>
+        <v>632</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:13.000Z</t>
+          <t>2026-07-10T05:25:02.000Z</t>
         </is>
       </c>
     </row>
@@ -1420,12 +1420,12 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>1135</v>
+        <v>918</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:14.000Z</t>
+          <t>2026-07-10T05:25:02.000Z</t>
         </is>
       </c>
     </row>
@@ -1449,12 +1449,12 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>529</v>
+        <v>571</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:14.000Z</t>
+          <t>2026-07-10T05:25:03.000Z</t>
         </is>
       </c>
     </row>
@@ -1478,12 +1478,12 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>956</v>
+        <v>1104</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:15.000Z</t>
+          <t>2026-07-10T05:25:04.000Z</t>
         </is>
       </c>
     </row>
@@ -1507,12 +1507,12 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>233</v>
+        <v>384</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:16.000Z</t>
+          <t>2026-07-10T05:25:05.000Z</t>
         </is>
       </c>
     </row>
@@ -1536,12 +1536,12 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>480</v>
+        <v>330</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:17.000Z</t>
+          <t>2026-07-10T05:25:06.000Z</t>
         </is>
       </c>
     </row>
@@ -1565,12 +1565,12 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>773</v>
+        <v>922</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:18.000Z</t>
+          <t>2026-07-10T05:25:06.000Z</t>
         </is>
       </c>
     </row>
@@ -1594,12 +1594,12 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>1037</v>
+        <v>416</v>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:18.000Z</t>
+          <t>2026-07-10T05:25:07.000Z</t>
         </is>
       </c>
     </row>
@@ -1623,12 +1623,12 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>520</v>
+        <v>284</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:19.000Z</t>
+          <t>2026-07-10T05:25:08.000Z</t>
         </is>
       </c>
     </row>
@@ -1652,12 +1652,12 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>203</v>
+        <v>925</v>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:20.000Z</t>
+          <t>2026-07-10T05:25:09.000Z</t>
         </is>
       </c>
     </row>
@@ -1681,12 +1681,12 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>955</v>
+        <v>911</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:21.000Z</t>
+          <t>2026-07-10T05:25:10.000Z</t>
         </is>
       </c>
     </row>
@@ -1710,12 +1710,12 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>1037</v>
+        <v>1005</v>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:22.000Z</t>
+          <t>2026-07-10T05:25:10.000Z</t>
         </is>
       </c>
     </row>
@@ -1739,12 +1739,12 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>735</v>
+        <v>110</v>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:22.000Z</t>
+          <t>2026-07-10T05:25:11.000Z</t>
         </is>
       </c>
     </row>
@@ -1768,12 +1768,12 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>1050</v>
+        <v>744</v>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:23.000Z</t>
+          <t>2026-07-10T05:25:12.000Z</t>
         </is>
       </c>
     </row>
@@ -1797,12 +1797,12 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>1041</v>
+        <v>618</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:24.000Z</t>
+          <t>2026-07-10T05:25:13.000Z</t>
         </is>
       </c>
     </row>
@@ -1826,12 +1826,12 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>297</v>
+        <v>166</v>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:25.000Z</t>
+          <t>2026-07-10T05:25:14.000Z</t>
         </is>
       </c>
     </row>
@@ -1855,12 +1855,12 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>660</v>
+        <v>973</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:26.000Z</t>
+          <t>2026-07-10T05:25:14.000Z</t>
         </is>
       </c>
     </row>
@@ -1884,12 +1884,12 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>946</v>
+        <v>246</v>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:26.000Z</t>
+          <t>2026-07-10T05:25:15.000Z</t>
         </is>
       </c>
     </row>
@@ -1913,12 +1913,12 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>943</v>
+        <v>252</v>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:27.000Z</t>
+          <t>2026-07-10T05:25:16.000Z</t>
         </is>
       </c>
     </row>
@@ -1942,12 +1942,12 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>1080</v>
+        <v>620</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:28.000Z</t>
+          <t>2026-07-10T05:25:17.000Z</t>
         </is>
       </c>
     </row>
@@ -1971,12 +1971,12 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>688</v>
+        <v>1072</v>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:29.000Z</t>
+          <t>2026-07-10T05:25:18.000Z</t>
         </is>
       </c>
     </row>
@@ -2000,12 +2000,12 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>1075</v>
+        <v>397</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:30.000Z</t>
+          <t>2026-07-10T05:25:18.000Z</t>
         </is>
       </c>
     </row>
@@ -2029,12 +2029,12 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>872</v>
+        <v>126</v>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:30.000Z</t>
+          <t>2026-07-10T05:25:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2058,12 +2058,12 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>726</v>
+        <v>576</v>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:31.000Z</t>
+          <t>2026-07-10T05:25:20.000Z</t>
         </is>
       </c>
     </row>
@@ -2087,12 +2087,12 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>580</v>
+        <v>806</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:32.000Z</t>
+          <t>2026-07-10T05:25:21.000Z</t>
         </is>
       </c>
     </row>
@@ -2116,12 +2116,12 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>104</v>
+        <v>1095</v>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:33.000Z</t>
+          <t>2026-07-10T05:25:22.000Z</t>
         </is>
       </c>
     </row>
@@ -2145,12 +2145,12 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>664</v>
+        <v>330</v>
       </c>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:34.000Z</t>
+          <t>2026-07-10T05:25:22.000Z</t>
         </is>
       </c>
     </row>
@@ -2174,12 +2174,12 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>857</v>
+        <v>90</v>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:34.000Z</t>
+          <t>2026-07-10T05:25:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2203,12 +2203,12 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>1129</v>
+        <v>555</v>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:35.000Z</t>
+          <t>2026-07-10T05:25:24.000Z</t>
         </is>
       </c>
     </row>
@@ -2232,12 +2232,12 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>376</v>
+        <v>557</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:36.000Z</t>
+          <t>2026-07-10T05:25:25.000Z</t>
         </is>
       </c>
     </row>
@@ -2261,12 +2261,12 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>149</v>
+        <v>843</v>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:37.000Z</t>
+          <t>2026-07-10T05:25:26.000Z</t>
         </is>
       </c>
     </row>
@@ -2290,12 +2290,12 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>1086</v>
+        <v>132</v>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:38.000Z</t>
+          <t>2026-07-10T05:25:26.000Z</t>
         </is>
       </c>
     </row>
@@ -2319,12 +2319,12 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>1074</v>
+        <v>762</v>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:38.000Z</t>
+          <t>2026-07-10T05:25:27.000Z</t>
         </is>
       </c>
     </row>
@@ -2348,12 +2348,12 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>1136</v>
+        <v>910</v>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:39.000Z</t>
+          <t>2026-07-10T05:25:28.000Z</t>
         </is>
       </c>
     </row>
@@ -2377,12 +2377,12 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>891</v>
+        <v>383</v>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:40.000Z</t>
+          <t>2026-07-10T05:25:29.000Z</t>
         </is>
       </c>
     </row>
@@ -2406,12 +2406,12 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>608</v>
+        <v>1183</v>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:41.000Z</t>
+          <t>2026-07-10T05:25:30.000Z</t>
         </is>
       </c>
     </row>
@@ -2435,12 +2435,12 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>741</v>
+        <v>142</v>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:42.000Z</t>
+          <t>2026-07-10T05:25:30.000Z</t>
         </is>
       </c>
     </row>
@@ -2464,12 +2464,12 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>83</v>
+        <v>978</v>
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:42.000Z</t>
+          <t>2026-07-10T05:25:31.000Z</t>
         </is>
       </c>
     </row>
@@ -2493,12 +2493,12 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>327</v>
+        <v>217</v>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:43.000Z</t>
+          <t>2026-07-10T05:25:32.000Z</t>
         </is>
       </c>
     </row>
@@ -2522,12 +2522,12 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>513</v>
+        <v>199</v>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:44.000Z</t>
+          <t>2026-07-10T05:25:33.000Z</t>
         </is>
       </c>
     </row>
@@ -2551,12 +2551,12 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>805</v>
+        <v>719</v>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:45.000Z</t>
+          <t>2026-07-10T05:25:34.000Z</t>
         </is>
       </c>
     </row>
@@ -2580,12 +2580,12 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>720</v>
+        <v>925</v>
       </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:46.000Z</t>
+          <t>2026-07-10T05:25:34.000Z</t>
         </is>
       </c>
     </row>
@@ -2609,12 +2609,12 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>446</v>
+        <v>101</v>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:46.000Z</t>
+          <t>2026-07-10T05:25:35.000Z</t>
         </is>
       </c>
     </row>
@@ -2638,12 +2638,12 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>693</v>
+        <v>574</v>
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:47.000Z</t>
+          <t>2026-07-10T05:25:36.000Z</t>
         </is>
       </c>
     </row>
@@ -2667,12 +2667,12 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>89</v>
+        <v>418</v>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:48.000Z</t>
+          <t>2026-07-10T05:25:37.000Z</t>
         </is>
       </c>
     </row>
@@ -2696,12 +2696,12 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>733</v>
+        <v>527</v>
       </c>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:49.000Z</t>
+          <t>2026-07-10T05:25:38.000Z</t>
         </is>
       </c>
     </row>
@@ -2725,12 +2725,12 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>1096</v>
+        <v>1043</v>
       </c>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:50.000Z</t>
+          <t>2026-07-10T05:25:38.000Z</t>
         </is>
       </c>
     </row>
@@ -2754,12 +2754,12 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:50.000Z</t>
+          <t>2026-07-10T05:25:39.000Z</t>
         </is>
       </c>
     </row>
@@ -2783,12 +2783,12 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>404</v>
+        <v>771</v>
       </c>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:51.000Z</t>
+          <t>2026-07-10T05:25:40.000Z</t>
         </is>
       </c>
     </row>
@@ -2812,12 +2812,12 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>153</v>
+        <v>821</v>
       </c>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:52.000Z</t>
+          <t>2026-07-10T05:25:41.000Z</t>
         </is>
       </c>
     </row>
@@ -2841,12 +2841,12 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>1088</v>
+        <v>156</v>
       </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:53.000Z</t>
+          <t>2026-07-10T05:25:42.000Z</t>
         </is>
       </c>
     </row>
@@ -2870,12 +2870,12 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>260</v>
+        <v>627</v>
       </c>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:54.000Z</t>
+          <t>2026-07-10T05:25:42.000Z</t>
         </is>
       </c>
     </row>
@@ -2899,12 +2899,12 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>1122</v>
+        <v>172</v>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:54.000Z</t>
+          <t>2026-07-10T05:25:43.000Z</t>
         </is>
       </c>
     </row>
@@ -2928,12 +2928,12 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>611</v>
+        <v>471</v>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:55.000Z</t>
+          <t>2026-07-10T05:25:44.000Z</t>
         </is>
       </c>
     </row>
@@ -2957,12 +2957,12 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>368</v>
+        <v>668</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:56.000Z</t>
+          <t>2026-07-10T05:25:45.000Z</t>
         </is>
       </c>
     </row>
@@ -2986,12 +2986,12 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>874</v>
+        <v>195</v>
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:57.000Z</t>
+          <t>2026-07-10T05:25:46.000Z</t>
         </is>
       </c>
     </row>
@@ -3015,12 +3015,12 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>972</v>
+        <v>702</v>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:58.000Z</t>
+          <t>2026-07-10T05:25:46.000Z</t>
         </is>
       </c>
     </row>
@@ -3044,12 +3044,12 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>904</v>
+        <v>832</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:58.000Z</t>
+          <t>2026-07-10T05:25:47.000Z</t>
         </is>
       </c>
     </row>
@@ -3073,12 +3073,12 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>1169</v>
+        <v>925</v>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026-07-10T04:54:59.000Z</t>
+          <t>2026-07-10T05:25:48.000Z</t>
         </is>
       </c>
     </row>
@@ -3102,12 +3102,12 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>1128</v>
+        <v>662</v>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:00.000Z</t>
+          <t>2026-07-10T05:25:49.000Z</t>
         </is>
       </c>
     </row>
@@ -3131,12 +3131,12 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>805</v>
+        <v>709</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:01.000Z</t>
+          <t>2026-07-10T05:25:50.000Z</t>
         </is>
       </c>
     </row>
@@ -3160,12 +3160,12 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>749</v>
+        <v>746</v>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:02.000Z</t>
+          <t>2026-07-10T05:25:50.000Z</t>
         </is>
       </c>
     </row>
@@ -3189,12 +3189,12 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>483</v>
+        <v>685</v>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:02.000Z</t>
+          <t>2026-07-10T05:25:51.000Z</t>
         </is>
       </c>
     </row>
@@ -3218,12 +3218,12 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>152</v>
+        <v>700</v>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:03.000Z</t>
+          <t>2026-07-10T05:25:52.000Z</t>
         </is>
       </c>
     </row>
@@ -3247,12 +3247,12 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>143</v>
+        <v>798</v>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:04.000Z</t>
+          <t>2026-07-10T05:25:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3276,12 +3276,12 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>879</v>
+        <v>963</v>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:05.000Z</t>
+          <t>2026-07-10T05:25:54.000Z</t>
         </is>
       </c>
     </row>
@@ -3305,12 +3305,12 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>176</v>
+        <v>1061</v>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:06.000Z</t>
+          <t>2026-07-10T05:25:54.000Z</t>
         </is>
       </c>
     </row>
@@ -3334,12 +3334,12 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>628</v>
+        <v>777</v>
       </c>
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:06.000Z</t>
+          <t>2026-07-10T05:25:55.000Z</t>
         </is>
       </c>
     </row>
@@ -3363,12 +3363,12 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>300</v>
+        <v>697</v>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:07.000Z</t>
+          <t>2026-07-10T05:25:56.000Z</t>
         </is>
       </c>
     </row>
@@ -3392,12 +3392,12 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>608</v>
+        <v>331</v>
       </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:08.000Z</t>
+          <t>2026-07-10T05:25:57.000Z</t>
         </is>
       </c>
     </row>
@@ -3421,12 +3421,12 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>1039</v>
+        <v>121</v>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:09.000Z</t>
+          <t>2026-07-10T05:25:58.000Z</t>
         </is>
       </c>
     </row>
@@ -3450,12 +3450,12 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>504</v>
+        <v>498</v>
       </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:10.000Z</t>
+          <t>2026-07-10T05:25:58.000Z</t>
         </is>
       </c>
     </row>
@@ -3479,12 +3479,12 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>741</v>
+        <v>597</v>
       </c>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:10.000Z</t>
+          <t>2026-07-10T05:25:59.000Z</t>
         </is>
       </c>
     </row>
@@ -3508,12 +3508,12 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>1006</v>
+        <v>336</v>
       </c>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:11.000Z</t>
+          <t>2026-07-10T05:26:00.000Z</t>
         </is>
       </c>
     </row>
@@ -3537,12 +3537,12 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>638</v>
+        <v>390</v>
       </c>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:12.000Z</t>
+          <t>2026-07-10T05:26:01.000Z</t>
         </is>
       </c>
     </row>
@@ -3566,12 +3566,12 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>143</v>
+        <v>781</v>
       </c>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:13.000Z</t>
+          <t>2026-07-10T05:26:02.000Z</t>
         </is>
       </c>
     </row>
@@ -3595,12 +3595,12 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>424</v>
+        <v>988</v>
       </c>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:14.000Z</t>
+          <t>2026-07-10T05:26:02.000Z</t>
         </is>
       </c>
     </row>
@@ -3624,12 +3624,12 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>610</v>
+        <v>575</v>
       </c>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:14.000Z</t>
+          <t>2026-07-10T05:26:03.000Z</t>
         </is>
       </c>
     </row>
@@ -3653,12 +3653,12 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:15.000Z</t>
+          <t>2026-07-10T05:26:04.000Z</t>
         </is>
       </c>
     </row>
@@ -3682,12 +3682,12 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>416</v>
+        <v>318</v>
       </c>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:16.000Z</t>
+          <t>2026-07-10T05:26:05.000Z</t>
         </is>
       </c>
     </row>
@@ -3711,12 +3711,12 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>445</v>
+        <v>347</v>
       </c>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:17.000Z</t>
+          <t>2026-07-10T05:26:06.000Z</t>
         </is>
       </c>
     </row>
@@ -3740,12 +3740,12 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>410</v>
+        <v>177</v>
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:18.000Z</t>
+          <t>2026-07-10T05:26:06.000Z</t>
         </is>
       </c>
     </row>
@@ -3769,12 +3769,12 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>1150</v>
+        <v>681</v>
       </c>
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:18.000Z</t>
+          <t>2026-07-10T05:26:07.000Z</t>
         </is>
       </c>
     </row>
@@ -3798,12 +3798,12 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>699</v>
+        <v>478</v>
       </c>
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:19.000Z</t>
+          <t>2026-07-10T05:26:08.000Z</t>
         </is>
       </c>
     </row>
@@ -3827,12 +3827,12 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>511</v>
+        <v>269</v>
       </c>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:20.000Z</t>
+          <t>2026-07-10T05:26:09.000Z</t>
         </is>
       </c>
     </row>
@@ -3856,12 +3856,12 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>1029</v>
+        <v>773</v>
       </c>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:21.000Z</t>
+          <t>2026-07-10T05:26:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3885,12 +3885,12 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>389</v>
+        <v>197</v>
       </c>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:22.000Z</t>
+          <t>2026-07-10T05:26:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3914,12 +3914,12 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>289</v>
+        <v>789</v>
       </c>
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:22.000Z</t>
+          <t>2026-07-10T05:26:11.000Z</t>
         </is>
       </c>
     </row>
@@ -3943,12 +3943,12 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>727</v>
+        <v>216</v>
       </c>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:23.000Z</t>
+          <t>2026-07-10T05:26:12.000Z</t>
         </is>
       </c>
     </row>
@@ -3972,12 +3972,12 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>204</v>
+        <v>1000</v>
       </c>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:24.000Z</t>
+          <t>2026-07-10T05:26:13.000Z</t>
         </is>
       </c>
     </row>
@@ -4001,12 +4001,12 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>1054</v>
+        <v>586</v>
       </c>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:25.000Z</t>
+          <t>2026-07-10T05:26:14.000Z</t>
         </is>
       </c>
     </row>
@@ -4030,12 +4030,12 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>410</v>
+        <v>688</v>
       </c>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:26.000Z</t>
+          <t>2026-07-10T05:26:14.000Z</t>
         </is>
       </c>
     </row>
@@ -4059,12 +4059,12 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>1144</v>
+        <v>1074</v>
       </c>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:26.000Z</t>
+          <t>2026-07-10T05:26:15.000Z</t>
         </is>
       </c>
     </row>
@@ -4088,12 +4088,12 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>997</v>
+        <v>815</v>
       </c>
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:27.000Z</t>
+          <t>2026-07-10T05:26:16.000Z</t>
         </is>
       </c>
     </row>
@@ -4117,12 +4117,12 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>414</v>
+        <v>1051</v>
       </c>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:28.000Z</t>
+          <t>2026-07-10T05:26:17.000Z</t>
         </is>
       </c>
     </row>
@@ -4146,12 +4146,12 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>191</v>
+        <v>939</v>
       </c>
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:29.000Z</t>
+          <t>2026-07-10T05:26:18.000Z</t>
         </is>
       </c>
     </row>
@@ -4175,12 +4175,12 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>307</v>
+        <v>524</v>
       </c>
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:30.000Z</t>
+          <t>2026-07-10T05:26:18.000Z</t>
         </is>
       </c>
     </row>
@@ -4204,12 +4204,12 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>323</v>
+        <v>238</v>
       </c>
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:30.000Z</t>
+          <t>2026-07-10T05:26:19.000Z</t>
         </is>
       </c>
     </row>
@@ -4233,12 +4233,12 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>257</v>
+        <v>501</v>
       </c>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:31.000Z</t>
+          <t>2026-07-10T05:26:20.000Z</t>
         </is>
       </c>
     </row>
@@ -4262,12 +4262,12 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>477</v>
+        <v>536</v>
       </c>
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:32.000Z</t>
+          <t>2026-07-10T05:26:21.000Z</t>
         </is>
       </c>
     </row>
@@ -4291,12 +4291,12 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>672</v>
+        <v>424</v>
       </c>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:33.000Z</t>
+          <t>2026-07-10T05:26:22.000Z</t>
         </is>
       </c>
     </row>
@@ -4320,12 +4320,12 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>899</v>
+        <v>866</v>
       </c>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:34.000Z</t>
+          <t>2026-07-10T05:26:22.000Z</t>
         </is>
       </c>
     </row>
@@ -4349,12 +4349,12 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>151</v>
+        <v>394</v>
       </c>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:34.000Z</t>
+          <t>2026-07-10T05:26:23.000Z</t>
         </is>
       </c>
     </row>
@@ -4378,12 +4378,12 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>1033</v>
+        <v>123</v>
       </c>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:35.000Z</t>
+          <t>2026-07-10T05:26:24.000Z</t>
         </is>
       </c>
     </row>
@@ -4407,12 +4407,12 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>390</v>
+        <v>774</v>
       </c>
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:36.000Z</t>
+          <t>2026-07-10T05:26:25.000Z</t>
         </is>
       </c>
     </row>
@@ -4436,12 +4436,12 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>423</v>
+        <v>383</v>
       </c>
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:37.000Z</t>
+          <t>2026-07-10T05:26:26.000Z</t>
         </is>
       </c>
     </row>
@@ -4465,12 +4465,12 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>803</v>
+        <v>1071</v>
       </c>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:38.000Z</t>
+          <t>2026-07-10T05:26:26.000Z</t>
         </is>
       </c>
     </row>
@@ -4494,12 +4494,12 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>940</v>
+        <v>902</v>
       </c>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:38.000Z</t>
+          <t>2026-07-10T05:26:27.000Z</t>
         </is>
       </c>
     </row>
@@ -4523,12 +4523,12 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>523</v>
+        <v>926</v>
       </c>
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:39.000Z</t>
+          <t>2026-07-10T05:26:28.000Z</t>
         </is>
       </c>
     </row>
@@ -4552,12 +4552,12 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>1060</v>
+        <v>997</v>
       </c>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:40.000Z</t>
+          <t>2026-07-10T05:26:29.000Z</t>
         </is>
       </c>
     </row>
@@ -4581,12 +4581,12 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>664</v>
+        <v>178</v>
       </c>
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:41.000Z</t>
+          <t>2026-07-10T05:26:30.000Z</t>
         </is>
       </c>
     </row>
@@ -4610,12 +4610,12 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>506</v>
+        <v>758</v>
       </c>
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:42.000Z</t>
+          <t>2026-07-10T05:26:30.000Z</t>
         </is>
       </c>
     </row>
@@ -4639,12 +4639,12 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>634</v>
+        <v>223</v>
       </c>
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:42.000Z</t>
+          <t>2026-07-10T05:26:31.000Z</t>
         </is>
       </c>
     </row>
@@ -4668,12 +4668,12 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>702</v>
+        <v>249</v>
       </c>
       <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:43.000Z</t>
+          <t>2026-07-10T05:26:32.000Z</t>
         </is>
       </c>
     </row>
@@ -4697,12 +4697,12 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>1082</v>
+        <v>1052</v>
       </c>
       <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:44.000Z</t>
+          <t>2026-07-10T05:26:33.000Z</t>
         </is>
       </c>
     </row>
@@ -4726,12 +4726,12 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>1174</v>
+        <v>712</v>
       </c>
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:45.000Z</t>
+          <t>2026-07-10T05:26:34.000Z</t>
         </is>
       </c>
     </row>
@@ -4755,12 +4755,12 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>576</v>
+        <v>590</v>
       </c>
       <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:46.000Z</t>
+          <t>2026-07-10T05:26:34.000Z</t>
         </is>
       </c>
     </row>
@@ -4784,12 +4784,12 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>284</v>
+        <v>977</v>
       </c>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:46.000Z</t>
+          <t>2026-07-10T05:26:35.000Z</t>
         </is>
       </c>
     </row>
@@ -4813,12 +4813,12 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>764</v>
+        <v>585</v>
       </c>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:47.000Z</t>
+          <t>2026-07-10T05:26:36.000Z</t>
         </is>
       </c>
     </row>
@@ -4842,12 +4842,12 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>635</v>
+        <v>801</v>
       </c>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:48.000Z</t>
+          <t>2026-07-10T05:26:37.000Z</t>
         </is>
       </c>
     </row>
@@ -4871,12 +4871,12 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>1048</v>
+        <v>1033</v>
       </c>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:49.000Z</t>
+          <t>2026-07-10T05:26:38.000Z</t>
         </is>
       </c>
     </row>
@@ -4900,12 +4900,12 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>562</v>
+        <v>1170</v>
       </c>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:50.000Z</t>
+          <t>2026-07-10T05:26:38.000Z</t>
         </is>
       </c>
     </row>
@@ -4929,12 +4929,12 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>332</v>
+        <v>526</v>
       </c>
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:50.000Z</t>
+          <t>2026-07-10T05:26:39.000Z</t>
         </is>
       </c>
     </row>
@@ -4958,12 +4958,12 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>1199</v>
+        <v>119</v>
       </c>
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:51.000Z</t>
+          <t>2026-07-10T05:26:40.000Z</t>
         </is>
       </c>
     </row>
@@ -4987,12 +4987,12 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>977</v>
+        <v>1048</v>
       </c>
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:52.000Z</t>
+          <t>2026-07-10T05:26:41.000Z</t>
         </is>
       </c>
     </row>
@@ -5016,12 +5016,12 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>659</v>
+        <v>613</v>
       </c>
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:53.000Z</t>
+          <t>2026-07-10T05:26:42.000Z</t>
         </is>
       </c>
     </row>
@@ -5045,12 +5045,12 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>431</v>
+        <v>721</v>
       </c>
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:54.000Z</t>
+          <t>2026-07-10T05:26:42.000Z</t>
         </is>
       </c>
     </row>
@@ -5074,12 +5074,12 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>471</v>
+        <v>967</v>
       </c>
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:54.000Z</t>
+          <t>2026-07-10T05:26:43.000Z</t>
         </is>
       </c>
     </row>
@@ -5103,12 +5103,12 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>570</v>
+        <v>906</v>
       </c>
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:55.000Z</t>
+          <t>2026-07-10T05:26:44.000Z</t>
         </is>
       </c>
     </row>
@@ -5132,12 +5132,12 @@
         </is>
       </c>
       <c r="E161" t="n">
-        <v>857</v>
+        <v>293</v>
       </c>
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:56.000Z</t>
+          <t>2026-07-10T05:26:45.000Z</t>
         </is>
       </c>
     </row>
@@ -5161,12 +5161,12 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>224</v>
+        <v>1114</v>
       </c>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:57.000Z</t>
+          <t>2026-07-10T05:26:46.000Z</t>
         </is>
       </c>
     </row>
@@ -5190,12 +5190,12 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>898</v>
+        <v>1112</v>
       </c>
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:58.000Z</t>
+          <t>2026-07-10T05:26:46.000Z</t>
         </is>
       </c>
     </row>
@@ -5219,12 +5219,12 @@
         </is>
       </c>
       <c r="E164" t="n">
-        <v>347</v>
+        <v>1049</v>
       </c>
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:58.000Z</t>
+          <t>2026-07-10T05:26:47.000Z</t>
         </is>
       </c>
     </row>
@@ -5248,12 +5248,12 @@
         </is>
       </c>
       <c r="E165" t="n">
-        <v>415</v>
+        <v>1166</v>
       </c>
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>2026-07-10T04:55:59.000Z</t>
+          <t>2026-07-10T05:26:48.000Z</t>
         </is>
       </c>
     </row>
@@ -5277,12 +5277,12 @@
         </is>
       </c>
       <c r="E166" t="n">
-        <v>394</v>
+        <v>248</v>
       </c>
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:00.000Z</t>
+          <t>2026-07-10T05:26:49.000Z</t>
         </is>
       </c>
     </row>
@@ -5306,12 +5306,12 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>931</v>
+        <v>618</v>
       </c>
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:01.000Z</t>
+          <t>2026-07-10T05:26:50.000Z</t>
         </is>
       </c>
     </row>
@@ -5335,12 +5335,12 @@
         </is>
       </c>
       <c r="E168" t="n">
-        <v>335</v>
+        <v>1199</v>
       </c>
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:02.000Z</t>
+          <t>2026-07-10T05:26:50.000Z</t>
         </is>
       </c>
     </row>
@@ -5364,12 +5364,12 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>609</v>
+        <v>660</v>
       </c>
       <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:02.000Z</t>
+          <t>2026-07-10T05:26:51.000Z</t>
         </is>
       </c>
     </row>
@@ -5393,12 +5393,12 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>1164</v>
+        <v>110</v>
       </c>
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:03.000Z</t>
+          <t>2026-07-10T05:26:52.000Z</t>
         </is>
       </c>
     </row>
@@ -5422,12 +5422,12 @@
         </is>
       </c>
       <c r="E171" t="n">
-        <v>760</v>
+        <v>514</v>
       </c>
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:04.000Z</t>
+          <t>2026-07-10T05:26:53.000Z</t>
         </is>
       </c>
     </row>
@@ -5451,12 +5451,12 @@
         </is>
       </c>
       <c r="E172" t="n">
-        <v>634</v>
+        <v>395</v>
       </c>
       <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:05.000Z</t>
+          <t>2026-07-10T05:26:54.000Z</t>
         </is>
       </c>
     </row>
@@ -5480,12 +5480,12 @@
         </is>
       </c>
       <c r="E173" t="n">
-        <v>740</v>
+        <v>1055</v>
       </c>
       <c r="F173" t="inlineStr"/>
       <c r="G173" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:06.000Z</t>
+          <t>2026-07-10T05:26:54.000Z</t>
         </is>
       </c>
     </row>
@@ -5509,12 +5509,12 @@
         </is>
       </c>
       <c r="E174" t="n">
-        <v>669</v>
+        <v>664</v>
       </c>
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:06.000Z</t>
+          <t>2026-07-10T05:26:55.000Z</t>
         </is>
       </c>
     </row>
@@ -5538,12 +5538,12 @@
         </is>
       </c>
       <c r="E175" t="n">
-        <v>1013</v>
+        <v>1198</v>
       </c>
       <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:07.000Z</t>
+          <t>2026-07-10T05:26:56.000Z</t>
         </is>
       </c>
     </row>
@@ -5567,12 +5567,12 @@
         </is>
       </c>
       <c r="E176" t="n">
-        <v>150</v>
+        <v>351</v>
       </c>
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:08.000Z</t>
+          <t>2026-07-10T05:26:57.000Z</t>
         </is>
       </c>
     </row>
@@ -5596,12 +5596,12 @@
         </is>
       </c>
       <c r="E177" t="n">
-        <v>583</v>
+        <v>270</v>
       </c>
       <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:09.000Z</t>
+          <t>2026-07-10T05:26:58.000Z</t>
         </is>
       </c>
     </row>
@@ -5625,12 +5625,12 @@
         </is>
       </c>
       <c r="E178" t="n">
-        <v>1136</v>
+        <v>253</v>
       </c>
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:10.000Z</t>
+          <t>2026-07-10T05:26:58.000Z</t>
         </is>
       </c>
     </row>
@@ -5654,12 +5654,12 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>1085</v>
+        <v>741</v>
       </c>
       <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:10.000Z</t>
+          <t>2026-07-10T05:26:59.000Z</t>
         </is>
       </c>
     </row>
@@ -5683,12 +5683,12 @@
         </is>
       </c>
       <c r="E180" t="n">
-        <v>630</v>
+        <v>785</v>
       </c>
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:11.000Z</t>
+          <t>2026-07-10T05:27:00.000Z</t>
         </is>
       </c>
     </row>
@@ -5712,12 +5712,12 @@
         </is>
       </c>
       <c r="E181" t="n">
-        <v>201</v>
+        <v>334</v>
       </c>
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:12.000Z</t>
+          <t>2026-07-10T05:27:01.000Z</t>
         </is>
       </c>
     </row>
@@ -5741,12 +5741,12 @@
         </is>
       </c>
       <c r="E182" t="n">
-        <v>460</v>
+        <v>526</v>
       </c>
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:13.000Z</t>
+          <t>2026-07-10T05:27:02.000Z</t>
         </is>
       </c>
     </row>
@@ -5770,12 +5770,12 @@
         </is>
       </c>
       <c r="E183" t="n">
-        <v>695</v>
+        <v>653</v>
       </c>
       <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:14.000Z</t>
+          <t>2026-07-10T05:27:02.000Z</t>
         </is>
       </c>
     </row>
@@ -5799,12 +5799,12 @@
         </is>
       </c>
       <c r="E184" t="n">
-        <v>877</v>
+        <v>576</v>
       </c>
       <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:14.000Z</t>
+          <t>2026-07-10T05:27:03.000Z</t>
         </is>
       </c>
     </row>
@@ -5828,12 +5828,12 @@
         </is>
       </c>
       <c r="E185" t="n">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:15.000Z</t>
+          <t>2026-07-10T05:27:04.000Z</t>
         </is>
       </c>
     </row>
@@ -5857,12 +5857,12 @@
         </is>
       </c>
       <c r="E186" t="n">
-        <v>364</v>
+        <v>776</v>
       </c>
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:16.000Z</t>
+          <t>2026-07-10T05:27:05.000Z</t>
         </is>
       </c>
     </row>
@@ -5886,12 +5886,12 @@
         </is>
       </c>
       <c r="E187" t="n">
-        <v>141</v>
+        <v>632</v>
       </c>
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:17.000Z</t>
+          <t>2026-07-10T05:27:06.000Z</t>
         </is>
       </c>
     </row>
@@ -5915,12 +5915,12 @@
         </is>
       </c>
       <c r="E188" t="n">
-        <v>645</v>
+        <v>199</v>
       </c>
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:18.000Z</t>
+          <t>2026-07-10T05:27:06.000Z</t>
         </is>
       </c>
     </row>
@@ -5944,12 +5944,12 @@
         </is>
       </c>
       <c r="E189" t="n">
-        <v>617</v>
+        <v>633</v>
       </c>
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:18.000Z</t>
+          <t>2026-07-10T05:27:07.000Z</t>
         </is>
       </c>
     </row>
@@ -5973,12 +5973,12 @@
         </is>
       </c>
       <c r="E190" t="n">
-        <v>459</v>
+        <v>684</v>
       </c>
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:19.000Z</t>
+          <t>2026-07-10T05:27:08.000Z</t>
         </is>
       </c>
     </row>
@@ -6002,12 +6002,12 @@
         </is>
       </c>
       <c r="E191" t="n">
-        <v>225</v>
+        <v>611</v>
       </c>
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:20.000Z</t>
+          <t>2026-07-10T05:27:09.000Z</t>
         </is>
       </c>
     </row>
@@ -6031,12 +6031,12 @@
         </is>
       </c>
       <c r="E192" t="n">
-        <v>1037</v>
+        <v>1084</v>
       </c>
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:21.000Z</t>
+          <t>2026-07-10T05:27:10.000Z</t>
         </is>
       </c>
     </row>
@@ -6060,12 +6060,12 @@
         </is>
       </c>
       <c r="E193" t="n">
-        <v>865</v>
+        <v>487</v>
       </c>
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:22.000Z</t>
+          <t>2026-07-10T05:27:10.000Z</t>
         </is>
       </c>
     </row>
@@ -6089,12 +6089,12 @@
         </is>
       </c>
       <c r="E194" t="n">
-        <v>864</v>
+        <v>161</v>
       </c>
       <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:22.000Z</t>
+          <t>2026-07-10T05:27:11.000Z</t>
         </is>
       </c>
     </row>
@@ -6118,12 +6118,12 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>1076</v>
+        <v>854</v>
       </c>
       <c r="F195" t="inlineStr"/>
       <c r="G195" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:23.000Z</t>
+          <t>2026-07-10T05:27:12.000Z</t>
         </is>
       </c>
     </row>
@@ -6147,12 +6147,12 @@
         </is>
       </c>
       <c r="E196" t="n">
-        <v>793</v>
+        <v>607</v>
       </c>
       <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:24.000Z</t>
+          <t>2026-07-10T05:27:13.000Z</t>
         </is>
       </c>
     </row>
@@ -6176,12 +6176,12 @@
         </is>
       </c>
       <c r="E197" t="n">
-        <v>750</v>
+        <v>624</v>
       </c>
       <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:25.000Z</t>
+          <t>2026-07-10T05:27:14.000Z</t>
         </is>
       </c>
     </row>
@@ -6205,12 +6205,12 @@
         </is>
       </c>
       <c r="E198" t="n">
-        <v>943</v>
+        <v>562</v>
       </c>
       <c r="F198" t="inlineStr"/>
       <c r="G198" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:26.000Z</t>
+          <t>2026-07-10T05:27:14.000Z</t>
         </is>
       </c>
     </row>
@@ -6234,12 +6234,12 @@
         </is>
       </c>
       <c r="E199" t="n">
-        <v>666</v>
+        <v>787</v>
       </c>
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:26.000Z</t>
+          <t>2026-07-10T05:27:15.000Z</t>
         </is>
       </c>
     </row>
@@ -6263,12 +6263,12 @@
         </is>
       </c>
       <c r="E200" t="n">
-        <v>618</v>
+        <v>419</v>
       </c>
       <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:27.000Z</t>
+          <t>2026-07-10T05:27:16.000Z</t>
         </is>
       </c>
     </row>
@@ -6292,12 +6292,12 @@
         </is>
       </c>
       <c r="E201" t="n">
-        <v>436</v>
+        <v>719</v>
       </c>
       <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:28.000Z</t>
+          <t>2026-07-10T05:27:17.000Z</t>
         </is>
       </c>
     </row>
@@ -6321,12 +6321,12 @@
         </is>
       </c>
       <c r="E202" t="n">
-        <v>926</v>
+        <v>315</v>
       </c>
       <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:29.000Z</t>
+          <t>2026-07-10T05:27:18.000Z</t>
         </is>
       </c>
     </row>
@@ -6350,12 +6350,12 @@
         </is>
       </c>
       <c r="E203" t="n">
-        <v>214</v>
+        <v>315</v>
       </c>
       <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:30.000Z</t>
+          <t>2026-07-10T05:27:18.000Z</t>
         </is>
       </c>
     </row>
@@ -6379,12 +6379,12 @@
         </is>
       </c>
       <c r="E204" t="n">
-        <v>570</v>
+        <v>664</v>
       </c>
       <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:30.000Z</t>
+          <t>2026-07-10T05:27:19.000Z</t>
         </is>
       </c>
     </row>
@@ -6408,12 +6408,12 @@
         </is>
       </c>
       <c r="E205" t="n">
-        <v>1043</v>
+        <v>393</v>
       </c>
       <c r="F205" t="inlineStr"/>
       <c r="G205" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:31.000Z</t>
+          <t>2026-07-10T05:27:20.000Z</t>
         </is>
       </c>
     </row>
@@ -6437,12 +6437,12 @@
         </is>
       </c>
       <c r="E206" t="n">
-        <v>872</v>
+        <v>574</v>
       </c>
       <c r="F206" t="inlineStr"/>
       <c r="G206" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:32.000Z</t>
+          <t>2026-07-10T05:27:21.000Z</t>
         </is>
       </c>
     </row>
@@ -6466,12 +6466,12 @@
         </is>
       </c>
       <c r="E207" t="n">
-        <v>120</v>
+        <v>1007</v>
       </c>
       <c r="F207" t="inlineStr"/>
       <c r="G207" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:33.000Z</t>
+          <t>2026-07-10T05:27:22.000Z</t>
         </is>
       </c>
     </row>
@@ -6495,12 +6495,12 @@
         </is>
       </c>
       <c r="E208" t="n">
-        <v>1104</v>
+        <v>476</v>
       </c>
       <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:34.000Z</t>
+          <t>2026-07-10T05:27:22.000Z</t>
         </is>
       </c>
     </row>
@@ -6524,12 +6524,12 @@
         </is>
       </c>
       <c r="E209" t="n">
-        <v>244</v>
+        <v>533</v>
       </c>
       <c r="F209" t="inlineStr"/>
       <c r="G209" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:34.000Z</t>
+          <t>2026-07-10T05:27:23.000Z</t>
         </is>
       </c>
     </row>
@@ -6553,12 +6553,12 @@
         </is>
       </c>
       <c r="E210" t="n">
-        <v>906</v>
+        <v>664</v>
       </c>
       <c r="F210" t="inlineStr"/>
       <c r="G210" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:35.000Z</t>
+          <t>2026-07-10T05:27:24.000Z</t>
         </is>
       </c>
     </row>
@@ -6582,12 +6582,12 @@
         </is>
       </c>
       <c r="E211" t="n">
-        <v>961</v>
+        <v>585</v>
       </c>
       <c r="F211" t="inlineStr"/>
       <c r="G211" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:36.000Z</t>
+          <t>2026-07-10T05:27:25.000Z</t>
         </is>
       </c>
     </row>
@@ -6611,12 +6611,12 @@
         </is>
       </c>
       <c r="E212" t="n">
-        <v>801</v>
+        <v>337</v>
       </c>
       <c r="F212" t="inlineStr"/>
       <c r="G212" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:37.000Z</t>
+          <t>2026-07-10T05:27:26.000Z</t>
         </is>
       </c>
     </row>
@@ -6640,12 +6640,12 @@
         </is>
       </c>
       <c r="E213" t="n">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="F213" t="inlineStr"/>
       <c r="G213" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:38.000Z</t>
+          <t>2026-07-10T05:27:26.000Z</t>
         </is>
       </c>
     </row>
@@ -6669,12 +6669,12 @@
         </is>
       </c>
       <c r="E214" t="n">
-        <v>662</v>
+        <v>1174</v>
       </c>
       <c r="F214" t="inlineStr"/>
       <c r="G214" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:38.000Z</t>
+          <t>2026-07-10T05:27:27.000Z</t>
         </is>
       </c>
     </row>
@@ -6698,12 +6698,12 @@
         </is>
       </c>
       <c r="E215" t="n">
-        <v>269</v>
+        <v>1116</v>
       </c>
       <c r="F215" t="inlineStr"/>
       <c r="G215" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:39.000Z</t>
+          <t>2026-07-10T05:27:28.000Z</t>
         </is>
       </c>
     </row>
@@ -6727,12 +6727,12 @@
         </is>
       </c>
       <c r="E216" t="n">
-        <v>107</v>
+        <v>1042</v>
       </c>
       <c r="F216" t="inlineStr"/>
       <c r="G216" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:40.000Z</t>
+          <t>2026-07-10T05:27:29.000Z</t>
         </is>
       </c>
     </row>
@@ -6756,12 +6756,12 @@
         </is>
       </c>
       <c r="E217" t="n">
-        <v>206</v>
+        <v>502</v>
       </c>
       <c r="F217" t="inlineStr"/>
       <c r="G217" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:41.000Z</t>
+          <t>2026-07-10T05:27:30.000Z</t>
         </is>
       </c>
     </row>
@@ -6785,12 +6785,12 @@
         </is>
       </c>
       <c r="E218" t="n">
-        <v>787</v>
+        <v>959</v>
       </c>
       <c r="F218" t="inlineStr"/>
       <c r="G218" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:42.000Z</t>
+          <t>2026-07-10T05:27:30.000Z</t>
         </is>
       </c>
     </row>
@@ -6814,12 +6814,12 @@
         </is>
       </c>
       <c r="E219" t="n">
-        <v>471</v>
+        <v>513</v>
       </c>
       <c r="F219" t="inlineStr"/>
       <c r="G219" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:42.000Z</t>
+          <t>2026-07-10T05:27:31.000Z</t>
         </is>
       </c>
     </row>
@@ -6843,12 +6843,12 @@
         </is>
       </c>
       <c r="E220" t="n">
-        <v>1088</v>
+        <v>208</v>
       </c>
       <c r="F220" t="inlineStr"/>
       <c r="G220" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:43.000Z</t>
+          <t>2026-07-10T05:27:32.000Z</t>
         </is>
       </c>
     </row>
@@ -6872,12 +6872,12 @@
         </is>
       </c>
       <c r="E221" t="n">
-        <v>1054</v>
+        <v>754</v>
       </c>
       <c r="F221" t="inlineStr"/>
       <c r="G221" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:44.000Z</t>
+          <t>2026-07-10T05:27:33.000Z</t>
         </is>
       </c>
     </row>
@@ -6901,12 +6901,12 @@
         </is>
       </c>
       <c r="E222" t="n">
-        <v>189</v>
+        <v>1064</v>
       </c>
       <c r="F222" t="inlineStr"/>
       <c r="G222" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:45.000Z</t>
+          <t>2026-07-10T05:27:34.000Z</t>
         </is>
       </c>
     </row>
@@ -6930,12 +6930,12 @@
         </is>
       </c>
       <c r="E223" t="n">
-        <v>1156</v>
+        <v>443</v>
       </c>
       <c r="F223" t="inlineStr"/>
       <c r="G223" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:46.000Z</t>
+          <t>2026-07-10T05:27:34.000Z</t>
         </is>
       </c>
     </row>
@@ -6959,12 +6959,12 @@
         </is>
       </c>
       <c r="E224" t="n">
-        <v>890</v>
+        <v>748</v>
       </c>
       <c r="F224" t="inlineStr"/>
       <c r="G224" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:46.000Z</t>
+          <t>2026-07-10T05:27:35.000Z</t>
         </is>
       </c>
     </row>
@@ -6988,12 +6988,12 @@
         </is>
       </c>
       <c r="E225" t="n">
-        <v>745</v>
+        <v>111</v>
       </c>
       <c r="F225" t="inlineStr"/>
       <c r="G225" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:47.000Z</t>
+          <t>2026-07-10T05:27:36.000Z</t>
         </is>
       </c>
     </row>
@@ -7017,12 +7017,12 @@
         </is>
       </c>
       <c r="E226" t="n">
-        <v>542</v>
+        <v>1187</v>
       </c>
       <c r="F226" t="inlineStr"/>
       <c r="G226" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:48.000Z</t>
+          <t>2026-07-10T05:27:37.000Z</t>
         </is>
       </c>
     </row>
@@ -7046,12 +7046,12 @@
         </is>
       </c>
       <c r="E227" t="n">
-        <v>420</v>
+        <v>1043</v>
       </c>
       <c r="F227" t="inlineStr"/>
       <c r="G227" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:49.000Z</t>
+          <t>2026-07-10T05:27:38.000Z</t>
         </is>
       </c>
     </row>
@@ -7075,12 +7075,12 @@
         </is>
       </c>
       <c r="E228" t="n">
-        <v>773</v>
+        <v>590</v>
       </c>
       <c r="F228" t="inlineStr"/>
       <c r="G228" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:50.000Z</t>
+          <t>2026-07-10T05:27:38.000Z</t>
         </is>
       </c>
     </row>
@@ -7104,12 +7104,12 @@
         </is>
       </c>
       <c r="E229" t="n">
-        <v>108</v>
+        <v>1073</v>
       </c>
       <c r="F229" t="inlineStr"/>
       <c r="G229" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:50.000Z</t>
+          <t>2026-07-10T05:27:39.000Z</t>
         </is>
       </c>
     </row>
@@ -7133,12 +7133,12 @@
         </is>
       </c>
       <c r="E230" t="n">
-        <v>1040</v>
+        <v>224</v>
       </c>
       <c r="F230" t="inlineStr"/>
       <c r="G230" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:51.000Z</t>
+          <t>2026-07-10T05:27:40.000Z</t>
         </is>
       </c>
     </row>
@@ -7162,12 +7162,12 @@
         </is>
       </c>
       <c r="E231" t="n">
-        <v>404</v>
+        <v>956</v>
       </c>
       <c r="F231" t="inlineStr"/>
       <c r="G231" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:52.000Z</t>
+          <t>2026-07-10T05:27:41.000Z</t>
         </is>
       </c>
     </row>
@@ -7191,12 +7191,12 @@
         </is>
       </c>
       <c r="E232" t="n">
-        <v>929</v>
+        <v>553</v>
       </c>
       <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:53.000Z</t>
+          <t>2026-07-10T05:27:42.000Z</t>
         </is>
       </c>
     </row>
@@ -7220,12 +7220,12 @@
         </is>
       </c>
       <c r="E233" t="n">
-        <v>881</v>
+        <v>930</v>
       </c>
       <c r="F233" t="inlineStr"/>
       <c r="G233" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:54.000Z</t>
+          <t>2026-07-10T05:27:42.000Z</t>
         </is>
       </c>
     </row>
@@ -7249,12 +7249,12 @@
         </is>
       </c>
       <c r="E234" t="n">
-        <v>1079</v>
+        <v>661</v>
       </c>
       <c r="F234" t="inlineStr"/>
       <c r="G234" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:54.000Z</t>
+          <t>2026-07-10T05:27:43.000Z</t>
         </is>
       </c>
     </row>
@@ -7278,12 +7278,12 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>248</v>
+        <v>821</v>
       </c>
       <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:55.000Z</t>
+          <t>2026-07-10T05:27:44.000Z</t>
         </is>
       </c>
     </row>
@@ -7307,12 +7307,12 @@
         </is>
       </c>
       <c r="E236" t="n">
-        <v>416</v>
+        <v>333</v>
       </c>
       <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:56.000Z</t>
+          <t>2026-07-10T05:27:45.000Z</t>
         </is>
       </c>
     </row>
@@ -7336,12 +7336,12 @@
         </is>
       </c>
       <c r="E237" t="n">
-        <v>754</v>
+        <v>586</v>
       </c>
       <c r="F237" t="inlineStr"/>
       <c r="G237" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:57.000Z</t>
+          <t>2026-07-10T05:27:46.000Z</t>
         </is>
       </c>
     </row>
@@ -7365,12 +7365,12 @@
         </is>
       </c>
       <c r="E238" t="n">
-        <v>165</v>
+        <v>234</v>
       </c>
       <c r="F238" t="inlineStr"/>
       <c r="G238" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:58.000Z</t>
+          <t>2026-07-10T05:27:46.000Z</t>
         </is>
       </c>
     </row>
@@ -7394,12 +7394,12 @@
         </is>
       </c>
       <c r="E239" t="n">
-        <v>97</v>
+        <v>498</v>
       </c>
       <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:58.000Z</t>
+          <t>2026-07-10T05:27:47.000Z</t>
         </is>
       </c>
     </row>
@@ -7423,12 +7423,12 @@
         </is>
       </c>
       <c r="E240" t="n">
-        <v>297</v>
+        <v>279</v>
       </c>
       <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
-          <t>2026-07-10T04:56:59.000Z</t>
+          <t>2026-07-10T05:27:48.000Z</t>
         </is>
       </c>
     </row>
@@ -7452,12 +7452,12 @@
         </is>
       </c>
       <c r="E241" t="n">
-        <v>124</v>
+        <v>872</v>
       </c>
       <c r="F241" t="inlineStr"/>
       <c r="G241" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:00.000Z</t>
+          <t>2026-07-10T05:27:49.000Z</t>
         </is>
       </c>
     </row>
@@ -7481,12 +7481,12 @@
         </is>
       </c>
       <c r="E242" t="n">
-        <v>1177</v>
+        <v>923</v>
       </c>
       <c r="F242" t="inlineStr"/>
       <c r="G242" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:01.000Z</t>
+          <t>2026-07-10T05:27:50.000Z</t>
         </is>
       </c>
     </row>
@@ -7510,12 +7510,12 @@
         </is>
       </c>
       <c r="E243" t="n">
-        <v>789</v>
+        <v>122</v>
       </c>
       <c r="F243" t="inlineStr"/>
       <c r="G243" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:02.000Z</t>
+          <t>2026-07-10T05:27:50.000Z</t>
         </is>
       </c>
     </row>
@@ -7539,12 +7539,12 @@
         </is>
       </c>
       <c r="E244" t="n">
-        <v>82</v>
+        <v>252</v>
       </c>
       <c r="F244" t="inlineStr"/>
       <c r="G244" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:02.000Z</t>
+          <t>2026-07-10T05:27:51.000Z</t>
         </is>
       </c>
     </row>
@@ -7568,12 +7568,12 @@
         </is>
       </c>
       <c r="E245" t="n">
-        <v>120</v>
+        <v>293</v>
       </c>
       <c r="F245" t="inlineStr"/>
       <c r="G245" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:03.000Z</t>
+          <t>2026-07-10T05:27:52.000Z</t>
         </is>
       </c>
     </row>
@@ -7597,12 +7597,12 @@
         </is>
       </c>
       <c r="E246" t="n">
-        <v>288</v>
+        <v>989</v>
       </c>
       <c r="F246" t="inlineStr"/>
       <c r="G246" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:04.000Z</t>
+          <t>2026-07-10T05:27:53.000Z</t>
         </is>
       </c>
     </row>
@@ -7626,12 +7626,12 @@
         </is>
       </c>
       <c r="E247" t="n">
-        <v>933</v>
+        <v>125</v>
       </c>
       <c r="F247" t="inlineStr"/>
       <c r="G247" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:05.000Z</t>
+          <t>2026-07-10T05:27:54.000Z</t>
         </is>
       </c>
     </row>
@@ -7655,12 +7655,12 @@
         </is>
       </c>
       <c r="E248" t="n">
-        <v>968</v>
+        <v>1039</v>
       </c>
       <c r="F248" t="inlineStr"/>
       <c r="G248" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:06.000Z</t>
+          <t>2026-07-10T05:27:54.000Z</t>
         </is>
       </c>
     </row>
@@ -7684,12 +7684,12 @@
         </is>
       </c>
       <c r="E249" t="n">
-        <v>377</v>
+        <v>604</v>
       </c>
       <c r="F249" t="inlineStr"/>
       <c r="G249" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:06.000Z</t>
+          <t>2026-07-10T05:27:55.000Z</t>
         </is>
       </c>
     </row>
@@ -7713,12 +7713,12 @@
         </is>
       </c>
       <c r="E250" t="n">
-        <v>831</v>
+        <v>109</v>
       </c>
       <c r="F250" t="inlineStr"/>
       <c r="G250" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:07.000Z</t>
+          <t>2026-07-10T05:27:56.000Z</t>
         </is>
       </c>
     </row>
@@ -7742,12 +7742,12 @@
         </is>
       </c>
       <c r="E251" t="n">
-        <v>803</v>
+        <v>460</v>
       </c>
       <c r="F251" t="inlineStr"/>
       <c r="G251" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:08.000Z</t>
+          <t>2026-07-10T05:27:57.000Z</t>
         </is>
       </c>
     </row>
@@ -7771,12 +7771,12 @@
         </is>
       </c>
       <c r="E252" t="n">
-        <v>539</v>
+        <v>971</v>
       </c>
       <c r="F252" t="inlineStr"/>
       <c r="G252" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:09.000Z</t>
+          <t>2026-07-10T05:27:58.000Z</t>
         </is>
       </c>
     </row>
@@ -7800,12 +7800,12 @@
         </is>
       </c>
       <c r="E253" t="n">
-        <v>1116</v>
+        <v>513</v>
       </c>
       <c r="F253" t="inlineStr"/>
       <c r="G253" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:10.000Z</t>
+          <t>2026-07-10T05:27:58.000Z</t>
         </is>
       </c>
     </row>
@@ -7829,12 +7829,12 @@
         </is>
       </c>
       <c r="E254" t="n">
-        <v>1056</v>
+        <v>477</v>
       </c>
       <c r="F254" t="inlineStr"/>
       <c r="G254" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:10.000Z</t>
+          <t>2026-07-10T05:27:59.000Z</t>
         </is>
       </c>
     </row>
@@ -7858,12 +7858,12 @@
         </is>
       </c>
       <c r="E255" t="n">
-        <v>107</v>
+        <v>523</v>
       </c>
       <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:11.000Z</t>
+          <t>2026-07-10T05:28:00.000Z</t>
         </is>
       </c>
     </row>
@@ -7887,12 +7887,12 @@
         </is>
       </c>
       <c r="E256" t="n">
-        <v>1073</v>
+        <v>945</v>
       </c>
       <c r="F256" t="inlineStr"/>
       <c r="G256" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:12.000Z</t>
+          <t>2026-07-10T05:28:01.000Z</t>
         </is>
       </c>
     </row>
@@ -7916,12 +7916,12 @@
         </is>
       </c>
       <c r="E257" t="n">
-        <v>541</v>
+        <v>778</v>
       </c>
       <c r="F257" t="inlineStr"/>
       <c r="G257" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:13.000Z</t>
+          <t>2026-07-10T05:28:02.000Z</t>
         </is>
       </c>
     </row>
@@ -7945,12 +7945,12 @@
         </is>
       </c>
       <c r="E258" t="n">
-        <v>949</v>
+        <v>427</v>
       </c>
       <c r="F258" t="inlineStr"/>
       <c r="G258" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:14.000Z</t>
+          <t>2026-07-10T05:28:02.000Z</t>
         </is>
       </c>
     </row>
@@ -7974,12 +7974,12 @@
         </is>
       </c>
       <c r="E259" t="n">
-        <v>91</v>
+        <v>956</v>
       </c>
       <c r="F259" t="inlineStr"/>
       <c r="G259" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:14.000Z</t>
+          <t>2026-07-10T05:28:03.000Z</t>
         </is>
       </c>
     </row>
@@ -8003,12 +8003,12 @@
         </is>
       </c>
       <c r="E260" t="n">
-        <v>461</v>
+        <v>121</v>
       </c>
       <c r="F260" t="inlineStr"/>
       <c r="G260" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:15.000Z</t>
+          <t>2026-07-10T05:28:04.000Z</t>
         </is>
       </c>
     </row>
@@ -8032,12 +8032,12 @@
         </is>
       </c>
       <c r="E261" t="n">
-        <v>488</v>
+        <v>1029</v>
       </c>
       <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:16.000Z</t>
+          <t>2026-07-10T05:28:05.000Z</t>
         </is>
       </c>
     </row>
@@ -8061,12 +8061,12 @@
         </is>
       </c>
       <c r="E262" t="n">
-        <v>782</v>
+        <v>716</v>
       </c>
       <c r="F262" t="inlineStr"/>
       <c r="G262" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:17.000Z</t>
+          <t>2026-07-10T05:28:06.000Z</t>
         </is>
       </c>
     </row>
@@ -8090,12 +8090,12 @@
         </is>
       </c>
       <c r="E263" t="n">
-        <v>863</v>
+        <v>157</v>
       </c>
       <c r="F263" t="inlineStr"/>
       <c r="G263" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:18.000Z</t>
+          <t>2026-07-10T05:28:06.000Z</t>
         </is>
       </c>
     </row>
@@ -8119,12 +8119,12 @@
         </is>
       </c>
       <c r="E264" t="n">
-        <v>445</v>
+        <v>1042</v>
       </c>
       <c r="F264" t="inlineStr"/>
       <c r="G264" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:18.000Z</t>
+          <t>2026-07-10T05:28:07.000Z</t>
         </is>
       </c>
     </row>
@@ -8148,12 +8148,12 @@
         </is>
       </c>
       <c r="E265" t="n">
-        <v>134</v>
+        <v>448</v>
       </c>
       <c r="F265" t="inlineStr"/>
       <c r="G265" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:19.000Z</t>
+          <t>2026-07-10T05:28:08.000Z</t>
         </is>
       </c>
     </row>
@@ -8177,12 +8177,12 @@
         </is>
       </c>
       <c r="E266" t="n">
-        <v>933</v>
+        <v>848</v>
       </c>
       <c r="F266" t="inlineStr"/>
       <c r="G266" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:20.000Z</t>
+          <t>2026-07-10T05:28:09.000Z</t>
         </is>
       </c>
     </row>
@@ -8206,12 +8206,12 @@
         </is>
       </c>
       <c r="E267" t="n">
-        <v>902</v>
+        <v>242</v>
       </c>
       <c r="F267" t="inlineStr"/>
       <c r="G267" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:21.000Z</t>
+          <t>2026-07-10T05:28:10.000Z</t>
         </is>
       </c>
     </row>
@@ -8235,12 +8235,12 @@
         </is>
       </c>
       <c r="E268" t="n">
-        <v>94</v>
+        <v>150</v>
       </c>
       <c r="F268" t="inlineStr"/>
       <c r="G268" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:22.000Z</t>
+          <t>2026-07-10T05:28:10.000Z</t>
         </is>
       </c>
     </row>
@@ -8264,12 +8264,12 @@
         </is>
       </c>
       <c r="E269" t="n">
-        <v>990</v>
+        <v>160</v>
       </c>
       <c r="F269" t="inlineStr"/>
       <c r="G269" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:22.000Z</t>
+          <t>2026-07-10T05:28:11.000Z</t>
         </is>
       </c>
     </row>
@@ -8293,12 +8293,12 @@
         </is>
       </c>
       <c r="E270" t="n">
-        <v>343</v>
+        <v>1023</v>
       </c>
       <c r="F270" t="inlineStr"/>
       <c r="G270" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:23.000Z</t>
+          <t>2026-07-10T05:28:12.000Z</t>
         </is>
       </c>
     </row>
@@ -8322,12 +8322,12 @@
         </is>
       </c>
       <c r="E271" t="n">
-        <v>333</v>
+        <v>714</v>
       </c>
       <c r="F271" t="inlineStr"/>
       <c r="G271" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:24.000Z</t>
+          <t>2026-07-10T05:28:13.000Z</t>
         </is>
       </c>
     </row>
@@ -8351,12 +8351,12 @@
         </is>
       </c>
       <c r="E272" t="n">
-        <v>905</v>
+        <v>532</v>
       </c>
       <c r="F272" t="inlineStr"/>
       <c r="G272" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:25.000Z</t>
+          <t>2026-07-10T05:28:14.000Z</t>
         </is>
       </c>
     </row>
@@ -8380,12 +8380,12 @@
         </is>
       </c>
       <c r="E273" t="n">
-        <v>891</v>
+        <v>658</v>
       </c>
       <c r="F273" t="inlineStr"/>
       <c r="G273" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:26.000Z</t>
+          <t>2026-07-10T05:28:14.000Z</t>
         </is>
       </c>
     </row>
@@ -8409,12 +8409,12 @@
         </is>
       </c>
       <c r="E274" t="n">
-        <v>329</v>
+        <v>732</v>
       </c>
       <c r="F274" t="inlineStr"/>
       <c r="G274" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:26.000Z</t>
+          <t>2026-07-10T05:28:15.000Z</t>
         </is>
       </c>
     </row>
@@ -8438,12 +8438,12 @@
         </is>
       </c>
       <c r="E275" t="n">
-        <v>242</v>
+        <v>380</v>
       </c>
       <c r="F275" t="inlineStr"/>
       <c r="G275" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:27.000Z</t>
+          <t>2026-07-10T05:28:16.000Z</t>
         </is>
       </c>
     </row>
@@ -8467,12 +8467,12 @@
         </is>
       </c>
       <c r="E276" t="n">
-        <v>716</v>
+        <v>244</v>
       </c>
       <c r="F276" t="inlineStr"/>
       <c r="G276" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:28.000Z</t>
+          <t>2026-07-10T05:28:17.000Z</t>
         </is>
       </c>
     </row>
@@ -8496,12 +8496,12 @@
         </is>
       </c>
       <c r="E277" t="n">
-        <v>1088</v>
+        <v>855</v>
       </c>
       <c r="F277" t="inlineStr"/>
       <c r="G277" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:29.000Z</t>
+          <t>2026-07-10T05:28:18.000Z</t>
         </is>
       </c>
     </row>
@@ -8525,12 +8525,12 @@
         </is>
       </c>
       <c r="E278" t="n">
-        <v>366</v>
+        <v>424</v>
       </c>
       <c r="F278" t="inlineStr"/>
       <c r="G278" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:30.000Z</t>
+          <t>2026-07-10T05:28:18.000Z</t>
         </is>
       </c>
     </row>
@@ -8554,12 +8554,12 @@
         </is>
       </c>
       <c r="E279" t="n">
-        <v>357</v>
+        <v>351</v>
       </c>
       <c r="F279" t="inlineStr"/>
       <c r="G279" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:30.000Z</t>
+          <t>2026-07-10T05:28:19.000Z</t>
         </is>
       </c>
     </row>
@@ -8583,12 +8583,12 @@
         </is>
       </c>
       <c r="E280" t="n">
-        <v>401</v>
+        <v>311</v>
       </c>
       <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:31.000Z</t>
+          <t>2026-07-10T05:28:20.000Z</t>
         </is>
       </c>
     </row>
@@ -8612,12 +8612,12 @@
         </is>
       </c>
       <c r="E281" t="n">
-        <v>312</v>
+        <v>987</v>
       </c>
       <c r="F281" t="inlineStr"/>
       <c r="G281" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:32.000Z</t>
+          <t>2026-07-10T05:28:21.000Z</t>
         </is>
       </c>
     </row>
@@ -8641,12 +8641,12 @@
         </is>
       </c>
       <c r="E282" t="n">
-        <v>269</v>
+        <v>744</v>
       </c>
       <c r="F282" t="inlineStr"/>
       <c r="G282" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:33.000Z</t>
+          <t>2026-07-10T05:28:22.000Z</t>
         </is>
       </c>
     </row>
@@ -8670,12 +8670,12 @@
         </is>
       </c>
       <c r="E283" t="n">
-        <v>502</v>
+        <v>1011</v>
       </c>
       <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:34.000Z</t>
+          <t>2026-07-10T05:28:22.000Z</t>
         </is>
       </c>
     </row>
@@ -8699,12 +8699,12 @@
         </is>
       </c>
       <c r="E284" t="n">
-        <v>522</v>
+        <v>662</v>
       </c>
       <c r="F284" t="inlineStr"/>
       <c r="G284" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:34.000Z</t>
+          <t>2026-07-10T05:28:23.000Z</t>
         </is>
       </c>
     </row>
@@ -8728,12 +8728,12 @@
         </is>
       </c>
       <c r="E285" t="n">
-        <v>1117</v>
+        <v>658</v>
       </c>
       <c r="F285" t="inlineStr"/>
       <c r="G285" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:35.000Z</t>
+          <t>2026-07-10T05:28:24.000Z</t>
         </is>
       </c>
     </row>
@@ -8757,12 +8757,12 @@
         </is>
       </c>
       <c r="E286" t="n">
-        <v>229</v>
+        <v>782</v>
       </c>
       <c r="F286" t="inlineStr"/>
       <c r="G286" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:36.000Z</t>
+          <t>2026-07-10T05:28:25.000Z</t>
         </is>
       </c>
     </row>
@@ -8786,12 +8786,12 @@
         </is>
       </c>
       <c r="E287" t="n">
-        <v>836</v>
+        <v>904</v>
       </c>
       <c r="F287" t="inlineStr"/>
       <c r="G287" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:37.000Z</t>
+          <t>2026-07-10T05:28:26.000Z</t>
         </is>
       </c>
     </row>
@@ -8815,12 +8815,12 @@
         </is>
       </c>
       <c r="E288" t="n">
-        <v>963</v>
+        <v>331</v>
       </c>
       <c r="F288" t="inlineStr"/>
       <c r="G288" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:38.000Z</t>
+          <t>2026-07-10T05:28:26.000Z</t>
         </is>
       </c>
     </row>
@@ -8844,12 +8844,12 @@
         </is>
       </c>
       <c r="E289" t="n">
-        <v>1014</v>
+        <v>696</v>
       </c>
       <c r="F289" t="inlineStr"/>
       <c r="G289" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:38.000Z</t>
+          <t>2026-07-10T05:28:27.000Z</t>
         </is>
       </c>
     </row>
@@ -8873,12 +8873,12 @@
         </is>
       </c>
       <c r="E290" t="n">
-        <v>941</v>
+        <v>1058</v>
       </c>
       <c r="F290" t="inlineStr"/>
       <c r="G290" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:39.000Z</t>
+          <t>2026-07-10T05:28:28.000Z</t>
         </is>
       </c>
     </row>
@@ -8902,12 +8902,12 @@
         </is>
       </c>
       <c r="E291" t="n">
-        <v>1098</v>
+        <v>974</v>
       </c>
       <c r="F291" t="inlineStr"/>
       <c r="G291" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:40.000Z</t>
+          <t>2026-07-10T05:28:29.000Z</t>
         </is>
       </c>
     </row>
@@ -8931,12 +8931,12 @@
         </is>
       </c>
       <c r="E292" t="n">
-        <v>1128</v>
+        <v>1197</v>
       </c>
       <c r="F292" t="inlineStr"/>
       <c r="G292" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:41.000Z</t>
+          <t>2026-07-10T05:28:30.000Z</t>
         </is>
       </c>
     </row>
@@ -8960,12 +8960,12 @@
         </is>
       </c>
       <c r="E293" t="n">
-        <v>1141</v>
+        <v>1116</v>
       </c>
       <c r="F293" t="inlineStr"/>
       <c r="G293" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:42.000Z</t>
+          <t>2026-07-10T05:28:30.000Z</t>
         </is>
       </c>
     </row>
@@ -8989,12 +8989,12 @@
         </is>
       </c>
       <c r="E294" t="n">
-        <v>204</v>
+        <v>1109</v>
       </c>
       <c r="F294" t="inlineStr"/>
       <c r="G294" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:42.000Z</t>
+          <t>2026-07-10T05:28:31.000Z</t>
         </is>
       </c>
     </row>
@@ -9018,12 +9018,12 @@
         </is>
       </c>
       <c r="E295" t="n">
-        <v>536</v>
+        <v>734</v>
       </c>
       <c r="F295" t="inlineStr"/>
       <c r="G295" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:43.000Z</t>
+          <t>2026-07-10T05:28:32.000Z</t>
         </is>
       </c>
     </row>
@@ -9047,12 +9047,12 @@
         </is>
       </c>
       <c r="E296" t="n">
-        <v>1000</v>
+        <v>585</v>
       </c>
       <c r="F296" t="inlineStr"/>
       <c r="G296" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:44.000Z</t>
+          <t>2026-07-10T05:28:33.000Z</t>
         </is>
       </c>
     </row>
@@ -9076,12 +9076,12 @@
         </is>
       </c>
       <c r="E297" t="n">
-        <v>573</v>
+        <v>120</v>
       </c>
       <c r="F297" t="inlineStr"/>
       <c r="G297" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:45.000Z</t>
+          <t>2026-07-10T05:28:34.000Z</t>
         </is>
       </c>
     </row>
@@ -9105,12 +9105,12 @@
         </is>
       </c>
       <c r="E298" t="n">
-        <v>1100</v>
+        <v>1104</v>
       </c>
       <c r="F298" t="inlineStr"/>
       <c r="G298" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:46.000Z</t>
+          <t>2026-07-10T05:28:34.000Z</t>
         </is>
       </c>
     </row>
@@ -9134,12 +9134,12 @@
         </is>
       </c>
       <c r="E299" t="n">
-        <v>851</v>
+        <v>551</v>
       </c>
       <c r="F299" t="inlineStr"/>
       <c r="G299" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:46.000Z</t>
+          <t>2026-07-10T05:28:35.000Z</t>
         </is>
       </c>
     </row>
@@ -9163,12 +9163,12 @@
         </is>
       </c>
       <c r="E300" t="n">
-        <v>564</v>
+        <v>135</v>
       </c>
       <c r="F300" t="inlineStr"/>
       <c r="G300" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:47.000Z</t>
+          <t>2026-07-10T05:28:36.000Z</t>
         </is>
       </c>
     </row>
@@ -9192,12 +9192,12 @@
         </is>
       </c>
       <c r="E301" t="n">
-        <v>253</v>
+        <v>725</v>
       </c>
       <c r="F301" t="inlineStr"/>
       <c r="G301" t="inlineStr">
         <is>
-          <t>2026-07-10T04:57:48.000Z</t>
+          <t>2026-07-10T05:28:37.000Z</t>
         </is>
       </c>
     </row>
@@ -9325,7 +9325,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-10T04:53:48.000Z</t>
+          <t>2026-07-10T05:24:37.000Z</t>
         </is>
       </c>
     </row>

</xml_diff>